<commit_message>
fixed unit conversion and updated unit mapping
</commit_message>
<xml_diff>
--- a/config_data/mapping_v4.xlsx
+++ b/config_data/mapping_v4.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28516"/>
-  <workbookPr defaultThemeVersion="166925"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aspat\Documents\GitHub\HiWi Project\data_adapter_times\config_data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Xchange\Studis\Apath\HiWi Project\config_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B66368B-05D7-4F10-A596-49E781B4A928}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720"/>
   </bookViews>
   <sheets>
     <sheet name="SEDOS_parameters" sheetId="5" r:id="rId1"/>
@@ -30,12 +29,12 @@
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Islam, Md Anik</author>
   </authors>
   <commentList>
-    <comment ref="B44" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
+    <comment ref="B45" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -65,12 +64,12 @@
 </file>
 
 <file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Gary Goldstein</author>
   </authors>
   <commentList>
-    <comment ref="D1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000001000000}">
+    <comment ref="D1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -92,7 +91,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="416" uniqueCount="309">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="419" uniqueCount="310">
   <si>
     <t>TIMES</t>
   </si>
@@ -1019,12 +1018,15 @@
   </si>
   <si>
     <t>capacity_tra_max</t>
+  </si>
+  <si>
+    <t>capacity_tra_min</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1189,8 +1191,8 @@
     </xf>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 10" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
+    <cellStyle name="Normal 10" xfId="1"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="1">
     <dxf>
@@ -1512,22 +1514,22 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O121"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:O122"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="37.77734375" customWidth="1"/>
-    <col min="2" max="2" width="25.77734375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="31.77734375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="37.7109375" customWidth="1"/>
+    <col min="2" max="2" width="25.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="31.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.28515625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="18" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.77734375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.77734375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="22.21875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.77734375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -1559,7 +1561,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>100</v>
       </c>
@@ -1570,7 +1572,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>5</v>
       </c>
@@ -1581,7 +1583,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>81</v>
       </c>
@@ -1595,7 +1597,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>101</v>
       </c>
@@ -1616,7 +1618,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
         <v>46</v>
       </c>
@@ -1629,7 +1631,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>6</v>
       </c>
@@ -1640,7 +1642,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
         <v>102</v>
       </c>
@@ -1649,7 +1651,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>74</v>
       </c>
@@ -1660,7 +1662,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>103</v>
       </c>
@@ -1674,7 +1676,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>104</v>
       </c>
@@ -1688,7 +1690,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>64</v>
       </c>
@@ -1699,7 +1701,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>105</v>
       </c>
@@ -1713,7 +1715,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>106</v>
       </c>
@@ -1727,7 +1729,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>56</v>
       </c>
@@ -1738,7 +1740,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>107</v>
       </c>
@@ -1752,7 +1754,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>108</v>
       </c>
@@ -1766,709 +1768,720 @@
         <v>19</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>9</v>
       </c>
       <c r="I18" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
+        <v>308</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="I19" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A19" s="2" t="s">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="B20" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C19" t="s">
+      <c r="C20" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A20" s="2" t="s">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A21" s="2" t="s">
         <v>75</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C20" t="s">
-        <v>170</v>
-      </c>
-      <c r="I20" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A21" s="2" t="s">
-        <v>72</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>9</v>
       </c>
       <c r="C21" t="s">
-        <v>73</v>
+        <v>170</v>
       </c>
       <c r="I21" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>63</v>
+        <v>72</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>9</v>
       </c>
       <c r="C22" t="s">
-        <v>13</v>
+        <v>73</v>
       </c>
       <c r="I22" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C23" t="s">
+        <v>13</v>
+      </c>
+      <c r="I23" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A24" s="2" t="s">
         <v>4</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="C23" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A24" s="2" t="s">
-        <v>110</v>
       </c>
       <c r="B24" s="2" t="s">
         <v>49</v>
       </c>
       <c r="C24" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A25" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C25" t="s">
         <v>171</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A25" s="9" t="s">
-        <v>111</v>
-      </c>
-      <c r="B25" s="9" t="s">
-        <v>150</v>
-      </c>
-      <c r="C25" t="s">
-        <v>172</v>
       </c>
       <c r="J25" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A26" s="2" t="s">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A26" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="B26" s="9" t="s">
+        <v>150</v>
+      </c>
+      <c r="C26" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A27" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="B26" s="2"/>
-      <c r="C26" t="s">
+      <c r="B27" s="2"/>
+      <c r="C27" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A27" s="2" t="s">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A28" s="2" t="s">
         <v>76</v>
-      </c>
-      <c r="B27" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="C27" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A28" s="2" t="s">
-        <v>66</v>
       </c>
       <c r="B28" s="2" t="s">
         <v>58</v>
       </c>
       <c r="C28" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>58</v>
       </c>
       <c r="C29" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>113</v>
+        <v>59</v>
       </c>
       <c r="B30" s="2" t="s">
         <v>58</v>
       </c>
       <c r="C30" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A31" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C31" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A31" s="2" t="s">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A32" s="2" t="s">
         <v>78</v>
-      </c>
-      <c r="B31" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C31" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A32" s="2" t="s">
-        <v>68</v>
       </c>
       <c r="B32" s="2" t="s">
         <v>11</v>
       </c>
       <c r="C32" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="B33" s="2" t="s">
         <v>11</v>
       </c>
       <c r="C33" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.3">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>114</v>
+        <v>60</v>
       </c>
       <c r="B34" s="2" t="s">
         <v>11</v>
       </c>
       <c r="C34" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A35" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C35" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A35" s="2" t="s">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A36" s="2" t="s">
         <v>70</v>
-      </c>
-      <c r="B35" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C35" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A36" s="2" t="s">
-        <v>115</v>
       </c>
       <c r="B36" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C36" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>61</v>
+        <v>115</v>
       </c>
       <c r="B37" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C37" t="s">
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A38" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C38" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A38" s="2" t="s">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A39" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="B38" s="2" t="s">
+      <c r="B39" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="C38" t="s">
+      <c r="C39" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A39" s="2" t="s">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A40" s="2" t="s">
         <v>117</v>
-      </c>
-      <c r="B39" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="C39" t="s">
-        <v>53</v>
-      </c>
-      <c r="I39" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A40" s="2" t="s">
-        <v>118</v>
       </c>
       <c r="B40" s="2" t="s">
         <v>25</v>
       </c>
       <c r="C40" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="I40" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.3">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B41" s="2" t="s">
         <v>25</v>
       </c>
       <c r="C41" t="s">
+        <v>54</v>
+      </c>
+      <c r="I41" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A42" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C42" t="s">
         <v>55</v>
       </c>
-      <c r="I41" t="s">
+      <c r="I42" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A42" s="2" t="s">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A43" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="B42" s="2" t="s">
+      <c r="B43" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="C42" t="s">
+      <c r="C43" t="s">
         <v>176</v>
-      </c>
-    </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A43" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="B43" s="2"/>
-      <c r="C43" t="s">
-        <v>177</v>
       </c>
       <c r="J43" s="2" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="B44" s="2"/>
+      <c r="C44" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A45" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="B44" s="2" t="s">
+      <c r="B45" s="2" t="s">
         <v>200</v>
       </c>
-      <c r="C44" t="s">
+      <c r="C45" t="s">
         <v>178</v>
       </c>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A45" s="2" t="s">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A46" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="B45" s="2" t="s">
+      <c r="B46" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="C45" t="s">
+      <c r="C46" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A46" s="2" t="s">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A47" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="B46" s="2" t="s">
+      <c r="B47" s="2" t="s">
         <v>153</v>
       </c>
-      <c r="C46" t="s">
+      <c r="C47" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A47" s="9" t="s">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A48" s="9" t="s">
         <v>125</v>
-      </c>
-      <c r="B47" s="9"/>
-      <c r="C47" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A48" s="9" t="s">
-        <v>126</v>
       </c>
       <c r="B48" s="9"/>
       <c r="C48" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" s="9" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B49" s="9"/>
       <c r="C49" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" s="9" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B50" s="9"/>
       <c r="C50" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" s="9" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B51" s="9"/>
       <c r="C51" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" s="9" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B52" s="9"/>
       <c r="C52" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" s="9" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B53" s="9"/>
       <c r="C53" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" s="9" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B54" s="9"/>
       <c r="C54" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A55" s="9" t="s">
+        <v>132</v>
+      </c>
+      <c r="B55" s="9"/>
+      <c r="C55" t="s">
         <v>188</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A55" s="2" t="s">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A56" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="B55" s="2" t="s">
+      <c r="B56" s="2" t="s">
         <v>306</v>
       </c>
-      <c r="C55" t="s">
+      <c r="C56" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A56" s="9" t="s">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A57" s="9" t="s">
         <v>134</v>
       </c>
-      <c r="B56" s="9"/>
-      <c r="C56" t="s">
+      <c r="B57" s="9"/>
+      <c r="C57" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A57" s="2" t="s">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A58" s="2" t="s">
         <v>135</v>
-      </c>
-      <c r="B57" s="2" t="s">
-        <v>307</v>
-      </c>
-      <c r="C57" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A58" s="10" t="s">
-        <v>136</v>
       </c>
       <c r="B58" s="2" t="s">
         <v>307</v>
       </c>
       <c r="C58" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A59" s="10" t="s">
+        <v>136</v>
+      </c>
+      <c r="B59" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="C59" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A59" s="10" t="s">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A60" s="10" t="s">
         <v>137</v>
-      </c>
-      <c r="B59" s="11"/>
-      <c r="C59" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A60" s="9" t="s">
-        <v>138</v>
       </c>
       <c r="B60" s="11"/>
       <c r="C60" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.3">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" s="9" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B61" s="11"/>
       <c r="C61" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A62" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="B62" s="11"/>
+      <c r="C62" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A62" s="10" t="s">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A63" s="10" t="s">
         <v>140</v>
       </c>
-      <c r="B62" s="10" t="s">
+      <c r="B63" s="10" t="s">
         <v>154</v>
       </c>
-      <c r="C62" t="s">
+      <c r="C63" t="s">
         <v>196</v>
       </c>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A63" s="7" t="s">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A64" s="7" t="s">
         <v>141</v>
       </c>
-      <c r="B63" s="6"/>
-    </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A64" s="7" t="s">
+      <c r="B64" s="6"/>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A65" s="7" t="s">
         <v>142</v>
       </c>
-      <c r="B64" s="6"/>
-    </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A65" s="7" t="s">
+      <c r="B65" s="6"/>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A66" s="7" t="s">
         <v>143</v>
       </c>
-      <c r="B65" s="8"/>
-      <c r="C65" t="s">
+      <c r="B66" s="8"/>
+      <c r="C66" t="s">
         <v>197</v>
       </c>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A66" s="7" t="s">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A67" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="B66" s="6"/>
-    </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A67" s="7" t="s">
+      <c r="B67" s="6"/>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A68" s="7" t="s">
         <v>144</v>
       </c>
-      <c r="B67" s="6"/>
-    </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A68" s="7" t="s">
+      <c r="B68" s="6"/>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A69" s="7" t="s">
         <v>145</v>
       </c>
-      <c r="B68" s="6"/>
-    </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A69" s="7" t="s">
+      <c r="B69" s="6"/>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A70" s="7" t="s">
         <v>146</v>
       </c>
-      <c r="B69" s="6"/>
-    </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A70" s="7" t="s">
+      <c r="B70" s="6"/>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A71" s="7" t="s">
         <v>147</v>
       </c>
-      <c r="B70" s="6"/>
-    </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A71" s="7" t="s">
+      <c r="B71" s="6"/>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A72" s="7" t="s">
         <v>148</v>
       </c>
-      <c r="B71" s="6"/>
-    </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A72" s="7" t="s">
+      <c r="B72" s="6"/>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A73" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="B72" s="6"/>
-    </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A73" s="7" t="s">
+      <c r="B73" s="6"/>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A74" s="7" t="s">
         <v>149</v>
       </c>
-      <c r="B73" s="6"/>
-    </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A74" s="7" t="s">
+      <c r="B74" s="6"/>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A75" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="B74" s="6"/>
-    </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B75" s="6"/>
     </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B76" s="6"/>
     </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B77" s="6"/>
     </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B78" s="6"/>
     </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B79" s="6"/>
     </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B80" s="6"/>
     </row>
-    <row r="81" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="81" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B81" s="6"/>
     </row>
-    <row r="82" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="82" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B82" s="6"/>
     </row>
-    <row r="83" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="83" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B83" s="6"/>
     </row>
-    <row r="84" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="84" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B84" s="6"/>
     </row>
-    <row r="85" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="85" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B85" s="6"/>
     </row>
-    <row r="86" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="86" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B86" s="6"/>
     </row>
-    <row r="87" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="87" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B87" s="6"/>
     </row>
-    <row r="88" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="88" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B88" s="6"/>
     </row>
-    <row r="89" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="89" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B89" s="6"/>
     </row>
-    <row r="90" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="90" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B90" s="6"/>
     </row>
-    <row r="91" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="91" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B91" s="6"/>
     </row>
-    <row r="92" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="92" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B92" s="6"/>
     </row>
-    <row r="93" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="93" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B93" s="6"/>
     </row>
-    <row r="94" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="94" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B94" s="6"/>
     </row>
-    <row r="95" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="95" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B95" s="6"/>
     </row>
-    <row r="96" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="96" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B96" s="6"/>
     </row>
-    <row r="97" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="97" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B97" s="6"/>
     </row>
-    <row r="98" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="98" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B98" s="6"/>
     </row>
-    <row r="99" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="99" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B99" s="6"/>
     </row>
-    <row r="100" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="100" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B100" s="6"/>
     </row>
-    <row r="101" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="101" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B101" s="6"/>
     </row>
-    <row r="102" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="102" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B102" s="6"/>
     </row>
-    <row r="103" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="103" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B103" s="6"/>
     </row>
-    <row r="104" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="104" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B104" s="6"/>
     </row>
-    <row r="105" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="105" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B105" s="6"/>
     </row>
-    <row r="106" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="106" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B106" s="6"/>
     </row>
-    <row r="107" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="107" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B107" s="6"/>
     </row>
-    <row r="108" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="108" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B108" s="6"/>
     </row>
-    <row r="109" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="109" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B109" s="6"/>
     </row>
-    <row r="110" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="110" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B110" s="6"/>
     </row>
-    <row r="111" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="111" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B111" s="6"/>
     </row>
-    <row r="112" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="112" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B112" s="6"/>
     </row>
-    <row r="113" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="113" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B113" s="6"/>
     </row>
-    <row r="114" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="114" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B114" s="6"/>
     </row>
-    <row r="115" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="115" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B115" s="6"/>
     </row>
-    <row r="116" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="116" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B116" s="6"/>
     </row>
-    <row r="117" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="117" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B117" s="6"/>
     </row>
-    <row r="118" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="118" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B118" s="6"/>
     </row>
-    <row r="119" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="119" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B119" s="6"/>
     </row>
-    <row r="120" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="120" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B120" s="6"/>
     </row>
-    <row r="121" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="121" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B121" s="6"/>
+    </row>
+    <row r="122" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B122" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2478,17 +2491,17 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D130"/>
-  <sheetFormatPr defaultColWidth="9.21875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="32.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.5546875" customWidth="1"/>
-    <col min="3" max="3" width="15.44140625" customWidth="1"/>
-    <col min="4" max="4" width="23.77734375" customWidth="1"/>
+    <col min="1" max="1" width="32.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.5703125" customWidth="1"/>
+    <col min="3" max="3" width="15.42578125" customWidth="1"/>
+    <col min="4" max="4" width="23.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>27</v>
       </c>
@@ -2502,7 +2515,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="31.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
         <v>31</v>
       </c>
@@ -2516,117 +2529,117 @@
         <v>33</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>250</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>251</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>252</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>253</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>254</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>256</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>257</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>258</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="13" t="s">
         <v>259</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="13" t="s">
         <v>260</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="14" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>261</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="13" t="s">
         <v>262</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="13" t="s">
         <v>228</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="13" t="s">
         <v>263</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>264</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="14" t="s">
         <v>265</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="14" t="s">
         <v>266</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="14" t="s">
         <v>267</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="14" t="s">
         <v>268</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="14" t="s">
         <v>269</v>
       </c>
@@ -2634,7 +2647,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="14" t="s">
         <v>270</v>
       </c>
@@ -2642,97 +2655,97 @@
         <v>35</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="13" t="s">
         <v>271</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="13" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="13" t="s">
         <v>272</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="13" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="13" t="s">
         <v>273</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="13" t="s">
         <v>274</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="13" t="s">
         <v>275</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" s="13" t="s">
         <v>276</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" s="13" t="s">
         <v>277</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" s="13" t="s">
         <v>278</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" s="13" t="s">
         <v>279</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" s="13" t="s">
         <v>280</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" s="13" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" s="13" t="s">
         <v>281</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" s="13" t="s">
         <v>282</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" s="13" t="s">
         <v>283</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" s="13" t="s">
         <v>284</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" s="13" t="s">
         <v>84</v>
       </c>
@@ -2740,7 +2753,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" s="13" t="s">
         <v>85</v>
       </c>
@@ -2748,7 +2761,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" s="13" t="s">
         <v>86</v>
       </c>
@@ -2756,7 +2769,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" s="13" t="s">
         <v>88</v>
       </c>
@@ -2764,7 +2777,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" s="13" t="s">
         <v>89</v>
       </c>
@@ -2772,7 +2785,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" s="13" t="s">
         <v>91</v>
       </c>
@@ -2780,7 +2793,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" s="13" t="s">
         <v>94</v>
       </c>
@@ -2788,7 +2801,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" s="13" t="s">
         <v>96</v>
       </c>
@@ -2796,7 +2809,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" s="13" t="s">
         <v>95</v>
       </c>
@@ -2804,7 +2817,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>92</v>
       </c>
@@ -2812,7 +2825,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>93</v>
       </c>
@@ -2820,7 +2833,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>36</v>
       </c>
@@ -2828,7 +2841,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>40</v>
       </c>
@@ -2836,7 +2849,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>39</v>
       </c>
@@ -2844,7 +2857,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>38</v>
       </c>
@@ -2852,7 +2865,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>34</v>
       </c>
@@ -2860,7 +2873,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>37</v>
       </c>
@@ -2868,7 +2881,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>98</v>
       </c>
@@ -2876,7 +2889,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>99</v>
       </c>
@@ -2884,107 +2897,107 @@
         <v>35</v>
       </c>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" s="14" t="s">
         <v>285</v>
       </c>
     </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>286</v>
       </c>
     </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>287</v>
       </c>
     </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>288</v>
       </c>
     </row>
-    <row r="69" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>289</v>
       </c>
     </row>
-    <row r="70" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>221</v>
       </c>
     </row>
-    <row r="71" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>290</v>
       </c>
     </row>
-    <row r="72" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>291</v>
       </c>
     </row>
-    <row r="73" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="74" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>214</v>
       </c>
     </row>
-    <row r="75" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>292</v>
       </c>
     </row>
-    <row r="76" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>293</v>
       </c>
     </row>
-    <row r="77" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="78" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>294</v>
       </c>
     </row>
-    <row r="79" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>295</v>
       </c>
     </row>
-    <row r="80" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>296</v>
       </c>
     </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>297</v>
       </c>
     </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>298</v>
       </c>
     </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>299</v>
       </c>
     </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>230</v>
       </c>
@@ -2992,7 +3005,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>246</v>
       </c>
@@ -3000,7 +3013,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>248</v>
       </c>
@@ -3008,7 +3021,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>217</v>
       </c>
@@ -3016,7 +3029,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>300</v>
       </c>
@@ -3024,7 +3037,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>208</v>
       </c>
@@ -3032,7 +3045,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>229</v>
       </c>
@@ -3040,7 +3053,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>211</v>
       </c>
@@ -3048,7 +3061,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>241</v>
       </c>
@@ -3056,7 +3069,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>226</v>
       </c>
@@ -3064,7 +3077,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>242</v>
       </c>
@@ -3072,7 +3085,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>243</v>
       </c>
@@ -3080,32 +3093,32 @@
         <v>35</v>
       </c>
     </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>301</v>
       </c>
     </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>302</v>
       </c>
     </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>303</v>
       </c>
     </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>304</v>
       </c>
     </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>305</v>
       </c>
     </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" s="15" t="s">
         <v>247</v>
       </c>
@@ -3113,7 +3126,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A102" s="15" t="s">
         <v>235</v>
       </c>
@@ -3121,7 +3134,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A103" s="15" t="s">
         <v>220</v>
       </c>
@@ -3129,7 +3142,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A104" s="15" t="s">
         <v>233</v>
       </c>
@@ -3137,7 +3150,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A105" s="15" t="s">
         <v>213</v>
       </c>
@@ -3145,7 +3158,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="106" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A106" s="15" t="s">
         <v>205</v>
       </c>
@@ -3153,7 +3166,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A107" s="15" t="s">
         <v>224</v>
       </c>
@@ -3161,7 +3174,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A108" s="15" t="s">
         <v>239</v>
       </c>
@@ -3169,7 +3182,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A109" s="15" t="s">
         <v>216</v>
       </c>
@@ -3177,7 +3190,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A110" s="15" t="s">
         <v>201</v>
       </c>
@@ -3185,7 +3198,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A111" s="15" t="s">
         <v>238</v>
       </c>
@@ -3193,7 +3206,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="112" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A112" s="15" t="s">
         <v>231</v>
       </c>
@@ -3201,7 +3214,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="113" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A113" s="15" t="s">
         <v>209</v>
       </c>
@@ -3209,7 +3222,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="114" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A114" s="15" t="s">
         <v>215</v>
       </c>
@@ -3217,7 +3230,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="115" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A115" s="15" t="s">
         <v>232</v>
       </c>
@@ -3225,7 +3238,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="116" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A116" s="15" t="s">
         <v>244</v>
       </c>
@@ -3233,7 +3246,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="117" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A117" s="15" t="s">
         <v>223</v>
       </c>
@@ -3241,7 +3254,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="118" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A118" s="15" t="s">
         <v>218</v>
       </c>
@@ -3249,7 +3262,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="119" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A119" s="15" t="s">
         <v>236</v>
       </c>
@@ -3257,7 +3270,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="120" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A120" s="15" t="s">
         <v>225</v>
       </c>
@@ -3265,7 +3278,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="121" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A121" s="15" t="s">
         <v>234</v>
       </c>
@@ -3273,7 +3286,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="122" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A122" s="15" t="s">
         <v>222</v>
       </c>
@@ -3281,7 +3294,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="123" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A123" s="15" t="s">
         <v>219</v>
       </c>
@@ -3289,7 +3302,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="124" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A124" s="15" t="s">
         <v>240</v>
       </c>
@@ -3297,7 +3310,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="125" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A125" s="15" t="s">
         <v>210</v>
       </c>
@@ -3305,7 +3318,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="126" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A126" s="15" t="s">
         <v>207</v>
       </c>
@@ -3313,7 +3326,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="127" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A127" s="15" t="s">
         <v>227</v>
       </c>
@@ -3321,7 +3334,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="128" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A128" s="15" t="s">
         <v>203</v>
       </c>
@@ -3329,7 +3342,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="129" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A129" s="15" t="s">
         <v>206</v>
       </c>
@@ -3337,7 +3350,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="130" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A130" s="15" t="s">
         <v>245</v>
       </c>
@@ -3346,7 +3359,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:A130" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
+  <autoFilter ref="A1:A130"/>
   <conditionalFormatting sqref="A3:A130">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
@@ -3356,11 +3369,11 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="9.21875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3371,7 +3384,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>19</v>
       </c>
@@ -3379,7 +3392,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>21</v>
       </c>
@@ -3387,7 +3400,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>23</v>
       </c>

</xml_diff>

<commit_message>
refactor emission factor processing for ind agri and enhance  flo share data mapping logic
</commit_message>
<xml_diff>
--- a/config_data/mapping_v4.xlsx
+++ b/config_data/mapping_v4.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20395"/>
-  <workbookPr defaultThemeVersion="166925"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Xchange\Studis\Apath\materials_DAdapter\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Xchange\Studis\Apath\HiWi Project\config_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF0B9B68-99F5-441C-B2EB-6655F9C29328}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="8150" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="8145" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="SEDOS_parameters" sheetId="5" r:id="rId1"/>
@@ -30,12 +29,12 @@
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Islam, Md Anik</author>
   </authors>
   <commentList>
-    <comment ref="B43" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
+    <comment ref="B43" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -65,12 +64,12 @@
 </file>
 
 <file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Gary Goldstein</author>
   </authors>
   <commentList>
-    <comment ref="D1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000001000000}">
+    <comment ref="D1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -92,7 +91,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="413" uniqueCount="308">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="419" uniqueCount="309">
   <si>
     <t>TIMES</t>
   </si>
@@ -1016,12 +1015,15 @@
   </si>
   <si>
     <t>ACTFLO~DEMO</t>
+  </si>
+  <si>
+    <t>emi_co2_neg_air_dacc</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1192,8 +1194,8 @@
     </xf>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 10" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
+    <cellStyle name="Normal 10" xfId="1"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="1">
     <dxf>
@@ -1515,22 +1517,22 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:O120"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="37.7265625" customWidth="1"/>
-    <col min="2" max="2" width="25.7265625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="31.81640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.26953125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="37.7109375" customWidth="1"/>
+    <col min="2" max="2" width="25.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="31.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.28515625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="18" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.7265625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.7265625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="22.26953125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -1562,7 +1564,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>100</v>
       </c>
@@ -1573,7 +1575,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>5</v>
       </c>
@@ -1584,7 +1586,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>81</v>
       </c>
@@ -1598,7 +1600,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>101</v>
       </c>
@@ -1619,7 +1621,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
         <v>46</v>
       </c>
@@ -1632,7 +1634,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>6</v>
       </c>
@@ -1643,7 +1645,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
         <v>102</v>
       </c>
@@ -1652,7 +1654,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>74</v>
       </c>
@@ -1663,7 +1665,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>103</v>
       </c>
@@ -1677,7 +1679,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>104</v>
       </c>
@@ -1691,7 +1693,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>64</v>
       </c>
@@ -1702,7 +1704,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>105</v>
       </c>
@@ -1716,7 +1718,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>106</v>
       </c>
@@ -1730,7 +1732,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>56</v>
       </c>
@@ -1741,7 +1743,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>107</v>
       </c>
@@ -1755,7 +1757,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>108</v>
       </c>
@@ -1769,7 +1771,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>109</v>
       </c>
@@ -1780,7 +1782,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>75</v>
       </c>
@@ -1794,7 +1796,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>72</v>
       </c>
@@ -1808,7 +1810,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>63</v>
       </c>
@@ -1822,7 +1824,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>4</v>
       </c>
@@ -1833,7 +1835,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>110</v>
       </c>
@@ -1844,7 +1846,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" s="9" t="s">
         <v>111</v>
       </c>
@@ -1855,7 +1857,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>112</v>
       </c>
@@ -1867,7 +1869,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>76</v>
       </c>
@@ -1878,7 +1880,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>66</v>
       </c>
@@ -1889,7 +1891,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>59</v>
       </c>
@@ -1900,7 +1902,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>113</v>
       </c>
@@ -1911,7 +1913,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>78</v>
       </c>
@@ -1922,7 +1924,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>68</v>
       </c>
@@ -1933,7 +1935,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>60</v>
       </c>
@@ -1944,7 +1946,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>114</v>
       </c>
@@ -1955,7 +1957,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>70</v>
       </c>
@@ -1966,7 +1968,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>115</v>
       </c>
@@ -1974,7 +1976,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>61</v>
       </c>
@@ -1985,7 +1987,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>116</v>
       </c>
@@ -1996,7 +1998,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>117</v>
       </c>
@@ -2010,7 +2012,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>118</v>
       </c>
@@ -2024,7 +2026,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
         <v>119</v>
       </c>
@@ -2038,7 +2040,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>120</v>
       </c>
@@ -2049,7 +2051,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
         <v>121</v>
       </c>
@@ -2058,7 +2060,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
         <v>122</v>
       </c>
@@ -2072,7 +2074,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
         <v>123</v>
       </c>
@@ -2083,7 +2085,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
         <v>124</v>
       </c>
@@ -2094,7 +2096,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" s="9" t="s">
         <v>125</v>
       </c>
@@ -2103,7 +2105,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" s="9" t="s">
         <v>126</v>
       </c>
@@ -2112,7 +2114,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" s="9" t="s">
         <v>127</v>
       </c>
@@ -2121,7 +2123,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" s="9" t="s">
         <v>128</v>
       </c>
@@ -2130,7 +2132,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" s="9" t="s">
         <v>129</v>
       </c>
@@ -2139,7 +2141,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" s="9" t="s">
         <v>130</v>
       </c>
@@ -2148,7 +2150,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" s="9" t="s">
         <v>131</v>
       </c>
@@ -2157,7 +2159,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" s="9" t="s">
         <v>132</v>
       </c>
@@ -2166,7 +2168,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
         <v>133</v>
       </c>
@@ -2177,7 +2179,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" s="9" t="s">
         <v>134</v>
       </c>
@@ -2186,7 +2188,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
         <v>135</v>
       </c>
@@ -2197,7 +2199,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57" s="10" t="s">
         <v>136</v>
       </c>
@@ -2208,7 +2210,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" s="10" t="s">
         <v>137</v>
       </c>
@@ -2217,7 +2219,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" s="9" t="s">
         <v>138</v>
       </c>
@@ -2226,7 +2228,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" s="9" t="s">
         <v>139</v>
       </c>
@@ -2235,7 +2237,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" s="10" t="s">
         <v>140</v>
       </c>
@@ -2246,19 +2248,19 @@
         <v>196</v>
       </c>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" s="7" t="s">
         <v>141</v>
       </c>
       <c r="B62" s="6"/>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" s="7" t="s">
         <v>142</v>
       </c>
       <c r="B63" s="6"/>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A64" s="7" t="s">
         <v>143</v>
       </c>
@@ -2267,199 +2269,199 @@
         <v>197</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65" s="7" t="s">
         <v>41</v>
       </c>
       <c r="B65" s="6"/>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A66" s="7" t="s">
         <v>144</v>
       </c>
       <c r="B66" s="6"/>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A67" s="7" t="s">
         <v>145</v>
       </c>
       <c r="B67" s="6"/>
     </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A68" s="7" t="s">
         <v>146</v>
       </c>
       <c r="B68" s="6"/>
     </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A69" s="7" t="s">
         <v>147</v>
       </c>
       <c r="B69" s="6"/>
     </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A70" s="7" t="s">
         <v>148</v>
       </c>
       <c r="B70" s="6"/>
     </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A71" s="7" t="s">
         <v>47</v>
       </c>
       <c r="B71" s="6"/>
     </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A72" s="7" t="s">
         <v>149</v>
       </c>
       <c r="B72" s="6"/>
     </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A73" s="7" t="s">
         <v>48</v>
       </c>
       <c r="B73" s="6"/>
     </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B74" s="6"/>
     </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B75" s="6"/>
     </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B76" s="6"/>
     </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B77" s="6"/>
     </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B78" s="6"/>
     </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B79" s="6"/>
     </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B80" s="6"/>
     </row>
-    <row r="81" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="81" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B81" s="6"/>
     </row>
-    <row r="82" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="82" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B82" s="6"/>
     </row>
-    <row r="83" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="83" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B83" s="6"/>
     </row>
-    <row r="84" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="84" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B84" s="6"/>
     </row>
-    <row r="85" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="85" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B85" s="6"/>
     </row>
-    <row r="86" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="86" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B86" s="6"/>
     </row>
-    <row r="87" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="87" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B87" s="6"/>
     </row>
-    <row r="88" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="88" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B88" s="6"/>
     </row>
-    <row r="89" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="89" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B89" s="6"/>
     </row>
-    <row r="90" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="90" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B90" s="6"/>
     </row>
-    <row r="91" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="91" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B91" s="6"/>
     </row>
-    <row r="92" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="92" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B92" s="6"/>
     </row>
-    <row r="93" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="93" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B93" s="6"/>
     </row>
-    <row r="94" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="94" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B94" s="6"/>
     </row>
-    <row r="95" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="95" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B95" s="6"/>
     </row>
-    <row r="96" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="96" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B96" s="6"/>
     </row>
-    <row r="97" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="97" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B97" s="6"/>
     </row>
-    <row r="98" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="98" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B98" s="6"/>
     </row>
-    <row r="99" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="99" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B99" s="6"/>
     </row>
-    <row r="100" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="100" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B100" s="6"/>
     </row>
-    <row r="101" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="101" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B101" s="6"/>
     </row>
-    <row r="102" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="102" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B102" s="6"/>
     </row>
-    <row r="103" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="103" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B103" s="6"/>
     </row>
-    <row r="104" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="104" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B104" s="6"/>
     </row>
-    <row r="105" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="105" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B105" s="6"/>
     </row>
-    <row r="106" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="106" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B106" s="6"/>
     </row>
-    <row r="107" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="107" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B107" s="6"/>
     </row>
-    <row r="108" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="108" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B108" s="6"/>
     </row>
-    <row r="109" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="109" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B109" s="6"/>
     </row>
-    <row r="110" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="110" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B110" s="6"/>
     </row>
-    <row r="111" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="111" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B111" s="6"/>
     </row>
-    <row r="112" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="112" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B112" s="6"/>
     </row>
-    <row r="113" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="113" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B113" s="6"/>
     </row>
-    <row r="114" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="114" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B114" s="6"/>
     </row>
-    <row r="115" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="115" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B115" s="6"/>
     </row>
-    <row r="116" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="116" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B116" s="6"/>
     </row>
-    <row r="117" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="117" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B117" s="6"/>
     </row>
-    <row r="118" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="118" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B118" s="6"/>
     </row>
-    <row r="119" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="119" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B119" s="6"/>
     </row>
-    <row r="120" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="120" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B120" s="6"/>
     </row>
   </sheetData>
@@ -2470,17 +2472,17 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:D130"/>
-  <sheetFormatPr defaultColWidth="9.26953125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D133"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="32.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.54296875" customWidth="1"/>
-    <col min="3" max="3" width="15.453125" customWidth="1"/>
-    <col min="4" max="4" width="23.7265625" customWidth="1"/>
+    <col min="1" max="1" width="32.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.5703125" customWidth="1"/>
+    <col min="3" max="3" width="15.42578125" customWidth="1"/>
+    <col min="4" max="4" width="23.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>27</v>
       </c>
@@ -2494,7 +2496,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:4" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
         <v>31</v>
       </c>
@@ -2508,134 +2510,134 @@
         <v>33</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
         <v>250</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="15" t="s">
         <v>251</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
         <v>252</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
         <v>253</v>
       </c>
       <c r="D6" s="13"/>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="15" t="s">
         <v>254</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
         <v>255</v>
       </c>
       <c r="D8" s="13"/>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
         <v>256</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
         <v>257</v>
       </c>
       <c r="D10" s="13"/>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
         <v>258</v>
       </c>
       <c r="D11" s="13"/>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="16" t="s">
         <v>259</v>
       </c>
       <c r="D12" s="13"/>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="16" t="s">
         <v>260</v>
       </c>
       <c r="D13" s="13"/>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="17" t="s">
         <v>204</v>
       </c>
       <c r="D14" s="13"/>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="18" t="s">
         <v>261</v>
       </c>
       <c r="D15" s="13"/>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="16" t="s">
         <v>262</v>
       </c>
       <c r="D16" s="13"/>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="16" t="s">
         <v>228</v>
       </c>
       <c r="D17" s="13"/>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="16" t="s">
         <v>263</v>
       </c>
       <c r="D18" s="13"/>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="15" t="s">
         <v>264</v>
       </c>
       <c r="D19" s="13"/>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="15" t="s">
         <v>87</v>
       </c>
       <c r="D20" s="13"/>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="17" t="s">
         <v>265</v>
       </c>
       <c r="D21" s="13"/>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="17" t="s">
         <v>266</v>
       </c>
       <c r="D22" s="13"/>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="17" t="s">
         <v>267</v>
       </c>
       <c r="D23" s="13"/>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="17" t="s">
         <v>268</v>
       </c>
       <c r="D24" s="13"/>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="17" t="s">
         <v>269</v>
       </c>
@@ -2643,7 +2645,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="17" t="s">
         <v>270</v>
       </c>
@@ -2651,115 +2653,115 @@
         <v>35</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="16" t="s">
         <v>271</v>
       </c>
       <c r="D27" s="13"/>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="16" t="s">
         <v>83</v>
       </c>
       <c r="D28" s="13"/>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="16" t="s">
         <v>272</v>
       </c>
       <c r="D29" s="13"/>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="16" t="s">
         <v>90</v>
       </c>
       <c r="D30" s="13"/>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="16" t="s">
         <v>273</v>
       </c>
       <c r="D31" s="13"/>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="16" t="s">
         <v>274</v>
       </c>
       <c r="D32" s="13"/>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="16" t="s">
         <v>275</v>
       </c>
       <c r="D33" s="13"/>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" s="16" t="s">
         <v>276</v>
       </c>
       <c r="D34" s="13"/>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" s="14" t="s">
         <v>97</v>
       </c>
       <c r="D35" s="13"/>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" s="16" t="s">
         <v>277</v>
       </c>
       <c r="D36" s="13"/>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" s="16" t="s">
         <v>278</v>
       </c>
       <c r="D37" s="13"/>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" s="16" t="s">
         <v>279</v>
       </c>
       <c r="D38" s="13"/>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" s="16" t="s">
         <v>280</v>
       </c>
       <c r="D39" s="13"/>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" s="16" t="s">
         <v>212</v>
       </c>
       <c r="D40" s="13"/>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" s="16" t="s">
         <v>281</v>
       </c>
       <c r="D41" s="13"/>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" s="16" t="s">
         <v>282</v>
       </c>
       <c r="D42" s="13"/>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" s="16" t="s">
         <v>283</v>
       </c>
       <c r="D43" s="13"/>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" s="16" t="s">
         <v>284</v>
       </c>
       <c r="D44" s="13"/>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" s="16" t="s">
         <v>84</v>
       </c>
@@ -2767,7 +2769,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" s="16" t="s">
         <v>85</v>
       </c>
@@ -2775,7 +2777,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" s="16" t="s">
         <v>86</v>
       </c>
@@ -2783,7 +2785,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" s="16" t="s">
         <v>88</v>
       </c>
@@ -2791,7 +2793,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" s="16" t="s">
         <v>89</v>
       </c>
@@ -2799,7 +2801,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" s="16" t="s">
         <v>91</v>
       </c>
@@ -2807,7 +2809,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" s="16" t="s">
         <v>94</v>
       </c>
@@ -2815,7 +2817,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" s="16" t="s">
         <v>96</v>
       </c>
@@ -2823,7 +2825,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" s="16" t="s">
         <v>95</v>
       </c>
@@ -2831,7 +2833,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" s="15" t="s">
         <v>92</v>
       </c>
@@ -2839,7 +2841,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" s="15" t="s">
         <v>93</v>
       </c>
@@ -2847,7 +2849,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" s="15" t="s">
         <v>36</v>
       </c>
@@ -2855,7 +2857,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" s="18" t="s">
         <v>40</v>
       </c>
@@ -2863,7 +2865,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" s="18" t="s">
         <v>39</v>
       </c>
@@ -2871,7 +2873,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" s="18" t="s">
         <v>38</v>
       </c>
@@ -2879,7 +2881,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" s="18" t="s">
         <v>34</v>
       </c>
@@ -2887,7 +2889,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" s="18" t="s">
         <v>37</v>
       </c>
@@ -2895,7 +2897,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" s="15" t="s">
         <v>98</v>
       </c>
@@ -2903,7 +2905,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" s="15" t="s">
         <v>99</v>
       </c>
@@ -2911,127 +2913,127 @@
         <v>35</v>
       </c>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" s="17" t="s">
         <v>285</v>
       </c>
       <c r="D64" s="13"/>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" s="13" t="s">
         <v>286</v>
       </c>
       <c r="D65" s="13"/>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" s="13" t="s">
         <v>287</v>
       </c>
       <c r="D66" s="13"/>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" s="13" t="s">
         <v>237</v>
       </c>
       <c r="D67" s="13"/>
     </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" s="13" t="s">
         <v>288</v>
       </c>
       <c r="D68" s="13"/>
     </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>289</v>
       </c>
       <c r="D69" s="13"/>
     </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>221</v>
       </c>
       <c r="D70" s="13"/>
     </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>290</v>
       </c>
       <c r="D71" s="13"/>
     </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>291</v>
       </c>
       <c r="D72" s="13"/>
     </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>249</v>
       </c>
       <c r="D73" s="13"/>
     </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>214</v>
       </c>
       <c r="D74" s="13"/>
     </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>292</v>
       </c>
       <c r="D75" s="13"/>
     </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>293</v>
       </c>
       <c r="D76" s="13"/>
     </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>202</v>
       </c>
       <c r="D77" s="13"/>
     </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>294</v>
       </c>
       <c r="D78" s="13"/>
     </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>295</v>
       </c>
       <c r="D79" s="13"/>
     </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>296</v>
       </c>
       <c r="D80" s="13"/>
     </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>297</v>
       </c>
       <c r="D81" s="13"/>
     </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>298</v>
       </c>
       <c r="D82" s="13"/>
     </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>299</v>
       </c>
       <c r="D83" s="13"/>
     </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>230</v>
       </c>
@@ -3039,7 +3041,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>246</v>
       </c>
@@ -3047,7 +3049,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>248</v>
       </c>
@@ -3055,7 +3057,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>217</v>
       </c>
@@ -3063,7 +3065,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>300</v>
       </c>
@@ -3071,7 +3073,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>208</v>
       </c>
@@ -3079,7 +3081,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>229</v>
       </c>
@@ -3087,7 +3089,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>211</v>
       </c>
@@ -3095,7 +3097,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>241</v>
       </c>
@@ -3103,7 +3105,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>226</v>
       </c>
@@ -3111,7 +3113,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>242</v>
       </c>
@@ -3119,7 +3121,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>243</v>
       </c>
@@ -3127,37 +3129,37 @@
         <v>35</v>
       </c>
     </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>301</v>
       </c>
       <c r="D96" s="13"/>
     </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>302</v>
       </c>
       <c r="D97" s="13"/>
     </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>303</v>
       </c>
       <c r="D98" s="13"/>
     </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>304</v>
       </c>
       <c r="D99" s="13"/>
     </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>305</v>
       </c>
       <c r="D100" s="13"/>
     </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" s="19" t="s">
         <v>247</v>
       </c>
@@ -3165,7 +3167,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A102" s="19" t="s">
         <v>235</v>
       </c>
@@ -3173,7 +3175,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A103" s="19" t="s">
         <v>220</v>
       </c>
@@ -3181,7 +3183,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A104" s="19" t="s">
         <v>233</v>
       </c>
@@ -3189,7 +3191,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A105" s="19" t="s">
         <v>213</v>
       </c>
@@ -3197,7 +3199,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="106" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A106" s="19" t="s">
         <v>205</v>
       </c>
@@ -3205,7 +3207,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A107" s="19" t="s">
         <v>224</v>
       </c>
@@ -3213,7 +3215,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A108" s="19" t="s">
         <v>239</v>
       </c>
@@ -3221,7 +3223,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A109" s="19" t="s">
         <v>216</v>
       </c>
@@ -3229,7 +3231,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A110" s="19" t="s">
         <v>201</v>
       </c>
@@ -3237,7 +3239,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A111" s="19" t="s">
         <v>238</v>
       </c>
@@ -3245,7 +3247,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="112" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A112" s="19" t="s">
         <v>231</v>
       </c>
@@ -3253,7 +3255,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="113" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A113" s="19" t="s">
         <v>209</v>
       </c>
@@ -3261,7 +3263,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="114" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A114" s="19" t="s">
         <v>215</v>
       </c>
@@ -3269,7 +3271,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="115" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A115" s="19" t="s">
         <v>232</v>
       </c>
@@ -3277,7 +3279,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="116" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A116" s="19" t="s">
         <v>244</v>
       </c>
@@ -3285,7 +3287,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="117" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A117" s="19" t="s">
         <v>223</v>
       </c>
@@ -3293,7 +3295,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="118" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A118" s="19" t="s">
         <v>218</v>
       </c>
@@ -3301,7 +3303,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="119" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A119" s="19" t="s">
         <v>236</v>
       </c>
@@ -3309,7 +3311,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="120" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A120" s="19" t="s">
         <v>225</v>
       </c>
@@ -3317,7 +3319,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="121" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A121" s="19" t="s">
         <v>234</v>
       </c>
@@ -3325,7 +3327,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="122" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A122" s="19" t="s">
         <v>222</v>
       </c>
@@ -3333,7 +3335,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="123" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A123" s="19" t="s">
         <v>219</v>
       </c>
@@ -3341,7 +3343,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="124" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A124" s="19" t="s">
         <v>240</v>
       </c>
@@ -3349,7 +3351,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="125" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A125" s="19" t="s">
         <v>210</v>
       </c>
@@ -3357,7 +3359,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="126" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A126" s="19" t="s">
         <v>207</v>
       </c>
@@ -3365,7 +3367,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="127" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A127" s="19" t="s">
         <v>227</v>
       </c>
@@ -3373,7 +3375,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="128" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A128" s="19" t="s">
         <v>203</v>
       </c>
@@ -3381,7 +3383,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="129" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A129" s="19" t="s">
         <v>206</v>
       </c>
@@ -3389,7 +3391,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="130" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A130" s="19" t="s">
         <v>245</v>
       </c>
@@ -3397,8 +3399,32 @@
         <v>35</v>
       </c>
     </row>
+    <row r="131" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A131" t="s">
+        <v>270</v>
+      </c>
+      <c r="D131" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="132" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A132" t="s">
+        <v>269</v>
+      </c>
+      <c r="D132" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="133" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A133" t="s">
+        <v>308</v>
+      </c>
+      <c r="D133" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:A130" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
+  <autoFilter ref="A1:A130"/>
   <conditionalFormatting sqref="A3:A130">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
@@ -3408,11 +3434,11 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="9.26953125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3423,7 +3449,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>19</v>
       </c>
@@ -3431,7 +3457,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>21</v>
       </c>
@@ -3439,7 +3465,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>23</v>
       </c>

</xml_diff>

<commit_message>
update process handling and unit definitions: refine commodity categorization and add new unit mapping
</commit_message>
<xml_diff>
--- a/config_data/mapping_v4.xlsx
+++ b/config_data/mapping_v4.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20395"/>
-  <workbookPr defaultThemeVersion="166925"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Xchange\Studis\Apath\materials_DAdapter\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Xchange\Studis\Apath\HiWi Project\config_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF0B9B68-99F5-441C-B2EB-6655F9C29328}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="8150" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="8145" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="SEDOS_parameters" sheetId="5" r:id="rId1"/>
@@ -18,7 +17,7 @@
     <sheet name="limits" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">commodity_set!$A$1:$A$130</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">commodity_set!$A$1:$A$131</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
@@ -30,12 +29,12 @@
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Islam, Md Anik</author>
   </authors>
   <commentList>
-    <comment ref="B43" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
+    <comment ref="B43" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -65,12 +64,12 @@
 </file>
 
 <file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Gary Goldstein</author>
   </authors>
   <commentList>
-    <comment ref="D1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000001000000}">
+    <comment ref="D1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -92,7 +91,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="413" uniqueCount="308">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="415" uniqueCount="309">
   <si>
     <t>TIMES</t>
   </si>
@@ -1016,12 +1015,15 @@
   </si>
   <si>
     <t>ACTFLO~DEMO</t>
+  </si>
+  <si>
+    <t>emi_co2_neg_air_dacc</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1192,8 +1194,8 @@
     </xf>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 10" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
+    <cellStyle name="Normal 10" xfId="1"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="1">
     <dxf>
@@ -1515,22 +1517,22 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:O120"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="37.7265625" customWidth="1"/>
-    <col min="2" max="2" width="25.7265625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="31.81640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.26953125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="37.7109375" customWidth="1"/>
+    <col min="2" max="2" width="25.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="31.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.28515625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="18" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.7265625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.7265625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="22.26953125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -1562,7 +1564,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>100</v>
       </c>
@@ -1573,7 +1575,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>5</v>
       </c>
@@ -1584,7 +1586,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>81</v>
       </c>
@@ -1598,7 +1600,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>101</v>
       </c>
@@ -1619,7 +1621,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
         <v>46</v>
       </c>
@@ -1632,7 +1634,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>6</v>
       </c>
@@ -1643,7 +1645,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
         <v>102</v>
       </c>
@@ -1652,7 +1654,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>74</v>
       </c>
@@ -1663,7 +1665,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>103</v>
       </c>
@@ -1677,7 +1679,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>104</v>
       </c>
@@ -1691,7 +1693,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>64</v>
       </c>
@@ -1702,7 +1704,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>105</v>
       </c>
@@ -1716,7 +1718,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>106</v>
       </c>
@@ -1730,7 +1732,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>56</v>
       </c>
@@ -1741,7 +1743,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>107</v>
       </c>
@@ -1755,7 +1757,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>108</v>
       </c>
@@ -1769,7 +1771,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>109</v>
       </c>
@@ -1780,7 +1782,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>75</v>
       </c>
@@ -1794,7 +1796,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>72</v>
       </c>
@@ -1808,7 +1810,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>63</v>
       </c>
@@ -1822,7 +1824,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>4</v>
       </c>
@@ -1833,7 +1835,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>110</v>
       </c>
@@ -1844,7 +1846,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" s="9" t="s">
         <v>111</v>
       </c>
@@ -1855,7 +1857,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>112</v>
       </c>
@@ -1867,7 +1869,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>76</v>
       </c>
@@ -1878,7 +1880,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>66</v>
       </c>
@@ -1889,7 +1891,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>59</v>
       </c>
@@ -1900,7 +1902,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>113</v>
       </c>
@@ -1911,7 +1913,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>78</v>
       </c>
@@ -1922,7 +1924,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>68</v>
       </c>
@@ -1933,7 +1935,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>60</v>
       </c>
@@ -1944,7 +1946,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>114</v>
       </c>
@@ -1955,7 +1957,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>70</v>
       </c>
@@ -1966,7 +1968,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>115</v>
       </c>
@@ -1974,7 +1976,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>61</v>
       </c>
@@ -1985,7 +1987,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>116</v>
       </c>
@@ -1996,7 +1998,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>117</v>
       </c>
@@ -2010,7 +2012,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>118</v>
       </c>
@@ -2024,7 +2026,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
         <v>119</v>
       </c>
@@ -2038,7 +2040,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>120</v>
       </c>
@@ -2049,7 +2051,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
         <v>121</v>
       </c>
@@ -2058,7 +2060,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
         <v>122</v>
       </c>
@@ -2072,7 +2074,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
         <v>123</v>
       </c>
@@ -2083,7 +2085,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
         <v>124</v>
       </c>
@@ -2094,7 +2096,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" s="9" t="s">
         <v>125</v>
       </c>
@@ -2103,7 +2105,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" s="9" t="s">
         <v>126</v>
       </c>
@@ -2112,7 +2114,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" s="9" t="s">
         <v>127</v>
       </c>
@@ -2121,7 +2123,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" s="9" t="s">
         <v>128</v>
       </c>
@@ -2130,7 +2132,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" s="9" t="s">
         <v>129</v>
       </c>
@@ -2139,7 +2141,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" s="9" t="s">
         <v>130</v>
       </c>
@@ -2148,7 +2150,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" s="9" t="s">
         <v>131</v>
       </c>
@@ -2157,7 +2159,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" s="9" t="s">
         <v>132</v>
       </c>
@@ -2166,7 +2168,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
         <v>133</v>
       </c>
@@ -2177,7 +2179,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" s="9" t="s">
         <v>134</v>
       </c>
@@ -2186,7 +2188,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
         <v>135</v>
       </c>
@@ -2197,7 +2199,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57" s="10" t="s">
         <v>136</v>
       </c>
@@ -2208,7 +2210,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" s="10" t="s">
         <v>137</v>
       </c>
@@ -2217,7 +2219,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" s="9" t="s">
         <v>138</v>
       </c>
@@ -2226,7 +2228,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" s="9" t="s">
         <v>139</v>
       </c>
@@ -2235,7 +2237,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" s="10" t="s">
         <v>140</v>
       </c>
@@ -2246,19 +2248,19 @@
         <v>196</v>
       </c>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" s="7" t="s">
         <v>141</v>
       </c>
       <c r="B62" s="6"/>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" s="7" t="s">
         <v>142</v>
       </c>
       <c r="B63" s="6"/>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A64" s="7" t="s">
         <v>143</v>
       </c>
@@ -2267,199 +2269,199 @@
         <v>197</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65" s="7" t="s">
         <v>41</v>
       </c>
       <c r="B65" s="6"/>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A66" s="7" t="s">
         <v>144</v>
       </c>
       <c r="B66" s="6"/>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A67" s="7" t="s">
         <v>145</v>
       </c>
       <c r="B67" s="6"/>
     </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A68" s="7" t="s">
         <v>146</v>
       </c>
       <c r="B68" s="6"/>
     </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A69" s="7" t="s">
         <v>147</v>
       </c>
       <c r="B69" s="6"/>
     </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A70" s="7" t="s">
         <v>148</v>
       </c>
       <c r="B70" s="6"/>
     </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A71" s="7" t="s">
         <v>47</v>
       </c>
       <c r="B71" s="6"/>
     </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A72" s="7" t="s">
         <v>149</v>
       </c>
       <c r="B72" s="6"/>
     </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A73" s="7" t="s">
         <v>48</v>
       </c>
       <c r="B73" s="6"/>
     </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B74" s="6"/>
     </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B75" s="6"/>
     </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B76" s="6"/>
     </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B77" s="6"/>
     </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B78" s="6"/>
     </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B79" s="6"/>
     </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B80" s="6"/>
     </row>
-    <row r="81" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="81" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B81" s="6"/>
     </row>
-    <row r="82" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="82" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B82" s="6"/>
     </row>
-    <row r="83" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="83" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B83" s="6"/>
     </row>
-    <row r="84" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="84" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B84" s="6"/>
     </row>
-    <row r="85" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="85" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B85" s="6"/>
     </row>
-    <row r="86" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="86" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B86" s="6"/>
     </row>
-    <row r="87" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="87" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B87" s="6"/>
     </row>
-    <row r="88" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="88" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B88" s="6"/>
     </row>
-    <row r="89" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="89" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B89" s="6"/>
     </row>
-    <row r="90" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="90" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B90" s="6"/>
     </row>
-    <row r="91" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="91" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B91" s="6"/>
     </row>
-    <row r="92" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="92" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B92" s="6"/>
     </row>
-    <row r="93" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="93" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B93" s="6"/>
     </row>
-    <row r="94" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="94" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B94" s="6"/>
     </row>
-    <row r="95" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="95" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B95" s="6"/>
     </row>
-    <row r="96" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="96" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B96" s="6"/>
     </row>
-    <row r="97" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="97" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B97" s="6"/>
     </row>
-    <row r="98" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="98" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B98" s="6"/>
     </row>
-    <row r="99" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="99" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B99" s="6"/>
     </row>
-    <row r="100" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="100" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B100" s="6"/>
     </row>
-    <row r="101" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="101" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B101" s="6"/>
     </row>
-    <row r="102" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="102" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B102" s="6"/>
     </row>
-    <row r="103" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="103" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B103" s="6"/>
     </row>
-    <row r="104" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="104" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B104" s="6"/>
     </row>
-    <row r="105" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="105" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B105" s="6"/>
     </row>
-    <row r="106" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="106" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B106" s="6"/>
     </row>
-    <row r="107" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="107" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B107" s="6"/>
     </row>
-    <row r="108" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="108" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B108" s="6"/>
     </row>
-    <row r="109" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="109" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B109" s="6"/>
     </row>
-    <row r="110" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="110" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B110" s="6"/>
     </row>
-    <row r="111" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="111" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B111" s="6"/>
     </row>
-    <row r="112" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="112" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B112" s="6"/>
     </row>
-    <row r="113" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="113" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B113" s="6"/>
     </row>
-    <row r="114" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="114" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B114" s="6"/>
     </row>
-    <row r="115" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="115" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B115" s="6"/>
     </row>
-    <row r="116" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="116" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B116" s="6"/>
     </row>
-    <row r="117" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="117" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B117" s="6"/>
     </row>
-    <row r="118" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="118" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B118" s="6"/>
     </row>
-    <row r="119" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="119" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B119" s="6"/>
     </row>
-    <row r="120" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="120" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B120" s="6"/>
     </row>
   </sheetData>
@@ -2470,17 +2472,17 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:D130"/>
-  <sheetFormatPr defaultColWidth="9.26953125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D131"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="32.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.54296875" customWidth="1"/>
-    <col min="3" max="3" width="15.453125" customWidth="1"/>
-    <col min="4" max="4" width="23.7265625" customWidth="1"/>
+    <col min="1" max="1" width="32.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.5703125" customWidth="1"/>
+    <col min="3" max="3" width="15.42578125" customWidth="1"/>
+    <col min="4" max="4" width="23.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>27</v>
       </c>
@@ -2494,7 +2496,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:4" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
         <v>31</v>
       </c>
@@ -2508,134 +2510,134 @@
         <v>33</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
         <v>250</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="15" t="s">
         <v>251</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
         <v>252</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
         <v>253</v>
       </c>
       <c r="D6" s="13"/>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="15" t="s">
         <v>254</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
         <v>255</v>
       </c>
       <c r="D8" s="13"/>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
         <v>256</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
         <v>257</v>
       </c>
       <c r="D10" s="13"/>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
         <v>258</v>
       </c>
       <c r="D11" s="13"/>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="16" t="s">
         <v>259</v>
       </c>
       <c r="D12" s="13"/>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="16" t="s">
         <v>260</v>
       </c>
       <c r="D13" s="13"/>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="17" t="s">
         <v>204</v>
       </c>
       <c r="D14" s="13"/>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="18" t="s">
         <v>261</v>
       </c>
       <c r="D15" s="13"/>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="16" t="s">
         <v>262</v>
       </c>
       <c r="D16" s="13"/>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="16" t="s">
         <v>228</v>
       </c>
       <c r="D17" s="13"/>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="16" t="s">
         <v>263</v>
       </c>
       <c r="D18" s="13"/>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="15" t="s">
         <v>264</v>
       </c>
       <c r="D19" s="13"/>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="15" t="s">
         <v>87</v>
       </c>
       <c r="D20" s="13"/>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="17" t="s">
         <v>265</v>
       </c>
       <c r="D21" s="13"/>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="17" t="s">
         <v>266</v>
       </c>
       <c r="D22" s="13"/>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="17" t="s">
         <v>267</v>
       </c>
       <c r="D23" s="13"/>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="17" t="s">
         <v>268</v>
       </c>
       <c r="D24" s="13"/>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="17" t="s">
         <v>269</v>
       </c>
@@ -2643,763 +2645,771 @@
         <v>35</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A26" s="17" t="s">
+    <row r="26" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>308</v>
+      </c>
+      <c r="D26" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27" s="17" t="s">
         <v>270</v>
       </c>
-      <c r="D26" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A27" s="16" t="s">
+      <c r="D27" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28" s="16" t="s">
         <v>271</v>
       </c>
-      <c r="D27" s="13"/>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A28" s="16" t="s">
+      <c r="D28" s="13"/>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29" s="16" t="s">
         <v>83</v>
       </c>
-      <c r="D28" s="13"/>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A29" s="16" t="s">
+      <c r="D29" s="13"/>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30" s="16" t="s">
         <v>272</v>
       </c>
-      <c r="D29" s="13"/>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A30" s="16" t="s">
+      <c r="D30" s="13"/>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A31" s="16" t="s">
         <v>90</v>
       </c>
-      <c r="D30" s="13"/>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A31" s="16" t="s">
+      <c r="D31" s="13"/>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A32" s="16" t="s">
         <v>273</v>
       </c>
-      <c r="D31" s="13"/>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A32" s="16" t="s">
+      <c r="D32" s="13"/>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A33" s="16" t="s">
         <v>274</v>
       </c>
-      <c r="D32" s="13"/>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A33" s="16" t="s">
+      <c r="D33" s="13"/>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A34" s="16" t="s">
         <v>275</v>
       </c>
-      <c r="D33" s="13"/>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A34" s="16" t="s">
+      <c r="D34" s="13"/>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A35" s="16" t="s">
         <v>276</v>
       </c>
-      <c r="D34" s="13"/>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A35" s="14" t="s">
+      <c r="D35" s="13"/>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A36" s="14" t="s">
         <v>97</v>
       </c>
-      <c r="D35" s="13"/>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A36" s="16" t="s">
+      <c r="D36" s="13"/>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A37" s="16" t="s">
         <v>277</v>
       </c>
-      <c r="D36" s="13"/>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A37" s="16" t="s">
+      <c r="D37" s="13"/>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A38" s="16" t="s">
         <v>278</v>
       </c>
-      <c r="D37" s="13"/>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A38" s="16" t="s">
+      <c r="D38" s="13"/>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A39" s="16" t="s">
         <v>279</v>
       </c>
-      <c r="D38" s="13"/>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A39" s="16" t="s">
+      <c r="D39" s="13"/>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A40" s="16" t="s">
         <v>280</v>
       </c>
-      <c r="D39" s="13"/>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A40" s="16" t="s">
+      <c r="D40" s="13"/>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A41" s="16" t="s">
         <v>212</v>
       </c>
-      <c r="D40" s="13"/>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A41" s="16" t="s">
+      <c r="D41" s="13"/>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A42" s="16" t="s">
         <v>281</v>
       </c>
-      <c r="D41" s="13"/>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A42" s="16" t="s">
+      <c r="D42" s="13"/>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A43" s="16" t="s">
         <v>282</v>
       </c>
-      <c r="D42" s="13"/>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A43" s="16" t="s">
+      <c r="D43" s="13"/>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A44" s="16" t="s">
         <v>283</v>
       </c>
-      <c r="D43" s="13"/>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A44" s="16" t="s">
+      <c r="D44" s="13"/>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A45" s="16" t="s">
         <v>284</v>
       </c>
-      <c r="D44" s="13"/>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A45" s="16" t="s">
+      <c r="D45" s="13"/>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A46" s="16" t="s">
         <v>84</v>
       </c>
-      <c r="D45" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A46" s="16" t="s">
+      <c r="D46" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A47" s="16" t="s">
         <v>85</v>
       </c>
-      <c r="D46" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A47" s="16" t="s">
+      <c r="D47" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A48" s="16" t="s">
         <v>86</v>
       </c>
-      <c r="D47" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A48" s="16" t="s">
+      <c r="D48" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A49" s="16" t="s">
         <v>88</v>
       </c>
-      <c r="D48" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A49" s="16" t="s">
+      <c r="D49" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A50" s="16" t="s">
         <v>89</v>
       </c>
-      <c r="D49" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A50" s="16" t="s">
+      <c r="D50" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A51" s="16" t="s">
         <v>91</v>
       </c>
-      <c r="D50" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A51" s="16" t="s">
+      <c r="D51" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A52" s="16" t="s">
         <v>94</v>
       </c>
-      <c r="D51" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A52" s="16" t="s">
+      <c r="D52" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A53" s="16" t="s">
         <v>96</v>
       </c>
-      <c r="D52" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A53" s="16" t="s">
+      <c r="D53" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A54" s="16" t="s">
         <v>95</v>
       </c>
-      <c r="D53" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A54" s="15" t="s">
+      <c r="D54" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A55" s="15" t="s">
         <v>92</v>
       </c>
-      <c r="D54" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A55" s="15" t="s">
+      <c r="D55" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A56" s="15" t="s">
         <v>93</v>
       </c>
-      <c r="D55" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A56" s="15" t="s">
+      <c r="D56" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A57" s="15" t="s">
         <v>36</v>
       </c>
-      <c r="D56" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A57" s="18" t="s">
+      <c r="D57" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A58" s="18" t="s">
         <v>40</v>
       </c>
-      <c r="D57" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A58" s="18" t="s">
+      <c r="D58" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A59" s="18" t="s">
         <v>39</v>
       </c>
-      <c r="D58" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A59" s="18" t="s">
+      <c r="D59" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A60" s="18" t="s">
         <v>38</v>
       </c>
-      <c r="D59" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A60" s="18" t="s">
+      <c r="D60" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A61" s="18" t="s">
         <v>34</v>
       </c>
-      <c r="D60" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A61" s="18" t="s">
+      <c r="D61" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A62" s="18" t="s">
         <v>37</v>
       </c>
-      <c r="D61" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A62" s="15" t="s">
+      <c r="D62" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A63" s="15" t="s">
         <v>98</v>
       </c>
-      <c r="D62" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A63" s="15" t="s">
+      <c r="D63" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A64" s="15" t="s">
         <v>99</v>
       </c>
-      <c r="D63" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A64" s="17" t="s">
+      <c r="D64" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A65" s="17" t="s">
         <v>285</v>
       </c>
-      <c r="D64" s="13"/>
-    </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A65" s="13" t="s">
+      <c r="D65" s="13"/>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A66" s="13" t="s">
         <v>286</v>
       </c>
-      <c r="D65" s="13"/>
-    </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A66" s="13" t="s">
+      <c r="D66" s="13"/>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A67" s="13" t="s">
         <v>287</v>
       </c>
-      <c r="D66" s="13"/>
-    </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A67" s="13" t="s">
+      <c r="D67" s="13"/>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A68" s="13" t="s">
         <v>237</v>
       </c>
-      <c r="D67" s="13"/>
-    </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A68" s="13" t="s">
+      <c r="D68" s="13"/>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A69" s="13" t="s">
         <v>288</v>
       </c>
-      <c r="D68" s="13"/>
-    </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A69" t="s">
+      <c r="D69" s="13"/>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
         <v>289</v>
       </c>
-      <c r="D69" s="13"/>
-    </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A70" t="s">
+      <c r="D70" s="13"/>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
         <v>221</v>
       </c>
-      <c r="D70" s="13"/>
-    </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A71" t="s">
+      <c r="D71" s="13"/>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
         <v>290</v>
       </c>
-      <c r="D71" s="13"/>
-    </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A72" t="s">
+      <c r="D72" s="13"/>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
         <v>291</v>
       </c>
-      <c r="D72" s="13"/>
-    </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A73" t="s">
+      <c r="D73" s="13"/>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
         <v>249</v>
       </c>
-      <c r="D73" s="13"/>
-    </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A74" t="s">
+      <c r="D74" s="13"/>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
         <v>214</v>
       </c>
-      <c r="D74" s="13"/>
-    </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A75" t="s">
+      <c r="D75" s="13"/>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
         <v>292</v>
       </c>
-      <c r="D75" s="13"/>
-    </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A76" t="s">
+      <c r="D76" s="13"/>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
         <v>293</v>
       </c>
-      <c r="D76" s="13"/>
-    </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A77" t="s">
+      <c r="D77" s="13"/>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
         <v>202</v>
       </c>
-      <c r="D77" s="13"/>
-    </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A78" t="s">
+      <c r="D78" s="13"/>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
         <v>294</v>
       </c>
-      <c r="D78" s="13"/>
-    </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A79" t="s">
+      <c r="D79" s="13"/>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
         <v>295</v>
       </c>
-      <c r="D79" s="13"/>
-    </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A80" t="s">
+      <c r="D80" s="13"/>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
         <v>296</v>
       </c>
-      <c r="D80" s="13"/>
-    </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A81" t="s">
+      <c r="D81" s="13"/>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
         <v>297</v>
       </c>
-      <c r="D81" s="13"/>
-    </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A82" t="s">
+      <c r="D82" s="13"/>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
         <v>298</v>
       </c>
-      <c r="D82" s="13"/>
-    </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A83" t="s">
+      <c r="D83" s="13"/>
+    </row>
+    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
         <v>299</v>
       </c>
-      <c r="D83" s="13"/>
-    </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A84" t="s">
+      <c r="D84" s="13"/>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
         <v>230</v>
       </c>
-      <c r="D84" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A85" t="s">
+      <c r="D85" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
         <v>246</v>
       </c>
-      <c r="D85" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A86" t="s">
+      <c r="D86" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
         <v>248</v>
       </c>
-      <c r="D86" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A87" t="s">
+      <c r="D87" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
         <v>217</v>
       </c>
-      <c r="D87" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A88" t="s">
+      <c r="D88" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
         <v>300</v>
       </c>
-      <c r="D88" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A89" t="s">
+      <c r="D89" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
         <v>208</v>
       </c>
-      <c r="D89" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A90" t="s">
+      <c r="D90" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
         <v>229</v>
       </c>
-      <c r="D90" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A91" t="s">
+      <c r="D91" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
         <v>211</v>
       </c>
-      <c r="D91" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A92" t="s">
+      <c r="D92" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
         <v>241</v>
       </c>
-      <c r="D92" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A93" t="s">
+      <c r="D93" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
         <v>226</v>
       </c>
-      <c r="D93" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A94" t="s">
+      <c r="D94" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
         <v>242</v>
       </c>
-      <c r="D94" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A95" t="s">
+      <c r="D95" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
         <v>243</v>
       </c>
-      <c r="D95" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A96" t="s">
+      <c r="D96" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
         <v>301</v>
       </c>
-      <c r="D96" s="13"/>
-    </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A97" t="s">
+      <c r="D97" s="13"/>
+    </row>
+    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
         <v>302</v>
       </c>
-      <c r="D97" s="13"/>
-    </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A98" t="s">
+      <c r="D98" s="13"/>
+    </row>
+    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
         <v>303</v>
       </c>
-      <c r="D98" s="13"/>
-    </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A99" t="s">
+      <c r="D99" s="13"/>
+    </row>
+    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
         <v>304</v>
       </c>
-      <c r="D99" s="13"/>
-    </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A100" t="s">
+      <c r="D100" s="13"/>
+    </row>
+    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
         <v>305</v>
       </c>
-      <c r="D100" s="13"/>
-    </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A101" s="19" t="s">
+      <c r="D101" s="13"/>
+    </row>
+    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A102" s="19" t="s">
         <v>247</v>
       </c>
-      <c r="D101" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A102" s="19" t="s">
+      <c r="D102" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A103" s="19" t="s">
         <v>235</v>
       </c>
-      <c r="D102" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A103" s="19" t="s">
+      <c r="D103" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A104" s="19" t="s">
         <v>220</v>
       </c>
-      <c r="D103" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A104" s="19" t="s">
+      <c r="D104" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A105" s="19" t="s">
         <v>233</v>
       </c>
-      <c r="D104" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A105" s="19" t="s">
+      <c r="D105" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A106" s="19" t="s">
         <v>213</v>
       </c>
-      <c r="D105" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="106" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A106" s="19" t="s">
+      <c r="D106" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A107" s="19" t="s">
         <v>205</v>
       </c>
-      <c r="D106" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A107" s="19" t="s">
+      <c r="D107" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A108" s="19" t="s">
         <v>224</v>
       </c>
-      <c r="D107" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A108" s="19" t="s">
+      <c r="D108" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A109" s="19" t="s">
         <v>239</v>
       </c>
-      <c r="D108" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A109" s="19" t="s">
+      <c r="D109" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A110" s="19" t="s">
         <v>216</v>
       </c>
-      <c r="D109" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A110" s="19" t="s">
+      <c r="D110" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A111" s="19" t="s">
         <v>201</v>
       </c>
-      <c r="D110" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A111" s="19" t="s">
+      <c r="D111" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A112" s="19" t="s">
         <v>238</v>
       </c>
-      <c r="D111" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="112" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A112" s="19" t="s">
+      <c r="D112" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="113" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A113" s="19" t="s">
         <v>231</v>
       </c>
-      <c r="D112" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="113" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A113" s="19" t="s">
+      <c r="D113" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="114" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A114" s="19" t="s">
         <v>209</v>
       </c>
-      <c r="D113" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="114" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A114" s="19" t="s">
+      <c r="D114" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="115" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A115" s="19" t="s">
         <v>215</v>
       </c>
-      <c r="D114" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="115" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A115" s="19" t="s">
+      <c r="D115" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="116" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A116" s="19" t="s">
         <v>232</v>
       </c>
-      <c r="D115" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="116" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A116" s="19" t="s">
+      <c r="D116" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="117" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A117" s="19" t="s">
         <v>244</v>
       </c>
-      <c r="D116" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="117" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A117" s="19" t="s">
+      <c r="D117" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="118" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A118" s="19" t="s">
         <v>223</v>
       </c>
-      <c r="D117" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="118" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A118" s="19" t="s">
+      <c r="D118" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="119" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A119" s="19" t="s">
         <v>218</v>
       </c>
-      <c r="D118" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="119" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A119" s="19" t="s">
+      <c r="D119" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="120" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A120" s="19" t="s">
         <v>236</v>
       </c>
-      <c r="D119" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="120" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A120" s="19" t="s">
+      <c r="D120" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="121" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A121" s="19" t="s">
         <v>225</v>
       </c>
-      <c r="D120" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="121" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A121" s="19" t="s">
+      <c r="D121" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="122" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A122" s="19" t="s">
         <v>234</v>
       </c>
-      <c r="D121" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="122" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A122" s="19" t="s">
+      <c r="D122" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="123" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A123" s="19" t="s">
         <v>222</v>
       </c>
-      <c r="D122" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="123" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A123" s="19" t="s">
+      <c r="D123" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="124" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A124" s="19" t="s">
         <v>219</v>
       </c>
-      <c r="D123" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="124" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A124" s="19" t="s">
+      <c r="D124" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="125" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A125" s="19" t="s">
         <v>240</v>
       </c>
-      <c r="D124" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="125" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A125" s="19" t="s">
+      <c r="D125" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="126" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A126" s="19" t="s">
         <v>210</v>
       </c>
-      <c r="D125" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="126" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A126" s="19" t="s">
+      <c r="D126" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="127" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A127" s="19" t="s">
         <v>207</v>
       </c>
-      <c r="D126" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="127" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A127" s="19" t="s">
+      <c r="D127" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="128" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A128" s="19" t="s">
         <v>227</v>
       </c>
-      <c r="D127" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="128" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A128" s="19" t="s">
+      <c r="D128" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="129" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A129" s="19" t="s">
         <v>203</v>
       </c>
-      <c r="D128" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="129" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A129" s="19" t="s">
+      <c r="D129" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="130" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A130" s="19" t="s">
         <v>206</v>
       </c>
-      <c r="D129" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="130" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A130" s="19" t="s">
+      <c r="D130" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="131" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A131" s="19" t="s">
         <v>245</v>
       </c>
-      <c r="D130" t="s">
+      <c r="D131" t="s">
         <v>35</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:A130" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
-  <conditionalFormatting sqref="A3:A130">
+  <autoFilter ref="A1:A131"/>
+  <conditionalFormatting sqref="A3:A25 A27:A131">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3408,11 +3418,11 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="9.26953125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3423,7 +3433,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>19</v>
       </c>
@@ -3431,7 +3441,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>21</v>
       </c>
@@ -3439,7 +3449,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>23</v>
       </c>

</xml_diff>

<commit_message>
Update commodity classification logic and modify related Excel files
</commit_message>
<xml_diff>
--- a/config_data/mapping_v4.xlsx
+++ b/config_data/mapping_v4.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20395"/>
-  <workbookPr defaultThemeVersion="166925"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Xchange\Studis\Apath\materials_DAdapter\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Xchange\Studis\Apath\HiWi Project\config_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF0B9B68-99F5-441C-B2EB-6655F9C29328}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="8150" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="8145" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="SEDOS_parameters" sheetId="5" r:id="rId1"/>
@@ -18,7 +17,7 @@
     <sheet name="limits" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">commodity_set!$A$1:$A$130</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">commodity_set!$A$1:$A$131</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
@@ -30,12 +29,12 @@
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Islam, Md Anik</author>
   </authors>
   <commentList>
-    <comment ref="B43" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
+    <comment ref="B43" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -65,12 +64,12 @@
 </file>
 
 <file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Gary Goldstein</author>
   </authors>
   <commentList>
-    <comment ref="D1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000001000000}">
+    <comment ref="D1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -92,7 +91,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="413" uniqueCount="308">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="415" uniqueCount="309">
   <si>
     <t>TIMES</t>
   </si>
@@ -1016,12 +1015,15 @@
   </si>
   <si>
     <t>ACTFLO~DEMO</t>
+  </si>
+  <si>
+    <t>emi_co2_neg_air_dacc</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1192,8 +1194,8 @@
     </xf>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 10" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
+    <cellStyle name="Normal 10" xfId="1"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="1">
     <dxf>
@@ -1515,22 +1517,22 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:O120"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="37.7265625" customWidth="1"/>
-    <col min="2" max="2" width="25.7265625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="31.81640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.26953125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="37.7109375" customWidth="1"/>
+    <col min="2" max="2" width="25.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="31.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.28515625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="18" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.7265625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.7265625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="22.26953125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -1562,7 +1564,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>100</v>
       </c>
@@ -1573,7 +1575,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>5</v>
       </c>
@@ -1584,7 +1586,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>81</v>
       </c>
@@ -1598,7 +1600,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>101</v>
       </c>
@@ -1619,7 +1621,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
         <v>46</v>
       </c>
@@ -1632,7 +1634,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>6</v>
       </c>
@@ -1643,7 +1645,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
         <v>102</v>
       </c>
@@ -1652,7 +1654,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>74</v>
       </c>
@@ -1663,7 +1665,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>103</v>
       </c>
@@ -1677,7 +1679,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>104</v>
       </c>
@@ -1691,7 +1693,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>64</v>
       </c>
@@ -1702,7 +1704,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>105</v>
       </c>
@@ -1716,7 +1718,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>106</v>
       </c>
@@ -1730,7 +1732,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>56</v>
       </c>
@@ -1741,7 +1743,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>107</v>
       </c>
@@ -1755,7 +1757,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>108</v>
       </c>
@@ -1769,7 +1771,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>109</v>
       </c>
@@ -1780,7 +1782,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>75</v>
       </c>
@@ -1794,7 +1796,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>72</v>
       </c>
@@ -1808,7 +1810,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>63</v>
       </c>
@@ -1822,7 +1824,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>4</v>
       </c>
@@ -1833,7 +1835,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>110</v>
       </c>
@@ -1844,7 +1846,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" s="9" t="s">
         <v>111</v>
       </c>
@@ -1855,7 +1857,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>112</v>
       </c>
@@ -1867,7 +1869,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>76</v>
       </c>
@@ -1878,7 +1880,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>66</v>
       </c>
@@ -1889,7 +1891,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>59</v>
       </c>
@@ -1900,7 +1902,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>113</v>
       </c>
@@ -1911,7 +1913,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>78</v>
       </c>
@@ -1922,7 +1924,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>68</v>
       </c>
@@ -1933,7 +1935,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>60</v>
       </c>
@@ -1944,7 +1946,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>114</v>
       </c>
@@ -1955,7 +1957,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>70</v>
       </c>
@@ -1966,7 +1968,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>115</v>
       </c>
@@ -1974,7 +1976,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>61</v>
       </c>
@@ -1985,7 +1987,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>116</v>
       </c>
@@ -1996,7 +1998,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>117</v>
       </c>
@@ -2010,7 +2012,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>118</v>
       </c>
@@ -2024,7 +2026,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
         <v>119</v>
       </c>
@@ -2038,7 +2040,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>120</v>
       </c>
@@ -2049,7 +2051,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
         <v>121</v>
       </c>
@@ -2058,7 +2060,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
         <v>122</v>
       </c>
@@ -2072,7 +2074,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
         <v>123</v>
       </c>
@@ -2083,7 +2085,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
         <v>124</v>
       </c>
@@ -2094,7 +2096,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" s="9" t="s">
         <v>125</v>
       </c>
@@ -2103,7 +2105,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" s="9" t="s">
         <v>126</v>
       </c>
@@ -2112,7 +2114,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" s="9" t="s">
         <v>127</v>
       </c>
@@ -2121,7 +2123,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" s="9" t="s">
         <v>128</v>
       </c>
@@ -2130,7 +2132,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" s="9" t="s">
         <v>129</v>
       </c>
@@ -2139,7 +2141,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" s="9" t="s">
         <v>130</v>
       </c>
@@ -2148,7 +2150,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" s="9" t="s">
         <v>131</v>
       </c>
@@ -2157,7 +2159,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" s="9" t="s">
         <v>132</v>
       </c>
@@ -2166,7 +2168,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
         <v>133</v>
       </c>
@@ -2177,7 +2179,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" s="9" t="s">
         <v>134</v>
       </c>
@@ -2186,7 +2188,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
         <v>135</v>
       </c>
@@ -2197,7 +2199,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57" s="10" t="s">
         <v>136</v>
       </c>
@@ -2208,7 +2210,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" s="10" t="s">
         <v>137</v>
       </c>
@@ -2217,7 +2219,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" s="9" t="s">
         <v>138</v>
       </c>
@@ -2226,7 +2228,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" s="9" t="s">
         <v>139</v>
       </c>
@@ -2235,7 +2237,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" s="10" t="s">
         <v>140</v>
       </c>
@@ -2246,19 +2248,19 @@
         <v>196</v>
       </c>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" s="7" t="s">
         <v>141</v>
       </c>
       <c r="B62" s="6"/>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" s="7" t="s">
         <v>142</v>
       </c>
       <c r="B63" s="6"/>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A64" s="7" t="s">
         <v>143</v>
       </c>
@@ -2267,199 +2269,199 @@
         <v>197</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65" s="7" t="s">
         <v>41</v>
       </c>
       <c r="B65" s="6"/>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A66" s="7" t="s">
         <v>144</v>
       </c>
       <c r="B66" s="6"/>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A67" s="7" t="s">
         <v>145</v>
       </c>
       <c r="B67" s="6"/>
     </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A68" s="7" t="s">
         <v>146</v>
       </c>
       <c r="B68" s="6"/>
     </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A69" s="7" t="s">
         <v>147</v>
       </c>
       <c r="B69" s="6"/>
     </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A70" s="7" t="s">
         <v>148</v>
       </c>
       <c r="B70" s="6"/>
     </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A71" s="7" t="s">
         <v>47</v>
       </c>
       <c r="B71" s="6"/>
     </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A72" s="7" t="s">
         <v>149</v>
       </c>
       <c r="B72" s="6"/>
     </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A73" s="7" t="s">
         <v>48</v>
       </c>
       <c r="B73" s="6"/>
     </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B74" s="6"/>
     </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B75" s="6"/>
     </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B76" s="6"/>
     </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B77" s="6"/>
     </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B78" s="6"/>
     </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B79" s="6"/>
     </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B80" s="6"/>
     </row>
-    <row r="81" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="81" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B81" s="6"/>
     </row>
-    <row r="82" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="82" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B82" s="6"/>
     </row>
-    <row r="83" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="83" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B83" s="6"/>
     </row>
-    <row r="84" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="84" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B84" s="6"/>
     </row>
-    <row r="85" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="85" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B85" s="6"/>
     </row>
-    <row r="86" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="86" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B86" s="6"/>
     </row>
-    <row r="87" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="87" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B87" s="6"/>
     </row>
-    <row r="88" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="88" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B88" s="6"/>
     </row>
-    <row r="89" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="89" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B89" s="6"/>
     </row>
-    <row r="90" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="90" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B90" s="6"/>
     </row>
-    <row r="91" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="91" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B91" s="6"/>
     </row>
-    <row r="92" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="92" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B92" s="6"/>
     </row>
-    <row r="93" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="93" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B93" s="6"/>
     </row>
-    <row r="94" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="94" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B94" s="6"/>
     </row>
-    <row r="95" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="95" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B95" s="6"/>
     </row>
-    <row r="96" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="96" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B96" s="6"/>
     </row>
-    <row r="97" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="97" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B97" s="6"/>
     </row>
-    <row r="98" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="98" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B98" s="6"/>
     </row>
-    <row r="99" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="99" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B99" s="6"/>
     </row>
-    <row r="100" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="100" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B100" s="6"/>
     </row>
-    <row r="101" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="101" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B101" s="6"/>
     </row>
-    <row r="102" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="102" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B102" s="6"/>
     </row>
-    <row r="103" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="103" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B103" s="6"/>
     </row>
-    <row r="104" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="104" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B104" s="6"/>
     </row>
-    <row r="105" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="105" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B105" s="6"/>
     </row>
-    <row r="106" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="106" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B106" s="6"/>
     </row>
-    <row r="107" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="107" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B107" s="6"/>
     </row>
-    <row r="108" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="108" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B108" s="6"/>
     </row>
-    <row r="109" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="109" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B109" s="6"/>
     </row>
-    <row r="110" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="110" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B110" s="6"/>
     </row>
-    <row r="111" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="111" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B111" s="6"/>
     </row>
-    <row r="112" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="112" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B112" s="6"/>
     </row>
-    <row r="113" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="113" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B113" s="6"/>
     </row>
-    <row r="114" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="114" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B114" s="6"/>
     </row>
-    <row r="115" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="115" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B115" s="6"/>
     </row>
-    <row r="116" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="116" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B116" s="6"/>
     </row>
-    <row r="117" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="117" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B117" s="6"/>
     </row>
-    <row r="118" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="118" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B118" s="6"/>
     </row>
-    <row r="119" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="119" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B119" s="6"/>
     </row>
-    <row r="120" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="120" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B120" s="6"/>
     </row>
   </sheetData>
@@ -2470,17 +2472,17 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:D130"/>
-  <sheetFormatPr defaultColWidth="9.26953125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D131"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="32.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.54296875" customWidth="1"/>
-    <col min="3" max="3" width="15.453125" customWidth="1"/>
-    <col min="4" max="4" width="23.7265625" customWidth="1"/>
+    <col min="1" max="1" width="32.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.5703125" customWidth="1"/>
+    <col min="3" max="3" width="15.42578125" customWidth="1"/>
+    <col min="4" max="4" width="23.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>27</v>
       </c>
@@ -2494,7 +2496,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:4" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
         <v>31</v>
       </c>
@@ -2508,898 +2510,906 @@
         <v>33</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
         <v>250</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="15" t="s">
         <v>251</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
         <v>252</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
         <v>253</v>
       </c>
       <c r="D6" s="13"/>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="15" t="s">
         <v>254</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
         <v>255</v>
       </c>
       <c r="D8" s="13"/>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
         <v>256</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
         <v>257</v>
       </c>
       <c r="D10" s="13"/>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
         <v>258</v>
       </c>
       <c r="D11" s="13"/>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="16" t="s">
         <v>259</v>
       </c>
       <c r="D12" s="13"/>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="16" t="s">
         <v>260</v>
       </c>
       <c r="D13" s="13"/>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="17" t="s">
         <v>204</v>
       </c>
       <c r="D14" s="13"/>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="18" t="s">
         <v>261</v>
       </c>
       <c r="D15" s="13"/>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="16" t="s">
         <v>262</v>
       </c>
       <c r="D16" s="13"/>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="16" t="s">
         <v>228</v>
       </c>
       <c r="D17" s="13"/>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="16" t="s">
         <v>263</v>
       </c>
       <c r="D18" s="13"/>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="15" t="s">
         <v>264</v>
       </c>
       <c r="D19" s="13"/>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="15" t="s">
         <v>87</v>
       </c>
       <c r="D20" s="13"/>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="17" t="s">
         <v>265</v>
       </c>
       <c r="D21" s="13"/>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="17" t="s">
         <v>266</v>
       </c>
       <c r="D22" s="13"/>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="17" t="s">
         <v>267</v>
       </c>
       <c r="D23" s="13"/>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="17" t="s">
         <v>268</v>
       </c>
       <c r="D24" s="13"/>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A25" s="17" t="s">
+    <row r="25" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>308</v>
+      </c>
+      <c r="D25" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" s="17" t="s">
         <v>269</v>
       </c>
-      <c r="D25" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A26" s="17" t="s">
+      <c r="D26" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27" s="17" t="s">
         <v>270</v>
       </c>
-      <c r="D26" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A27" s="16" t="s">
+      <c r="D27" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28" s="16" t="s">
         <v>271</v>
       </c>
-      <c r="D27" s="13"/>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A28" s="16" t="s">
+      <c r="D28" s="13"/>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29" s="16" t="s">
         <v>83</v>
       </c>
-      <c r="D28" s="13"/>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A29" s="16" t="s">
+      <c r="D29" s="13"/>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30" s="16" t="s">
         <v>272</v>
       </c>
-      <c r="D29" s="13"/>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A30" s="16" t="s">
+      <c r="D30" s="13"/>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A31" s="16" t="s">
         <v>90</v>
       </c>
-      <c r="D30" s="13"/>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A31" s="16" t="s">
+      <c r="D31" s="13"/>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A32" s="16" t="s">
         <v>273</v>
       </c>
-      <c r="D31" s="13"/>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A32" s="16" t="s">
+      <c r="D32" s="13"/>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A33" s="16" t="s">
         <v>274</v>
       </c>
-      <c r="D32" s="13"/>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A33" s="16" t="s">
+      <c r="D33" s="13"/>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A34" s="16" t="s">
         <v>275</v>
       </c>
-      <c r="D33" s="13"/>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A34" s="16" t="s">
+      <c r="D34" s="13"/>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A35" s="16" t="s">
         <v>276</v>
       </c>
-      <c r="D34" s="13"/>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A35" s="14" t="s">
+      <c r="D35" s="13"/>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A36" s="14" t="s">
         <v>97</v>
       </c>
-      <c r="D35" s="13"/>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A36" s="16" t="s">
+      <c r="D36" s="13"/>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A37" s="16" t="s">
         <v>277</v>
       </c>
-      <c r="D36" s="13"/>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A37" s="16" t="s">
+      <c r="D37" s="13"/>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A38" s="16" t="s">
         <v>278</v>
       </c>
-      <c r="D37" s="13"/>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A38" s="16" t="s">
+      <c r="D38" s="13"/>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A39" s="16" t="s">
         <v>279</v>
       </c>
-      <c r="D38" s="13"/>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A39" s="16" t="s">
+      <c r="D39" s="13"/>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A40" s="16" t="s">
         <v>280</v>
       </c>
-      <c r="D39" s="13"/>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A40" s="16" t="s">
+      <c r="D40" s="13"/>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A41" s="16" t="s">
         <v>212</v>
       </c>
-      <c r="D40" s="13"/>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A41" s="16" t="s">
+      <c r="D41" s="13"/>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A42" s="16" t="s">
         <v>281</v>
       </c>
-      <c r="D41" s="13"/>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A42" s="16" t="s">
+      <c r="D42" s="13"/>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A43" s="16" t="s">
         <v>282</v>
       </c>
-      <c r="D42" s="13"/>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A43" s="16" t="s">
+      <c r="D43" s="13"/>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A44" s="16" t="s">
         <v>283</v>
       </c>
-      <c r="D43" s="13"/>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A44" s="16" t="s">
+      <c r="D44" s="13"/>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A45" s="16" t="s">
         <v>284</v>
       </c>
-      <c r="D44" s="13"/>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A45" s="16" t="s">
+      <c r="D45" s="13"/>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A46" s="16" t="s">
         <v>84</v>
       </c>
-      <c r="D45" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A46" s="16" t="s">
+      <c r="D46" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A47" s="16" t="s">
         <v>85</v>
       </c>
-      <c r="D46" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A47" s="16" t="s">
+      <c r="D47" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A48" s="16" t="s">
         <v>86</v>
       </c>
-      <c r="D47" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A48" s="16" t="s">
+      <c r="D48" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A49" s="16" t="s">
         <v>88</v>
       </c>
-      <c r="D48" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A49" s="16" t="s">
+      <c r="D49" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A50" s="16" t="s">
         <v>89</v>
       </c>
-      <c r="D49" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A50" s="16" t="s">
+      <c r="D50" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A51" s="16" t="s">
         <v>91</v>
       </c>
-      <c r="D50" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A51" s="16" t="s">
+      <c r="D51" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A52" s="16" t="s">
         <v>94</v>
       </c>
-      <c r="D51" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A52" s="16" t="s">
+      <c r="D52" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A53" s="16" t="s">
         <v>96</v>
       </c>
-      <c r="D52" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A53" s="16" t="s">
+      <c r="D53" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A54" s="16" t="s">
         <v>95</v>
       </c>
-      <c r="D53" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A54" s="15" t="s">
+      <c r="D54" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A55" s="15" t="s">
         <v>92</v>
       </c>
-      <c r="D54" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A55" s="15" t="s">
+      <c r="D55" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A56" s="15" t="s">
         <v>93</v>
       </c>
-      <c r="D55" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A56" s="15" t="s">
+      <c r="D56" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A57" s="15" t="s">
         <v>36</v>
       </c>
-      <c r="D56" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A57" s="18" t="s">
+      <c r="D57" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A58" s="18" t="s">
         <v>40</v>
       </c>
-      <c r="D57" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A58" s="18" t="s">
+      <c r="D58" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A59" s="18" t="s">
         <v>39</v>
       </c>
-      <c r="D58" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A59" s="18" t="s">
+      <c r="D59" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A60" s="18" t="s">
         <v>38</v>
       </c>
-      <c r="D59" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A60" s="18" t="s">
+      <c r="D60" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A61" s="18" t="s">
         <v>34</v>
       </c>
-      <c r="D60" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A61" s="18" t="s">
+      <c r="D61" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A62" s="18" t="s">
         <v>37</v>
       </c>
-      <c r="D61" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A62" s="15" t="s">
+      <c r="D62" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A63" s="15" t="s">
         <v>98</v>
       </c>
-      <c r="D62" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A63" s="15" t="s">
+      <c r="D63" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A64" s="15" t="s">
         <v>99</v>
       </c>
-      <c r="D63" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A64" s="17" t="s">
+      <c r="D64" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A65" s="17" t="s">
         <v>285</v>
       </c>
-      <c r="D64" s="13"/>
-    </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A65" s="13" t="s">
+      <c r="D65" s="13"/>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A66" s="13" t="s">
         <v>286</v>
       </c>
-      <c r="D65" s="13"/>
-    </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A66" s="13" t="s">
+      <c r="D66" s="13"/>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A67" s="13" t="s">
         <v>287</v>
       </c>
-      <c r="D66" s="13"/>
-    </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A67" s="13" t="s">
+      <c r="D67" s="13"/>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A68" s="13" t="s">
         <v>237</v>
       </c>
-      <c r="D67" s="13"/>
-    </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A68" s="13" t="s">
+      <c r="D68" s="13"/>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A69" s="13" t="s">
         <v>288</v>
       </c>
-      <c r="D68" s="13"/>
-    </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A69" t="s">
+      <c r="D69" s="13"/>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
         <v>289</v>
       </c>
-      <c r="D69" s="13"/>
-    </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A70" t="s">
+      <c r="D70" s="13"/>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
         <v>221</v>
       </c>
-      <c r="D70" s="13"/>
-    </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A71" t="s">
+      <c r="D71" s="13"/>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
         <v>290</v>
       </c>
-      <c r="D71" s="13"/>
-    </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A72" t="s">
+      <c r="D72" s="13"/>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
         <v>291</v>
       </c>
-      <c r="D72" s="13"/>
-    </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A73" t="s">
+      <c r="D73" s="13"/>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
         <v>249</v>
       </c>
-      <c r="D73" s="13"/>
-    </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A74" t="s">
+      <c r="D74" s="13"/>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
         <v>214</v>
       </c>
-      <c r="D74" s="13"/>
-    </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A75" t="s">
+      <c r="D75" s="13"/>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
         <v>292</v>
       </c>
-      <c r="D75" s="13"/>
-    </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A76" t="s">
+      <c r="D76" s="13"/>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
         <v>293</v>
       </c>
-      <c r="D76" s="13"/>
-    </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A77" t="s">
+      <c r="D77" s="13"/>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
         <v>202</v>
       </c>
-      <c r="D77" s="13"/>
-    </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A78" t="s">
+      <c r="D78" s="13"/>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
         <v>294</v>
       </c>
-      <c r="D78" s="13"/>
-    </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A79" t="s">
+      <c r="D79" s="13"/>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
         <v>295</v>
       </c>
-      <c r="D79" s="13"/>
-    </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A80" t="s">
+      <c r="D80" s="13"/>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
         <v>296</v>
       </c>
-      <c r="D80" s="13"/>
-    </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A81" t="s">
+      <c r="D81" s="13"/>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
         <v>297</v>
       </c>
-      <c r="D81" s="13"/>
-    </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A82" t="s">
+      <c r="D82" s="13"/>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
         <v>298</v>
       </c>
-      <c r="D82" s="13"/>
-    </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A83" t="s">
+      <c r="D83" s="13"/>
+    </row>
+    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
         <v>299</v>
       </c>
-      <c r="D83" s="13"/>
-    </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A84" t="s">
+      <c r="D84" s="13"/>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
         <v>230</v>
       </c>
-      <c r="D84" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A85" t="s">
+      <c r="D85" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
         <v>246</v>
       </c>
-      <c r="D85" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A86" t="s">
+      <c r="D86" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
         <v>248</v>
       </c>
-      <c r="D86" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A87" t="s">
+      <c r="D87" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
         <v>217</v>
       </c>
-      <c r="D87" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A88" t="s">
+      <c r="D88" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
         <v>300</v>
       </c>
-      <c r="D88" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A89" t="s">
+      <c r="D89" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
         <v>208</v>
       </c>
-      <c r="D89" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A90" t="s">
+      <c r="D90" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
         <v>229</v>
       </c>
-      <c r="D90" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A91" t="s">
+      <c r="D91" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
         <v>211</v>
       </c>
-      <c r="D91" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A92" t="s">
+      <c r="D92" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
         <v>241</v>
       </c>
-      <c r="D92" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A93" t="s">
+      <c r="D93" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
         <v>226</v>
       </c>
-      <c r="D93" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A94" t="s">
+      <c r="D94" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
         <v>242</v>
       </c>
-      <c r="D94" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A95" t="s">
+      <c r="D95" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
         <v>243</v>
       </c>
-      <c r="D95" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A96" t="s">
+      <c r="D96" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
         <v>301</v>
       </c>
-      <c r="D96" s="13"/>
-    </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A97" t="s">
+      <c r="D97" s="13"/>
+    </row>
+    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
         <v>302</v>
       </c>
-      <c r="D97" s="13"/>
-    </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A98" t="s">
+      <c r="D98" s="13"/>
+    </row>
+    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
         <v>303</v>
       </c>
-      <c r="D98" s="13"/>
-    </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A99" t="s">
+      <c r="D99" s="13"/>
+    </row>
+    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
         <v>304</v>
       </c>
-      <c r="D99" s="13"/>
-    </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A100" t="s">
+      <c r="D100" s="13"/>
+    </row>
+    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
         <v>305</v>
       </c>
-      <c r="D100" s="13"/>
-    </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A101" s="19" t="s">
+      <c r="D101" s="13"/>
+    </row>
+    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A102" s="19" t="s">
         <v>247</v>
       </c>
-      <c r="D101" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A102" s="19" t="s">
+      <c r="D102" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A103" s="19" t="s">
         <v>235</v>
       </c>
-      <c r="D102" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A103" s="19" t="s">
+      <c r="D103" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A104" s="19" t="s">
         <v>220</v>
       </c>
-      <c r="D103" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A104" s="19" t="s">
+      <c r="D104" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A105" s="19" t="s">
         <v>233</v>
       </c>
-      <c r="D104" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A105" s="19" t="s">
+      <c r="D105" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A106" s="19" t="s">
         <v>213</v>
       </c>
-      <c r="D105" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="106" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A106" s="19" t="s">
+      <c r="D106" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A107" s="19" t="s">
         <v>205</v>
       </c>
-      <c r="D106" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A107" s="19" t="s">
+      <c r="D107" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A108" s="19" t="s">
         <v>224</v>
       </c>
-      <c r="D107" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A108" s="19" t="s">
+      <c r="D108" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A109" s="19" t="s">
         <v>239</v>
       </c>
-      <c r="D108" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A109" s="19" t="s">
+      <c r="D109" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A110" s="19" t="s">
         <v>216</v>
       </c>
-      <c r="D109" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A110" s="19" t="s">
+      <c r="D110" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A111" s="19" t="s">
         <v>201</v>
       </c>
-      <c r="D110" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A111" s="19" t="s">
+      <c r="D111" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A112" s="19" t="s">
         <v>238</v>
       </c>
-      <c r="D111" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="112" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A112" s="19" t="s">
+      <c r="D112" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="113" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A113" s="19" t="s">
         <v>231</v>
       </c>
-      <c r="D112" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="113" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A113" s="19" t="s">
+      <c r="D113" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="114" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A114" s="19" t="s">
         <v>209</v>
       </c>
-      <c r="D113" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="114" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A114" s="19" t="s">
+      <c r="D114" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="115" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A115" s="19" t="s">
         <v>215</v>
       </c>
-      <c r="D114" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="115" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A115" s="19" t="s">
+      <c r="D115" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="116" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A116" s="19" t="s">
         <v>232</v>
       </c>
-      <c r="D115" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="116" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A116" s="19" t="s">
+      <c r="D116" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="117" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A117" s="19" t="s">
         <v>244</v>
       </c>
-      <c r="D116" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="117" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A117" s="19" t="s">
+      <c r="D117" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="118" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A118" s="19" t="s">
         <v>223</v>
       </c>
-      <c r="D117" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="118" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A118" s="19" t="s">
+      <c r="D118" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="119" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A119" s="19" t="s">
         <v>218</v>
       </c>
-      <c r="D118" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="119" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A119" s="19" t="s">
+      <c r="D119" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="120" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A120" s="19" t="s">
         <v>236</v>
       </c>
-      <c r="D119" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="120" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A120" s="19" t="s">
+      <c r="D120" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="121" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A121" s="19" t="s">
         <v>225</v>
       </c>
-      <c r="D120" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="121" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A121" s="19" t="s">
+      <c r="D121" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="122" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A122" s="19" t="s">
         <v>234</v>
       </c>
-      <c r="D121" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="122" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A122" s="19" t="s">
+      <c r="D122" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="123" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A123" s="19" t="s">
         <v>222</v>
       </c>
-      <c r="D122" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="123" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A123" s="19" t="s">
+      <c r="D123" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="124" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A124" s="19" t="s">
         <v>219</v>
       </c>
-      <c r="D123" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="124" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A124" s="19" t="s">
+      <c r="D124" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="125" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A125" s="19" t="s">
         <v>240</v>
       </c>
-      <c r="D124" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="125" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A125" s="19" t="s">
+      <c r="D125" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="126" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A126" s="19" t="s">
         <v>210</v>
       </c>
-      <c r="D125" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="126" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A126" s="19" t="s">
+      <c r="D126" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="127" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A127" s="19" t="s">
         <v>207</v>
       </c>
-      <c r="D126" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="127" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A127" s="19" t="s">
+      <c r="D127" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="128" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A128" s="19" t="s">
         <v>227</v>
       </c>
-      <c r="D127" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="128" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A128" s="19" t="s">
+      <c r="D128" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="129" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A129" s="19" t="s">
         <v>203</v>
       </c>
-      <c r="D128" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="129" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A129" s="19" t="s">
+      <c r="D129" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="130" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A130" s="19" t="s">
         <v>206</v>
       </c>
-      <c r="D129" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="130" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A130" s="19" t="s">
+      <c r="D130" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="131" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A131" s="19" t="s">
         <v>245</v>
       </c>
-      <c r="D130" t="s">
+      <c r="D131" t="s">
         <v>35</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:A130" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
-  <conditionalFormatting sqref="A3:A130">
+  <autoFilter ref="A1:A131"/>
+  <conditionalFormatting sqref="A3:A24 A26:A131">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3408,11 +3418,11 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="9.26953125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3423,7 +3433,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>19</v>
       </c>
@@ -3431,7 +3441,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>21</v>
       </c>
@@ -3439,7 +3449,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>23</v>
       </c>

</xml_diff>

<commit_message>
Refactor commodity classification logic in process_input.py for improved readability and maintainability
</commit_message>
<xml_diff>
--- a/config_data/mapping_v4.xlsx
+++ b/config_data/mapping_v4.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20395"/>
-  <workbookPr defaultThemeVersion="166925"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Xchange\Studis\Apath\materials_DAdapter\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Xchange\Studis\Apath\HiWi Project\config_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF0B9B68-99F5-441C-B2EB-6655F9C29328}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="8150" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="8145" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="SEDOS_parameters" sheetId="5" r:id="rId1"/>
@@ -18,7 +17,7 @@
     <sheet name="limits" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">commodity_set!$A$1:$A$130</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">commodity_set!$A$1:$A$131</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
@@ -30,12 +29,12 @@
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Islam, Md Anik</author>
   </authors>
   <commentList>
-    <comment ref="B43" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
+    <comment ref="B43" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -65,12 +64,12 @@
 </file>
 
 <file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Gary Goldstein</author>
   </authors>
   <commentList>
-    <comment ref="D1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000001000000}">
+    <comment ref="D1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -92,7 +91,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="413" uniqueCount="308">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="415" uniqueCount="309">
   <si>
     <t>TIMES</t>
   </si>
@@ -1016,12 +1015,15 @@
   </si>
   <si>
     <t>ACTFLO~DEMO</t>
+  </si>
+  <si>
+    <t>emi_co2_neg_air_dacc</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1192,8 +1194,8 @@
     </xf>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 10" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
+    <cellStyle name="Normal 10" xfId="1"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="1">
     <dxf>
@@ -1515,22 +1517,22 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:O120"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="37.7265625" customWidth="1"/>
-    <col min="2" max="2" width="25.7265625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="31.81640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.26953125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="37.7109375" customWidth="1"/>
+    <col min="2" max="2" width="25.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="31.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.28515625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="18" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.7265625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.7265625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="22.26953125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -1562,7 +1564,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>100</v>
       </c>
@@ -1573,7 +1575,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>5</v>
       </c>
@@ -1584,7 +1586,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>81</v>
       </c>
@@ -1598,7 +1600,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>101</v>
       </c>
@@ -1619,7 +1621,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
         <v>46</v>
       </c>
@@ -1632,7 +1634,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>6</v>
       </c>
@@ -1643,7 +1645,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
         <v>102</v>
       </c>
@@ -1652,7 +1654,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>74</v>
       </c>
@@ -1663,7 +1665,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>103</v>
       </c>
@@ -1677,7 +1679,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>104</v>
       </c>
@@ -1691,7 +1693,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>64</v>
       </c>
@@ -1702,7 +1704,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>105</v>
       </c>
@@ -1716,7 +1718,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>106</v>
       </c>
@@ -1730,7 +1732,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>56</v>
       </c>
@@ -1741,7 +1743,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>107</v>
       </c>
@@ -1755,7 +1757,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>108</v>
       </c>
@@ -1769,7 +1771,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>109</v>
       </c>
@@ -1780,7 +1782,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>75</v>
       </c>
@@ -1794,7 +1796,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>72</v>
       </c>
@@ -1808,7 +1810,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>63</v>
       </c>
@@ -1822,7 +1824,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>4</v>
       </c>
@@ -1833,7 +1835,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>110</v>
       </c>
@@ -1844,7 +1846,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" s="9" t="s">
         <v>111</v>
       </c>
@@ -1855,7 +1857,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>112</v>
       </c>
@@ -1867,7 +1869,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>76</v>
       </c>
@@ -1878,7 +1880,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>66</v>
       </c>
@@ -1889,7 +1891,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>59</v>
       </c>
@@ -1900,7 +1902,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>113</v>
       </c>
@@ -1911,7 +1913,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>78</v>
       </c>
@@ -1922,7 +1924,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>68</v>
       </c>
@@ -1933,7 +1935,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>60</v>
       </c>
@@ -1944,7 +1946,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>114</v>
       </c>
@@ -1955,7 +1957,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>70</v>
       </c>
@@ -1966,7 +1968,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>115</v>
       </c>
@@ -1974,7 +1976,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>61</v>
       </c>
@@ -1985,7 +1987,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>116</v>
       </c>
@@ -1996,7 +1998,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>117</v>
       </c>
@@ -2010,7 +2012,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>118</v>
       </c>
@@ -2024,7 +2026,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
         <v>119</v>
       </c>
@@ -2038,7 +2040,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>120</v>
       </c>
@@ -2049,7 +2051,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
         <v>121</v>
       </c>
@@ -2058,7 +2060,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
         <v>122</v>
       </c>
@@ -2072,7 +2074,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
         <v>123</v>
       </c>
@@ -2083,7 +2085,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
         <v>124</v>
       </c>
@@ -2094,7 +2096,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" s="9" t="s">
         <v>125</v>
       </c>
@@ -2103,7 +2105,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" s="9" t="s">
         <v>126</v>
       </c>
@@ -2112,7 +2114,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" s="9" t="s">
         <v>127</v>
       </c>
@@ -2121,7 +2123,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" s="9" t="s">
         <v>128</v>
       </c>
@@ -2130,7 +2132,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" s="9" t="s">
         <v>129</v>
       </c>
@@ -2139,7 +2141,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" s="9" t="s">
         <v>130</v>
       </c>
@@ -2148,7 +2150,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" s="9" t="s">
         <v>131</v>
       </c>
@@ -2157,7 +2159,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" s="9" t="s">
         <v>132</v>
       </c>
@@ -2166,7 +2168,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
         <v>133</v>
       </c>
@@ -2177,7 +2179,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" s="9" t="s">
         <v>134</v>
       </c>
@@ -2186,7 +2188,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
         <v>135</v>
       </c>
@@ -2197,7 +2199,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57" s="10" t="s">
         <v>136</v>
       </c>
@@ -2208,7 +2210,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" s="10" t="s">
         <v>137</v>
       </c>
@@ -2217,7 +2219,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" s="9" t="s">
         <v>138</v>
       </c>
@@ -2226,7 +2228,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" s="9" t="s">
         <v>139</v>
       </c>
@@ -2235,7 +2237,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" s="10" t="s">
         <v>140</v>
       </c>
@@ -2246,19 +2248,19 @@
         <v>196</v>
       </c>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" s="7" t="s">
         <v>141</v>
       </c>
       <c r="B62" s="6"/>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" s="7" t="s">
         <v>142</v>
       </c>
       <c r="B63" s="6"/>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A64" s="7" t="s">
         <v>143</v>
       </c>
@@ -2267,199 +2269,199 @@
         <v>197</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65" s="7" t="s">
         <v>41</v>
       </c>
       <c r="B65" s="6"/>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A66" s="7" t="s">
         <v>144</v>
       </c>
       <c r="B66" s="6"/>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A67" s="7" t="s">
         <v>145</v>
       </c>
       <c r="B67" s="6"/>
     </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A68" s="7" t="s">
         <v>146</v>
       </c>
       <c r="B68" s="6"/>
     </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A69" s="7" t="s">
         <v>147</v>
       </c>
       <c r="B69" s="6"/>
     </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A70" s="7" t="s">
         <v>148</v>
       </c>
       <c r="B70" s="6"/>
     </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A71" s="7" t="s">
         <v>47</v>
       </c>
       <c r="B71" s="6"/>
     </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A72" s="7" t="s">
         <v>149</v>
       </c>
       <c r="B72" s="6"/>
     </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A73" s="7" t="s">
         <v>48</v>
       </c>
       <c r="B73" s="6"/>
     </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B74" s="6"/>
     </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B75" s="6"/>
     </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B76" s="6"/>
     </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B77" s="6"/>
     </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B78" s="6"/>
     </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B79" s="6"/>
     </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B80" s="6"/>
     </row>
-    <row r="81" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="81" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B81" s="6"/>
     </row>
-    <row r="82" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="82" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B82" s="6"/>
     </row>
-    <row r="83" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="83" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B83" s="6"/>
     </row>
-    <row r="84" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="84" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B84" s="6"/>
     </row>
-    <row r="85" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="85" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B85" s="6"/>
     </row>
-    <row r="86" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="86" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B86" s="6"/>
     </row>
-    <row r="87" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="87" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B87" s="6"/>
     </row>
-    <row r="88" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="88" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B88" s="6"/>
     </row>
-    <row r="89" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="89" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B89" s="6"/>
     </row>
-    <row r="90" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="90" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B90" s="6"/>
     </row>
-    <row r="91" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="91" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B91" s="6"/>
     </row>
-    <row r="92" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="92" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B92" s="6"/>
     </row>
-    <row r="93" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="93" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B93" s="6"/>
     </row>
-    <row r="94" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="94" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B94" s="6"/>
     </row>
-    <row r="95" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="95" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B95" s="6"/>
     </row>
-    <row r="96" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="96" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B96" s="6"/>
     </row>
-    <row r="97" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="97" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B97" s="6"/>
     </row>
-    <row r="98" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="98" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B98" s="6"/>
     </row>
-    <row r="99" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="99" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B99" s="6"/>
     </row>
-    <row r="100" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="100" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B100" s="6"/>
     </row>
-    <row r="101" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="101" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B101" s="6"/>
     </row>
-    <row r="102" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="102" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B102" s="6"/>
     </row>
-    <row r="103" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="103" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B103" s="6"/>
     </row>
-    <row r="104" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="104" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B104" s="6"/>
     </row>
-    <row r="105" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="105" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B105" s="6"/>
     </row>
-    <row r="106" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="106" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B106" s="6"/>
     </row>
-    <row r="107" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="107" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B107" s="6"/>
     </row>
-    <row r="108" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="108" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B108" s="6"/>
     </row>
-    <row r="109" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="109" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B109" s="6"/>
     </row>
-    <row r="110" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="110" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B110" s="6"/>
     </row>
-    <row r="111" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="111" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B111" s="6"/>
     </row>
-    <row r="112" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="112" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B112" s="6"/>
     </row>
-    <row r="113" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="113" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B113" s="6"/>
     </row>
-    <row r="114" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="114" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B114" s="6"/>
     </row>
-    <row r="115" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="115" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B115" s="6"/>
     </row>
-    <row r="116" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="116" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B116" s="6"/>
     </row>
-    <row r="117" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="117" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B117" s="6"/>
     </row>
-    <row r="118" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="118" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B118" s="6"/>
     </row>
-    <row r="119" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="119" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B119" s="6"/>
     </row>
-    <row r="120" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="120" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B120" s="6"/>
     </row>
   </sheetData>
@@ -2470,17 +2472,17 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:D130"/>
-  <sheetFormatPr defaultColWidth="9.26953125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D131"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="32.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.54296875" customWidth="1"/>
-    <col min="3" max="3" width="15.453125" customWidth="1"/>
-    <col min="4" max="4" width="23.7265625" customWidth="1"/>
+    <col min="1" max="1" width="32.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.5703125" customWidth="1"/>
+    <col min="3" max="3" width="15.42578125" customWidth="1"/>
+    <col min="4" max="4" width="23.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>27</v>
       </c>
@@ -2494,7 +2496,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:4" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
         <v>31</v>
       </c>
@@ -2508,134 +2510,134 @@
         <v>33</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
         <v>250</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="15" t="s">
         <v>251</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
         <v>252</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
         <v>253</v>
       </c>
       <c r="D6" s="13"/>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="15" t="s">
         <v>254</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
         <v>255</v>
       </c>
       <c r="D8" s="13"/>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
         <v>256</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
         <v>257</v>
       </c>
       <c r="D10" s="13"/>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
         <v>258</v>
       </c>
       <c r="D11" s="13"/>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="16" t="s">
         <v>259</v>
       </c>
       <c r="D12" s="13"/>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="16" t="s">
         <v>260</v>
       </c>
       <c r="D13" s="13"/>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="17" t="s">
         <v>204</v>
       </c>
       <c r="D14" s="13"/>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="18" t="s">
         <v>261</v>
       </c>
       <c r="D15" s="13"/>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="16" t="s">
         <v>262</v>
       </c>
       <c r="D16" s="13"/>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="16" t="s">
         <v>228</v>
       </c>
       <c r="D17" s="13"/>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="16" t="s">
         <v>263</v>
       </c>
       <c r="D18" s="13"/>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="15" t="s">
         <v>264</v>
       </c>
       <c r="D19" s="13"/>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="15" t="s">
         <v>87</v>
       </c>
       <c r="D20" s="13"/>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="17" t="s">
         <v>265</v>
       </c>
       <c r="D21" s="13"/>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="17" t="s">
         <v>266</v>
       </c>
       <c r="D22" s="13"/>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="17" t="s">
         <v>267</v>
       </c>
       <c r="D23" s="13"/>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="17" t="s">
         <v>268</v>
       </c>
       <c r="D24" s="13"/>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="17" t="s">
         <v>269</v>
       </c>
@@ -2643,763 +2645,771 @@
         <v>35</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="17" t="s">
+        <v>308</v>
+      </c>
+      <c r="D26" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27" s="17" t="s">
         <v>270</v>
       </c>
-      <c r="D26" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A27" s="16" t="s">
+      <c r="D27" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28" s="16" t="s">
         <v>271</v>
       </c>
-      <c r="D27" s="13"/>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A28" s="16" t="s">
+      <c r="D28" s="13"/>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29" s="16" t="s">
         <v>83</v>
       </c>
-      <c r="D28" s="13"/>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A29" s="16" t="s">
+      <c r="D29" s="13"/>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30" s="16" t="s">
         <v>272</v>
       </c>
-      <c r="D29" s="13"/>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A30" s="16" t="s">
+      <c r="D30" s="13"/>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A31" s="16" t="s">
         <v>90</v>
       </c>
-      <c r="D30" s="13"/>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A31" s="16" t="s">
+      <c r="D31" s="13"/>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A32" s="16" t="s">
         <v>273</v>
       </c>
-      <c r="D31" s="13"/>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A32" s="16" t="s">
+      <c r="D32" s="13"/>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A33" s="16" t="s">
         <v>274</v>
       </c>
-      <c r="D32" s="13"/>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A33" s="16" t="s">
+      <c r="D33" s="13"/>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A34" s="16" t="s">
         <v>275</v>
       </c>
-      <c r="D33" s="13"/>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A34" s="16" t="s">
+      <c r="D34" s="13"/>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A35" s="16" t="s">
         <v>276</v>
       </c>
-      <c r="D34" s="13"/>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A35" s="14" t="s">
+      <c r="D35" s="13"/>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A36" s="14" t="s">
         <v>97</v>
       </c>
-      <c r="D35" s="13"/>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A36" s="16" t="s">
+      <c r="D36" s="13"/>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A37" s="16" t="s">
         <v>277</v>
       </c>
-      <c r="D36" s="13"/>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A37" s="16" t="s">
+      <c r="D37" s="13"/>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A38" s="16" t="s">
         <v>278</v>
       </c>
-      <c r="D37" s="13"/>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A38" s="16" t="s">
+      <c r="D38" s="13"/>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A39" s="16" t="s">
         <v>279</v>
       </c>
-      <c r="D38" s="13"/>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A39" s="16" t="s">
+      <c r="D39" s="13"/>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A40" s="16" t="s">
         <v>280</v>
       </c>
-      <c r="D39" s="13"/>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A40" s="16" t="s">
+      <c r="D40" s="13"/>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A41" s="16" t="s">
         <v>212</v>
       </c>
-      <c r="D40" s="13"/>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A41" s="16" t="s">
+      <c r="D41" s="13"/>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A42" s="16" t="s">
         <v>281</v>
       </c>
-      <c r="D41" s="13"/>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A42" s="16" t="s">
+      <c r="D42" s="13"/>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A43" s="16" t="s">
         <v>282</v>
       </c>
-      <c r="D42" s="13"/>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A43" s="16" t="s">
+      <c r="D43" s="13"/>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A44" s="16" t="s">
         <v>283</v>
       </c>
-      <c r="D43" s="13"/>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A44" s="16" t="s">
+      <c r="D44" s="13"/>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A45" s="16" t="s">
         <v>284</v>
       </c>
-      <c r="D44" s="13"/>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A45" s="16" t="s">
+      <c r="D45" s="13"/>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A46" s="16" t="s">
         <v>84</v>
       </c>
-      <c r="D45" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A46" s="16" t="s">
+      <c r="D46" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A47" s="16" t="s">
         <v>85</v>
       </c>
-      <c r="D46" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A47" s="16" t="s">
+      <c r="D47" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A48" s="16" t="s">
         <v>86</v>
       </c>
-      <c r="D47" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A48" s="16" t="s">
+      <c r="D48" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A49" s="16" t="s">
         <v>88</v>
       </c>
-      <c r="D48" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A49" s="16" t="s">
+      <c r="D49" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A50" s="16" t="s">
         <v>89</v>
       </c>
-      <c r="D49" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A50" s="16" t="s">
+      <c r="D50" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A51" s="16" t="s">
         <v>91</v>
       </c>
-      <c r="D50" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A51" s="16" t="s">
+      <c r="D51" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A52" s="16" t="s">
         <v>94</v>
       </c>
-      <c r="D51" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A52" s="16" t="s">
+      <c r="D52" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A53" s="16" t="s">
         <v>96</v>
       </c>
-      <c r="D52" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A53" s="16" t="s">
+      <c r="D53" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A54" s="16" t="s">
         <v>95</v>
       </c>
-      <c r="D53" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A54" s="15" t="s">
+      <c r="D54" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A55" s="15" t="s">
         <v>92</v>
       </c>
-      <c r="D54" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A55" s="15" t="s">
+      <c r="D55" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A56" s="15" t="s">
         <v>93</v>
       </c>
-      <c r="D55" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A56" s="15" t="s">
+      <c r="D56" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A57" s="15" t="s">
         <v>36</v>
       </c>
-      <c r="D56" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A57" s="18" t="s">
+      <c r="D57" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A58" s="18" t="s">
         <v>40</v>
       </c>
-      <c r="D57" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A58" s="18" t="s">
+      <c r="D58" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A59" s="18" t="s">
         <v>39</v>
       </c>
-      <c r="D58" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A59" s="18" t="s">
+      <c r="D59" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A60" s="18" t="s">
         <v>38</v>
       </c>
-      <c r="D59" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A60" s="18" t="s">
+      <c r="D60" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A61" s="18" t="s">
         <v>34</v>
       </c>
-      <c r="D60" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A61" s="18" t="s">
+      <c r="D61" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A62" s="18" t="s">
         <v>37</v>
       </c>
-      <c r="D61" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A62" s="15" t="s">
+      <c r="D62" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A63" s="15" t="s">
         <v>98</v>
       </c>
-      <c r="D62" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A63" s="15" t="s">
+      <c r="D63" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A64" s="15" t="s">
         <v>99</v>
       </c>
-      <c r="D63" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A64" s="17" t="s">
+      <c r="D64" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A65" s="17" t="s">
         <v>285</v>
       </c>
-      <c r="D64" s="13"/>
-    </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A65" s="13" t="s">
+      <c r="D65" s="13"/>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A66" s="13" t="s">
         <v>286</v>
       </c>
-      <c r="D65" s="13"/>
-    </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A66" s="13" t="s">
+      <c r="D66" s="13"/>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A67" s="13" t="s">
         <v>287</v>
       </c>
-      <c r="D66" s="13"/>
-    </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A67" s="13" t="s">
+      <c r="D67" s="13"/>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A68" s="13" t="s">
         <v>237</v>
       </c>
-      <c r="D67" s="13"/>
-    </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A68" s="13" t="s">
+      <c r="D68" s="13"/>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A69" s="13" t="s">
         <v>288</v>
       </c>
-      <c r="D68" s="13"/>
-    </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A69" t="s">
+      <c r="D69" s="13"/>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
         <v>289</v>
       </c>
-      <c r="D69" s="13"/>
-    </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A70" t="s">
+      <c r="D70" s="13"/>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
         <v>221</v>
       </c>
-      <c r="D70" s="13"/>
-    </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A71" t="s">
+      <c r="D71" s="13"/>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
         <v>290</v>
       </c>
-      <c r="D71" s="13"/>
-    </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A72" t="s">
+      <c r="D72" s="13"/>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
         <v>291</v>
       </c>
-      <c r="D72" s="13"/>
-    </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A73" t="s">
+      <c r="D73" s="13"/>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
         <v>249</v>
       </c>
-      <c r="D73" s="13"/>
-    </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A74" t="s">
+      <c r="D74" s="13"/>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
         <v>214</v>
       </c>
-      <c r="D74" s="13"/>
-    </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A75" t="s">
+      <c r="D75" s="13"/>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
         <v>292</v>
       </c>
-      <c r="D75" s="13"/>
-    </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A76" t="s">
+      <c r="D76" s="13"/>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
         <v>293</v>
       </c>
-      <c r="D76" s="13"/>
-    </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A77" t="s">
+      <c r="D77" s="13"/>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
         <v>202</v>
       </c>
-      <c r="D77" s="13"/>
-    </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A78" t="s">
+      <c r="D78" s="13"/>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
         <v>294</v>
       </c>
-      <c r="D78" s="13"/>
-    </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A79" t="s">
+      <c r="D79" s="13"/>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
         <v>295</v>
       </c>
-      <c r="D79" s="13"/>
-    </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A80" t="s">
+      <c r="D80" s="13"/>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
         <v>296</v>
       </c>
-      <c r="D80" s="13"/>
-    </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A81" t="s">
+      <c r="D81" s="13"/>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
         <v>297</v>
       </c>
-      <c r="D81" s="13"/>
-    </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A82" t="s">
+      <c r="D82" s="13"/>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
         <v>298</v>
       </c>
-      <c r="D82" s="13"/>
-    </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A83" t="s">
+      <c r="D83" s="13"/>
+    </row>
+    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
         <v>299</v>
       </c>
-      <c r="D83" s="13"/>
-    </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A84" t="s">
+      <c r="D84" s="13"/>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
         <v>230</v>
       </c>
-      <c r="D84" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A85" t="s">
+      <c r="D85" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
         <v>246</v>
       </c>
-      <c r="D85" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A86" t="s">
+      <c r="D86" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
         <v>248</v>
       </c>
-      <c r="D86" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A87" t="s">
+      <c r="D87" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
         <v>217</v>
       </c>
-      <c r="D87" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A88" t="s">
+      <c r="D88" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
         <v>300</v>
       </c>
-      <c r="D88" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A89" t="s">
+      <c r="D89" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
         <v>208</v>
       </c>
-      <c r="D89" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A90" t="s">
+      <c r="D90" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
         <v>229</v>
       </c>
-      <c r="D90" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A91" t="s">
+      <c r="D91" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
         <v>211</v>
       </c>
-      <c r="D91" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A92" t="s">
+      <c r="D92" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
         <v>241</v>
       </c>
-      <c r="D92" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A93" t="s">
+      <c r="D93" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
         <v>226</v>
       </c>
-      <c r="D93" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A94" t="s">
+      <c r="D94" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
         <v>242</v>
       </c>
-      <c r="D94" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A95" t="s">
+      <c r="D95" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
         <v>243</v>
       </c>
-      <c r="D95" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A96" t="s">
+      <c r="D96" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
         <v>301</v>
       </c>
-      <c r="D96" s="13"/>
-    </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A97" t="s">
+      <c r="D97" s="13"/>
+    </row>
+    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
         <v>302</v>
       </c>
-      <c r="D97" s="13"/>
-    </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A98" t="s">
+      <c r="D98" s="13"/>
+    </row>
+    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
         <v>303</v>
       </c>
-      <c r="D98" s="13"/>
-    </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A99" t="s">
+      <c r="D99" s="13"/>
+    </row>
+    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
         <v>304</v>
       </c>
-      <c r="D99" s="13"/>
-    </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A100" t="s">
+      <c r="D100" s="13"/>
+    </row>
+    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
         <v>305</v>
       </c>
-      <c r="D100" s="13"/>
-    </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A101" s="19" t="s">
+      <c r="D101" s="13"/>
+    </row>
+    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A102" s="19" t="s">
         <v>247</v>
       </c>
-      <c r="D101" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A102" s="19" t="s">
+      <c r="D102" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A103" s="19" t="s">
         <v>235</v>
       </c>
-      <c r="D102" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A103" s="19" t="s">
+      <c r="D103" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A104" s="19" t="s">
         <v>220</v>
       </c>
-      <c r="D103" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A104" s="19" t="s">
+      <c r="D104" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A105" s="19" t="s">
         <v>233</v>
       </c>
-      <c r="D104" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A105" s="19" t="s">
+      <c r="D105" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A106" s="19" t="s">
         <v>213</v>
       </c>
-      <c r="D105" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="106" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A106" s="19" t="s">
+      <c r="D106" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A107" s="19" t="s">
         <v>205</v>
       </c>
-      <c r="D106" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A107" s="19" t="s">
+      <c r="D107" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A108" s="19" t="s">
         <v>224</v>
       </c>
-      <c r="D107" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A108" s="19" t="s">
+      <c r="D108" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A109" s="19" t="s">
         <v>239</v>
       </c>
-      <c r="D108" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A109" s="19" t="s">
+      <c r="D109" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A110" s="19" t="s">
         <v>216</v>
       </c>
-      <c r="D109" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A110" s="19" t="s">
+      <c r="D110" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A111" s="19" t="s">
         <v>201</v>
       </c>
-      <c r="D110" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A111" s="19" t="s">
+      <c r="D111" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A112" s="19" t="s">
         <v>238</v>
       </c>
-      <c r="D111" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="112" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A112" s="19" t="s">
+      <c r="D112" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="113" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A113" s="19" t="s">
         <v>231</v>
       </c>
-      <c r="D112" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="113" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A113" s="19" t="s">
+      <c r="D113" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="114" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A114" s="19" t="s">
         <v>209</v>
       </c>
-      <c r="D113" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="114" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A114" s="19" t="s">
+      <c r="D114" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="115" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A115" s="19" t="s">
         <v>215</v>
       </c>
-      <c r="D114" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="115" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A115" s="19" t="s">
+      <c r="D115" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="116" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A116" s="19" t="s">
         <v>232</v>
       </c>
-      <c r="D115" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="116" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A116" s="19" t="s">
+      <c r="D116" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="117" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A117" s="19" t="s">
         <v>244</v>
       </c>
-      <c r="D116" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="117" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A117" s="19" t="s">
+      <c r="D117" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="118" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A118" s="19" t="s">
         <v>223</v>
       </c>
-      <c r="D117" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="118" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A118" s="19" t="s">
+      <c r="D118" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="119" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A119" s="19" t="s">
         <v>218</v>
       </c>
-      <c r="D118" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="119" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A119" s="19" t="s">
+      <c r="D119" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="120" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A120" s="19" t="s">
         <v>236</v>
       </c>
-      <c r="D119" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="120" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A120" s="19" t="s">
+      <c r="D120" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="121" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A121" s="19" t="s">
         <v>225</v>
       </c>
-      <c r="D120" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="121" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A121" s="19" t="s">
+      <c r="D121" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="122" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A122" s="19" t="s">
         <v>234</v>
       </c>
-      <c r="D121" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="122" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A122" s="19" t="s">
+      <c r="D122" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="123" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A123" s="19" t="s">
         <v>222</v>
       </c>
-      <c r="D122" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="123" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A123" s="19" t="s">
+      <c r="D123" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="124" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A124" s="19" t="s">
         <v>219</v>
       </c>
-      <c r="D123" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="124" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A124" s="19" t="s">
+      <c r="D124" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="125" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A125" s="19" t="s">
         <v>240</v>
       </c>
-      <c r="D124" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="125" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A125" s="19" t="s">
+      <c r="D125" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="126" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A126" s="19" t="s">
         <v>210</v>
       </c>
-      <c r="D125" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="126" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A126" s="19" t="s">
+      <c r="D126" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="127" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A127" s="19" t="s">
         <v>207</v>
       </c>
-      <c r="D126" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="127" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A127" s="19" t="s">
+      <c r="D127" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="128" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A128" s="19" t="s">
         <v>227</v>
       </c>
-      <c r="D127" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="128" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A128" s="19" t="s">
+      <c r="D128" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="129" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A129" s="19" t="s">
         <v>203</v>
       </c>
-      <c r="D128" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="129" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A129" s="19" t="s">
+      <c r="D129" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="130" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A130" s="19" t="s">
         <v>206</v>
       </c>
-      <c r="D129" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="130" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A130" s="19" t="s">
+      <c r="D130" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="131" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A131" s="19" t="s">
         <v>245</v>
       </c>
-      <c r="D130" t="s">
+      <c r="D131" t="s">
         <v>35</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:A130" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
-  <conditionalFormatting sqref="A3:A130">
+  <autoFilter ref="A1:A131"/>
+  <conditionalFormatting sqref="A3:A131">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3408,11 +3418,11 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="9.26953125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3423,7 +3433,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>19</v>
       </c>
@@ -3431,7 +3441,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>21</v>
       </c>
@@ -3439,7 +3449,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>23</v>
       </c>

</xml_diff>

<commit_message>
enhance data mapping logic to handle new attributes and improve efficiency calculations
</commit_message>
<xml_diff>
--- a/config_data/mapping_v4.xlsx
+++ b/config_data/mapping_v4.xlsx
@@ -91,7 +91,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="419" uniqueCount="310">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="420" uniqueCount="311">
   <si>
     <t>TIMES</t>
   </si>
@@ -1021,6 +1021,9 @@
   </si>
   <si>
     <t>capacity_tra_min</t>
+  </si>
+  <si>
+    <t>*market_share_range</t>
   </si>
 </sst>
 </file>
@@ -2202,7 +2205,9 @@
       <c r="A57" s="9" t="s">
         <v>134</v>
       </c>
-      <c r="B57" s="9"/>
+      <c r="B57" s="9" t="s">
+        <v>310</v>
+      </c>
       <c r="C57" t="s">
         <v>190</v>
       </c>

</xml_diff>

<commit_message>
update emi_co2_neg_air attribute as OUTPUT in fill_emission_factors
</commit_message>
<xml_diff>
--- a/config_data/mapping_v4.xlsx
+++ b/config_data/mapping_v4.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20416"/>
+  <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Xchange\Studis\Apath\HiWi Project\config_data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Xchange\Studis\Apath\materials_DAdapter\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20378953-E476-477C-B1EA-F383DD9AB48D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="8145" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="8150" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SEDOS_parameters" sheetId="5" r:id="rId1"/>
@@ -17,7 +18,7 @@
     <sheet name="limits" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">commodity_set!$A$1:$A$131</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">commodity_set!$A$1:$A$130</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
@@ -29,12 +30,12 @@
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>Islam, Md Anik</author>
   </authors>
   <commentList>
-    <comment ref="B43" authorId="0" shapeId="0">
+    <comment ref="B43" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
       <text>
         <r>
           <rPr>
@@ -64,12 +65,12 @@
 </file>
 
 <file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>Gary Goldstein</author>
   </authors>
   <commentList>
-    <comment ref="D1" authorId="0" shapeId="0">
+    <comment ref="D1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000001000000}">
       <text>
         <r>
           <rPr>
@@ -91,7 +92,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="415" uniqueCount="309">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="417" uniqueCount="310">
   <si>
     <t>TIMES</t>
   </si>
@@ -1017,13 +1018,16 @@
     <t>ACTFLO~DEMO</t>
   </si>
   <si>
-    <t>emi_co2_neg_air_dacc</t>
+    <t>emi_co2_neg_imp</t>
+  </si>
+  <si>
+    <t>emi_co2_neg_air_bio</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1147,7 +1151,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1192,10 +1196,11 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Normal 10" xfId="1"/>
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 10" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
   </cellStyles>
   <dxfs count="1">
     <dxf>
@@ -1517,22 +1522,22 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:O120"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="37.7109375" customWidth="1"/>
-    <col min="2" max="2" width="25.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="31.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="37.7265625" customWidth="1"/>
+    <col min="2" max="2" width="25.7265625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="31.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.26953125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="18" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="22.28515625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.7265625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.7265625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="22.26953125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -1564,7 +1569,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>100</v>
       </c>
@@ -1575,7 +1580,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>5</v>
       </c>
@@ -1586,7 +1591,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>81</v>
       </c>
@@ -1600,7 +1605,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>101</v>
       </c>
@@ -1621,7 +1626,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A6" s="9" t="s">
         <v>46</v>
       </c>
@@ -1634,7 +1639,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>6</v>
       </c>
@@ -1645,7 +1650,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A8" s="9" t="s">
         <v>102</v>
       </c>
@@ -1654,7 +1659,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>74</v>
       </c>
@@ -1665,7 +1670,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>103</v>
       </c>
@@ -1679,7 +1684,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>104</v>
       </c>
@@ -1693,7 +1698,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>64</v>
       </c>
@@ -1704,7 +1709,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>105</v>
       </c>
@@ -1718,7 +1723,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>106</v>
       </c>
@@ -1732,7 +1737,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>56</v>
       </c>
@@ -1743,7 +1748,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
         <v>107</v>
       </c>
@@ -1757,7 +1762,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
         <v>108</v>
       </c>
@@ -1771,7 +1776,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
         <v>109</v>
       </c>
@@ -1782,7 +1787,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
         <v>75</v>
       </c>
@@ -1796,7 +1801,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
         <v>72</v>
       </c>
@@ -1810,7 +1815,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A21" s="2" t="s">
         <v>63</v>
       </c>
@@ -1824,7 +1829,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
         <v>4</v>
       </c>
@@ -1835,7 +1840,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A23" s="2" t="s">
         <v>110</v>
       </c>
@@ -1846,7 +1851,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A24" s="9" t="s">
         <v>111</v>
       </c>
@@ -1857,7 +1862,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
         <v>112</v>
       </c>
@@ -1869,7 +1874,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
         <v>76</v>
       </c>
@@ -1880,7 +1885,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A27" s="2" t="s">
         <v>66</v>
       </c>
@@ -1891,7 +1896,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
         <v>59</v>
       </c>
@@ -1902,7 +1907,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A29" s="2" t="s">
         <v>113</v>
       </c>
@@ -1913,7 +1918,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
         <v>78</v>
       </c>
@@ -1924,7 +1929,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A31" s="2" t="s">
         <v>68</v>
       </c>
@@ -1935,7 +1940,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A32" s="2" t="s">
         <v>60</v>
       </c>
@@ -1946,7 +1951,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A33" s="2" t="s">
         <v>114</v>
       </c>
@@ -1957,7 +1962,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A34" s="2" t="s">
         <v>70</v>
       </c>
@@ -1968,7 +1973,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A35" s="2" t="s">
         <v>115</v>
       </c>
@@ -1976,7 +1981,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A36" s="2" t="s">
         <v>61</v>
       </c>
@@ -1987,7 +1992,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A37" s="2" t="s">
         <v>116</v>
       </c>
@@ -1998,7 +2003,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A38" s="2" t="s">
         <v>117</v>
       </c>
@@ -2012,7 +2017,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A39" s="2" t="s">
         <v>118</v>
       </c>
@@ -2026,7 +2031,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A40" s="2" t="s">
         <v>119</v>
       </c>
@@ -2040,7 +2045,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A41" s="2" t="s">
         <v>120</v>
       </c>
@@ -2051,7 +2056,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A42" s="2" t="s">
         <v>121</v>
       </c>
@@ -2060,7 +2065,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A43" s="2" t="s">
         <v>122</v>
       </c>
@@ -2074,7 +2079,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A44" s="2" t="s">
         <v>123</v>
       </c>
@@ -2085,7 +2090,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A45" s="2" t="s">
         <v>124</v>
       </c>
@@ -2096,7 +2101,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A46" s="9" t="s">
         <v>125</v>
       </c>
@@ -2105,7 +2110,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A47" s="9" t="s">
         <v>126</v>
       </c>
@@ -2114,7 +2119,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A48" s="9" t="s">
         <v>127</v>
       </c>
@@ -2123,7 +2128,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A49" s="9" t="s">
         <v>128</v>
       </c>
@@ -2132,7 +2137,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A50" s="9" t="s">
         <v>129</v>
       </c>
@@ -2141,7 +2146,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A51" s="9" t="s">
         <v>130</v>
       </c>
@@ -2150,7 +2155,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A52" s="9" t="s">
         <v>131</v>
       </c>
@@ -2159,7 +2164,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A53" s="9" t="s">
         <v>132</v>
       </c>
@@ -2168,7 +2173,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A54" s="2" t="s">
         <v>133</v>
       </c>
@@ -2179,7 +2184,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A55" s="9" t="s">
         <v>134</v>
       </c>
@@ -2188,7 +2193,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A56" s="2" t="s">
         <v>135</v>
       </c>
@@ -2199,7 +2204,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A57" s="10" t="s">
         <v>136</v>
       </c>
@@ -2210,7 +2215,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A58" s="10" t="s">
         <v>137</v>
       </c>
@@ -2219,7 +2224,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A59" s="9" t="s">
         <v>138</v>
       </c>
@@ -2228,7 +2233,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A60" s="9" t="s">
         <v>139</v>
       </c>
@@ -2237,7 +2242,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A61" s="10" t="s">
         <v>140</v>
       </c>
@@ -2248,19 +2253,19 @@
         <v>196</v>
       </c>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A62" s="7" t="s">
         <v>141</v>
       </c>
       <c r="B62" s="6"/>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A63" s="7" t="s">
         <v>142</v>
       </c>
       <c r="B63" s="6"/>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A64" s="7" t="s">
         <v>143</v>
       </c>
@@ -2269,199 +2274,199 @@
         <v>197</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A65" s="7" t="s">
         <v>41</v>
       </c>
       <c r="B65" s="6"/>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A66" s="7" t="s">
         <v>144</v>
       </c>
       <c r="B66" s="6"/>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A67" s="7" t="s">
         <v>145</v>
       </c>
       <c r="B67" s="6"/>
     </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A68" s="7" t="s">
         <v>146</v>
       </c>
       <c r="B68" s="6"/>
     </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A69" s="7" t="s">
         <v>147</v>
       </c>
       <c r="B69" s="6"/>
     </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A70" s="7" t="s">
         <v>148</v>
       </c>
       <c r="B70" s="6"/>
     </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A71" s="7" t="s">
         <v>47</v>
       </c>
       <c r="B71" s="6"/>
     </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A72" s="7" t="s">
         <v>149</v>
       </c>
       <c r="B72" s="6"/>
     </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A73" s="7" t="s">
         <v>48</v>
       </c>
       <c r="B73" s="6"/>
     </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B74" s="6"/>
     </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B75" s="6"/>
     </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B76" s="6"/>
     </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B77" s="6"/>
     </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B78" s="6"/>
     </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B79" s="6"/>
     </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B80" s="6"/>
     </row>
-    <row r="81" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="81" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B81" s="6"/>
     </row>
-    <row r="82" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="82" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B82" s="6"/>
     </row>
-    <row r="83" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="83" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B83" s="6"/>
     </row>
-    <row r="84" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="84" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B84" s="6"/>
     </row>
-    <row r="85" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="85" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B85" s="6"/>
     </row>
-    <row r="86" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="86" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B86" s="6"/>
     </row>
-    <row r="87" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="87" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B87" s="6"/>
     </row>
-    <row r="88" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="88" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B88" s="6"/>
     </row>
-    <row r="89" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="89" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B89" s="6"/>
     </row>
-    <row r="90" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="90" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B90" s="6"/>
     </row>
-    <row r="91" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="91" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B91" s="6"/>
     </row>
-    <row r="92" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="92" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B92" s="6"/>
     </row>
-    <row r="93" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="93" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B93" s="6"/>
     </row>
-    <row r="94" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="94" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B94" s="6"/>
     </row>
-    <row r="95" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="95" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B95" s="6"/>
     </row>
-    <row r="96" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="96" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B96" s="6"/>
     </row>
-    <row r="97" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="97" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B97" s="6"/>
     </row>
-    <row r="98" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="98" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B98" s="6"/>
     </row>
-    <row r="99" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="99" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B99" s="6"/>
     </row>
-    <row r="100" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="100" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B100" s="6"/>
     </row>
-    <row r="101" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="101" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B101" s="6"/>
     </row>
-    <row r="102" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="102" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B102" s="6"/>
     </row>
-    <row r="103" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="103" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B103" s="6"/>
     </row>
-    <row r="104" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="104" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B104" s="6"/>
     </row>
-    <row r="105" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="105" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B105" s="6"/>
     </row>
-    <row r="106" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="106" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B106" s="6"/>
     </row>
-    <row r="107" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="107" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B107" s="6"/>
     </row>
-    <row r="108" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="108" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B108" s="6"/>
     </row>
-    <row r="109" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="109" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B109" s="6"/>
     </row>
-    <row r="110" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="110" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B110" s="6"/>
     </row>
-    <row r="111" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="111" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B111" s="6"/>
     </row>
-    <row r="112" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="112" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B112" s="6"/>
     </row>
-    <row r="113" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="113" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B113" s="6"/>
     </row>
-    <row r="114" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="114" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B114" s="6"/>
     </row>
-    <row r="115" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="115" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B115" s="6"/>
     </row>
-    <row r="116" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="116" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B116" s="6"/>
     </row>
-    <row r="117" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="117" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B117" s="6"/>
     </row>
-    <row r="118" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="118" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B118" s="6"/>
     </row>
-    <row r="119" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="119" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B119" s="6"/>
     </row>
-    <row r="120" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="120" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B120" s="6"/>
     </row>
   </sheetData>
@@ -2472,17 +2477,17 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D131"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:D132"/>
+  <sheetFormatPr defaultColWidth="9.26953125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="32.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.5703125" customWidth="1"/>
-    <col min="3" max="3" width="15.42578125" customWidth="1"/>
-    <col min="4" max="4" width="23.7109375" customWidth="1"/>
+    <col min="1" max="1" width="32.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.54296875" customWidth="1"/>
+    <col min="3" max="3" width="15.453125" customWidth="1"/>
+    <col min="4" max="4" width="23.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>27</v>
       </c>
@@ -2496,7 +2501,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" s="5" t="s">
         <v>31</v>
       </c>
@@ -2510,134 +2515,134 @@
         <v>33</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" s="14" t="s">
         <v>250</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="15" t="s">
         <v>251</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" s="14" t="s">
         <v>252</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" s="14" t="s">
         <v>253</v>
       </c>
       <c r="D6" s="13"/>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="15" t="s">
         <v>254</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" s="14" t="s">
         <v>255</v>
       </c>
       <c r="D8" s="13"/>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" s="14" t="s">
         <v>256</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" s="14" t="s">
         <v>257</v>
       </c>
       <c r="D10" s="13"/>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" s="14" t="s">
         <v>258</v>
       </c>
       <c r="D11" s="13"/>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" s="16" t="s">
         <v>259</v>
       </c>
       <c r="D12" s="13"/>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" s="16" t="s">
         <v>260</v>
       </c>
       <c r="D13" s="13"/>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" s="17" t="s">
         <v>204</v>
       </c>
       <c r="D14" s="13"/>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" s="18" t="s">
         <v>261</v>
       </c>
       <c r="D15" s="13"/>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" s="16" t="s">
         <v>262</v>
       </c>
       <c r="D16" s="13"/>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" s="16" t="s">
         <v>228</v>
       </c>
       <c r="D17" s="13"/>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" s="16" t="s">
         <v>263</v>
       </c>
       <c r="D18" s="13"/>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" s="15" t="s">
         <v>264</v>
       </c>
       <c r="D19" s="13"/>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" s="15" t="s">
         <v>87</v>
       </c>
       <c r="D20" s="13"/>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21" s="17" t="s">
         <v>265</v>
       </c>
       <c r="D21" s="13"/>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" s="17" t="s">
         <v>266</v>
       </c>
       <c r="D22" s="13"/>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" s="17" t="s">
         <v>267</v>
       </c>
       <c r="D23" s="13"/>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A24" s="17" t="s">
         <v>268</v>
       </c>
       <c r="D24" s="13"/>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A25" s="17" t="s">
         <v>269</v>
       </c>
@@ -2645,771 +2650,779 @@
         <v>35</v>
       </c>
     </row>
-    <row r="26" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A26" s="17" t="s">
+        <v>270</v>
+      </c>
+      <c r="D26" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A27" s="16" t="s">
+        <v>271</v>
+      </c>
+      <c r="D27" s="13"/>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A28" s="16" t="s">
+        <v>83</v>
+      </c>
+      <c r="D28" s="13"/>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A29" s="16" t="s">
+        <v>272</v>
+      </c>
+      <c r="D29" s="13"/>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A30" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="D30" s="13"/>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A31" s="16" t="s">
+        <v>273</v>
+      </c>
+      <c r="D31" s="13"/>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A32" s="16" t="s">
+        <v>274</v>
+      </c>
+      <c r="D32" s="13"/>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A33" s="16" t="s">
+        <v>275</v>
+      </c>
+      <c r="D33" s="13"/>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A34" s="16" t="s">
+        <v>276</v>
+      </c>
+      <c r="D34" s="13"/>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A35" s="14" t="s">
+        <v>97</v>
+      </c>
+      <c r="D35" s="13"/>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A36" s="16" t="s">
+        <v>277</v>
+      </c>
+      <c r="D36" s="13"/>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A37" s="16" t="s">
+        <v>278</v>
+      </c>
+      <c r="D37" s="13"/>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A38" s="16" t="s">
+        <v>279</v>
+      </c>
+      <c r="D38" s="13"/>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A39" s="16" t="s">
+        <v>280</v>
+      </c>
+      <c r="D39" s="13"/>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A40" s="16" t="s">
+        <v>212</v>
+      </c>
+      <c r="D40" s="13"/>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A41" s="16" t="s">
+        <v>281</v>
+      </c>
+      <c r="D41" s="13"/>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A42" s="16" t="s">
+        <v>282</v>
+      </c>
+      <c r="D42" s="13"/>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A43" s="16" t="s">
+        <v>283</v>
+      </c>
+      <c r="D43" s="13"/>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A44" s="16" t="s">
+        <v>284</v>
+      </c>
+      <c r="D44" s="13"/>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A45" s="16" t="s">
+        <v>84</v>
+      </c>
+      <c r="D45" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A46" s="16" t="s">
+        <v>85</v>
+      </c>
+      <c r="D46" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A47" s="16" t="s">
+        <v>86</v>
+      </c>
+      <c r="D47" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A48" s="16" t="s">
+        <v>88</v>
+      </c>
+      <c r="D48" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A49" s="16" t="s">
+        <v>89</v>
+      </c>
+      <c r="D49" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A50" s="16" t="s">
+        <v>91</v>
+      </c>
+      <c r="D50" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A51" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="D51" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A52" s="16" t="s">
+        <v>96</v>
+      </c>
+      <c r="D52" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A53" s="16" t="s">
+        <v>95</v>
+      </c>
+      <c r="D53" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A54" s="15" t="s">
+        <v>92</v>
+      </c>
+      <c r="D54" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A55" s="15" t="s">
+        <v>93</v>
+      </c>
+      <c r="D55" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A56" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="D56" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A57" s="18" t="s">
+        <v>40</v>
+      </c>
+      <c r="D57" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A58" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="D58" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A59" s="18" t="s">
+        <v>38</v>
+      </c>
+      <c r="D59" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A60" s="18" t="s">
+        <v>34</v>
+      </c>
+      <c r="D60" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A61" s="18" t="s">
+        <v>37</v>
+      </c>
+      <c r="D61" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A62" s="15" t="s">
+        <v>98</v>
+      </c>
+      <c r="D62" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A63" s="15" t="s">
+        <v>99</v>
+      </c>
+      <c r="D63" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A64" s="17" t="s">
+        <v>285</v>
+      </c>
+      <c r="D64" s="13"/>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A65" s="13" t="s">
+        <v>286</v>
+      </c>
+      <c r="D65" s="13"/>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A66" s="13" t="s">
+        <v>287</v>
+      </c>
+      <c r="D66" s="13"/>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A67" s="13" t="s">
+        <v>237</v>
+      </c>
+      <c r="D67" s="13"/>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A68" s="13" t="s">
+        <v>288</v>
+      </c>
+      <c r="D68" s="13"/>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A69" t="s">
+        <v>289</v>
+      </c>
+      <c r="D69" s="13"/>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A70" t="s">
+        <v>221</v>
+      </c>
+      <c r="D70" s="13"/>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A71" t="s">
+        <v>290</v>
+      </c>
+      <c r="D71" s="13"/>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A72" t="s">
+        <v>291</v>
+      </c>
+      <c r="D72" s="13"/>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A73" t="s">
+        <v>249</v>
+      </c>
+      <c r="D73" s="13"/>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A74" t="s">
+        <v>214</v>
+      </c>
+      <c r="D74" s="13"/>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A75" t="s">
+        <v>292</v>
+      </c>
+      <c r="D75" s="13"/>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A76" t="s">
+        <v>293</v>
+      </c>
+      <c r="D76" s="13"/>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A77" t="s">
+        <v>202</v>
+      </c>
+      <c r="D77" s="13"/>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A78" t="s">
+        <v>294</v>
+      </c>
+      <c r="D78" s="13"/>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A79" t="s">
+        <v>295</v>
+      </c>
+      <c r="D79" s="13"/>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A80" t="s">
+        <v>296</v>
+      </c>
+      <c r="D80" s="13"/>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A81" t="s">
+        <v>297</v>
+      </c>
+      <c r="D81" s="13"/>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A82" t="s">
+        <v>298</v>
+      </c>
+      <c r="D82" s="13"/>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A83" t="s">
+        <v>299</v>
+      </c>
+      <c r="D83" s="13"/>
+    </row>
+    <row r="84" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A84" t="s">
+        <v>230</v>
+      </c>
+      <c r="D84" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A85" t="s">
+        <v>246</v>
+      </c>
+      <c r="D85" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A86" t="s">
+        <v>248</v>
+      </c>
+      <c r="D86" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A87" t="s">
+        <v>217</v>
+      </c>
+      <c r="D87" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A88" t="s">
+        <v>300</v>
+      </c>
+      <c r="D88" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A89" t="s">
+        <v>208</v>
+      </c>
+      <c r="D89" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A90" t="s">
+        <v>229</v>
+      </c>
+      <c r="D90" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A91" t="s">
+        <v>211</v>
+      </c>
+      <c r="D91" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A92" t="s">
+        <v>241</v>
+      </c>
+      <c r="D92" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A93" t="s">
+        <v>226</v>
+      </c>
+      <c r="D93" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A94" t="s">
+        <v>242</v>
+      </c>
+      <c r="D94" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A95" t="s">
+        <v>243</v>
+      </c>
+      <c r="D95" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="96" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A96" t="s">
+        <v>301</v>
+      </c>
+      <c r="D96" s="13"/>
+    </row>
+    <row r="97" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A97" t="s">
+        <v>302</v>
+      </c>
+      <c r="D97" s="13"/>
+    </row>
+    <row r="98" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A98" t="s">
+        <v>303</v>
+      </c>
+      <c r="D98" s="13"/>
+    </row>
+    <row r="99" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A99" t="s">
+        <v>304</v>
+      </c>
+      <c r="D99" s="13"/>
+    </row>
+    <row r="100" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A100" t="s">
+        <v>305</v>
+      </c>
+      <c r="D100" s="13"/>
+    </row>
+    <row r="101" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A101" s="19" t="s">
+        <v>247</v>
+      </c>
+      <c r="D101" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="102" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A102" s="19" t="s">
+        <v>235</v>
+      </c>
+      <c r="D102" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="103" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A103" s="19" t="s">
+        <v>220</v>
+      </c>
+      <c r="D103" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="104" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A104" s="19" t="s">
+        <v>233</v>
+      </c>
+      <c r="D104" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="105" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A105" s="19" t="s">
+        <v>213</v>
+      </c>
+      <c r="D105" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="106" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A106" s="19" t="s">
+        <v>205</v>
+      </c>
+      <c r="D106" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="107" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A107" s="19" t="s">
+        <v>224</v>
+      </c>
+      <c r="D107" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="108" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A108" s="19" t="s">
+        <v>239</v>
+      </c>
+      <c r="D108" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="109" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A109" s="19" t="s">
+        <v>216</v>
+      </c>
+      <c r="D109" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="110" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A110" s="19" t="s">
+        <v>201</v>
+      </c>
+      <c r="D110" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="111" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A111" s="19" t="s">
+        <v>238</v>
+      </c>
+      <c r="D111" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="112" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A112" s="19" t="s">
+        <v>231</v>
+      </c>
+      <c r="D112" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="113" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A113" s="19" t="s">
+        <v>209</v>
+      </c>
+      <c r="D113" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="114" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A114" s="19" t="s">
+        <v>215</v>
+      </c>
+      <c r="D114" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="115" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A115" s="19" t="s">
+        <v>232</v>
+      </c>
+      <c r="D115" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="116" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A116" s="19" t="s">
+        <v>244</v>
+      </c>
+      <c r="D116" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="117" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A117" s="19" t="s">
+        <v>223</v>
+      </c>
+      <c r="D117" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="118" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A118" s="19" t="s">
+        <v>218</v>
+      </c>
+      <c r="D118" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="119" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A119" s="19" t="s">
+        <v>236</v>
+      </c>
+      <c r="D119" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="120" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A120" s="19" t="s">
+        <v>225</v>
+      </c>
+      <c r="D120" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="121" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A121" s="19" t="s">
+        <v>234</v>
+      </c>
+      <c r="D121" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="122" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A122" s="19" t="s">
+        <v>222</v>
+      </c>
+      <c r="D122" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="123" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A123" s="19" t="s">
+        <v>219</v>
+      </c>
+      <c r="D123" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="124" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A124" s="19" t="s">
+        <v>240</v>
+      </c>
+      <c r="D124" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="125" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A125" s="19" t="s">
+        <v>210</v>
+      </c>
+      <c r="D125" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="126" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A126" s="19" t="s">
+        <v>207</v>
+      </c>
+      <c r="D126" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="127" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A127" s="19" t="s">
+        <v>227</v>
+      </c>
+      <c r="D127" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="128" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A128" s="19" t="s">
+        <v>203</v>
+      </c>
+      <c r="D128" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="129" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A129" s="19" t="s">
+        <v>206</v>
+      </c>
+      <c r="D129" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="130" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A130" s="19" t="s">
+        <v>245</v>
+      </c>
+      <c r="D130" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="131" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A131" t="s">
         <v>308</v>
       </c>
-      <c r="D26" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" s="17" t="s">
-        <v>270</v>
-      </c>
-      <c r="D27" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" s="16" t="s">
-        <v>271</v>
-      </c>
-      <c r="D28" s="13"/>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29" s="16" t="s">
-        <v>83</v>
-      </c>
-      <c r="D29" s="13"/>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A30" s="16" t="s">
-        <v>272</v>
-      </c>
-      <c r="D30" s="13"/>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A31" s="16" t="s">
-        <v>90</v>
-      </c>
-      <c r="D31" s="13"/>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A32" s="16" t="s">
-        <v>273</v>
-      </c>
-      <c r="D32" s="13"/>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33" s="16" t="s">
-        <v>274</v>
-      </c>
-      <c r="D33" s="13"/>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A34" s="16" t="s">
-        <v>275</v>
-      </c>
-      <c r="D34" s="13"/>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35" s="16" t="s">
-        <v>276</v>
-      </c>
-      <c r="D35" s="13"/>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" s="14" t="s">
-        <v>97</v>
-      </c>
-      <c r="D36" s="13"/>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37" s="16" t="s">
-        <v>277</v>
-      </c>
-      <c r="D37" s="13"/>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A38" s="16" t="s">
-        <v>278</v>
-      </c>
-      <c r="D38" s="13"/>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39" s="16" t="s">
-        <v>279</v>
-      </c>
-      <c r="D39" s="13"/>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" s="16" t="s">
-        <v>280</v>
-      </c>
-      <c r="D40" s="13"/>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41" s="16" t="s">
-        <v>212</v>
-      </c>
-      <c r="D41" s="13"/>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42" s="16" t="s">
-        <v>281</v>
-      </c>
-      <c r="D42" s="13"/>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A43" s="16" t="s">
-        <v>282</v>
-      </c>
-      <c r="D43" s="13"/>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A44" s="16" t="s">
-        <v>283</v>
-      </c>
-      <c r="D44" s="13"/>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A45" s="16" t="s">
-        <v>284</v>
-      </c>
-      <c r="D45" s="13"/>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46" s="16" t="s">
-        <v>84</v>
-      </c>
-      <c r="D46" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A47" s="16" t="s">
-        <v>85</v>
-      </c>
-      <c r="D47" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A48" s="16" t="s">
-        <v>86</v>
-      </c>
-      <c r="D48" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A49" s="16" t="s">
-        <v>88</v>
-      </c>
-      <c r="D49" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A50" s="16" t="s">
-        <v>89</v>
-      </c>
-      <c r="D50" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A51" s="16" t="s">
-        <v>91</v>
-      </c>
-      <c r="D51" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A52" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="D52" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A53" s="16" t="s">
-        <v>96</v>
-      </c>
-      <c r="D53" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A54" s="16" t="s">
-        <v>95</v>
-      </c>
-      <c r="D54" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A55" s="15" t="s">
-        <v>92</v>
-      </c>
-      <c r="D55" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A56" s="15" t="s">
-        <v>93</v>
-      </c>
-      <c r="D56" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A57" s="15" t="s">
-        <v>36</v>
-      </c>
-      <c r="D57" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A58" s="18" t="s">
-        <v>40</v>
-      </c>
-      <c r="D58" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A59" s="18" t="s">
-        <v>39</v>
-      </c>
-      <c r="D59" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A60" s="18" t="s">
-        <v>38</v>
-      </c>
-      <c r="D60" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A61" s="18" t="s">
-        <v>34</v>
-      </c>
-      <c r="D61" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A62" s="18" t="s">
-        <v>37</v>
-      </c>
-      <c r="D62" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A63" s="15" t="s">
-        <v>98</v>
-      </c>
-      <c r="D63" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A64" s="15" t="s">
-        <v>99</v>
-      </c>
-      <c r="D64" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A65" s="17" t="s">
-        <v>285</v>
-      </c>
-      <c r="D65" s="13"/>
-    </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A66" s="13" t="s">
-        <v>286</v>
-      </c>
-      <c r="D66" s="13"/>
-    </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A67" s="13" t="s">
-        <v>287</v>
-      </c>
-      <c r="D67" s="13"/>
-    </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A68" s="13" t="s">
-        <v>237</v>
-      </c>
-      <c r="D68" s="13"/>
-    </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A69" s="13" t="s">
-        <v>288</v>
-      </c>
-      <c r="D69" s="13"/>
-    </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A70" t="s">
-        <v>289</v>
-      </c>
-      <c r="D70" s="13"/>
-    </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A71" t="s">
-        <v>221</v>
-      </c>
-      <c r="D71" s="13"/>
-    </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A72" t="s">
-        <v>290</v>
-      </c>
-      <c r="D72" s="13"/>
-    </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A73" t="s">
-        <v>291</v>
-      </c>
-      <c r="D73" s="13"/>
-    </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A74" t="s">
-        <v>249</v>
-      </c>
-      <c r="D74" s="13"/>
-    </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A75" t="s">
-        <v>214</v>
-      </c>
-      <c r="D75" s="13"/>
-    </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A76" t="s">
-        <v>292</v>
-      </c>
-      <c r="D76" s="13"/>
-    </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A77" t="s">
-        <v>293</v>
-      </c>
-      <c r="D77" s="13"/>
-    </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A78" t="s">
-        <v>202</v>
-      </c>
-      <c r="D78" s="13"/>
-    </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A79" t="s">
-        <v>294</v>
-      </c>
-      <c r="D79" s="13"/>
-    </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A80" t="s">
-        <v>295</v>
-      </c>
-      <c r="D80" s="13"/>
-    </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A81" t="s">
-        <v>296</v>
-      </c>
-      <c r="D81" s="13"/>
-    </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A82" t="s">
-        <v>297</v>
-      </c>
-      <c r="D82" s="13"/>
-    </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A83" t="s">
-        <v>298</v>
-      </c>
-      <c r="D83" s="13"/>
-    </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A84" t="s">
-        <v>299</v>
-      </c>
-      <c r="D84" s="13"/>
-    </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A85" t="s">
-        <v>230</v>
-      </c>
-      <c r="D85" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A86" t="s">
-        <v>246</v>
-      </c>
-      <c r="D86" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A87" t="s">
-        <v>248</v>
-      </c>
-      <c r="D87" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A88" t="s">
-        <v>217</v>
-      </c>
-      <c r="D88" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A89" t="s">
-        <v>300</v>
-      </c>
-      <c r="D89" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A90" t="s">
-        <v>208</v>
-      </c>
-      <c r="D90" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A91" t="s">
-        <v>229</v>
-      </c>
-      <c r="D91" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A92" t="s">
-        <v>211</v>
-      </c>
-      <c r="D92" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A93" t="s">
-        <v>241</v>
-      </c>
-      <c r="D93" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A94" t="s">
-        <v>226</v>
-      </c>
-      <c r="D94" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A95" t="s">
-        <v>242</v>
-      </c>
-      <c r="D95" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A96" t="s">
-        <v>243</v>
-      </c>
-      <c r="D96" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A97" t="s">
-        <v>301</v>
-      </c>
-      <c r="D97" s="13"/>
-    </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A98" t="s">
-        <v>302</v>
-      </c>
-      <c r="D98" s="13"/>
-    </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A99" t="s">
-        <v>303</v>
-      </c>
-      <c r="D99" s="13"/>
-    </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A100" t="s">
-        <v>304</v>
-      </c>
-      <c r="D100" s="13"/>
-    </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A101" t="s">
-        <v>305</v>
-      </c>
-      <c r="D101" s="13"/>
-    </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A102" s="19" t="s">
-        <v>247</v>
-      </c>
-      <c r="D102" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A103" s="19" t="s">
-        <v>235</v>
-      </c>
-      <c r="D103" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A104" s="19" t="s">
-        <v>220</v>
-      </c>
-      <c r="D104" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A105" s="19" t="s">
-        <v>233</v>
-      </c>
-      <c r="D105" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A106" s="19" t="s">
-        <v>213</v>
-      </c>
-      <c r="D106" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A107" s="19" t="s">
-        <v>205</v>
-      </c>
-      <c r="D107" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A108" s="19" t="s">
-        <v>224</v>
-      </c>
-      <c r="D108" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A109" s="19" t="s">
-        <v>239</v>
-      </c>
-      <c r="D109" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A110" s="19" t="s">
-        <v>216</v>
-      </c>
-      <c r="D110" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A111" s="19" t="s">
-        <v>201</v>
-      </c>
-      <c r="D111" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A112" s="19" t="s">
-        <v>238</v>
-      </c>
-      <c r="D112" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="113" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A113" s="19" t="s">
-        <v>231</v>
-      </c>
-      <c r="D113" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="114" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A114" s="19" t="s">
-        <v>209</v>
-      </c>
-      <c r="D114" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="115" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A115" s="19" t="s">
-        <v>215</v>
-      </c>
-      <c r="D115" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="116" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A116" s="19" t="s">
-        <v>232</v>
-      </c>
-      <c r="D116" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="117" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A117" s="19" t="s">
-        <v>244</v>
-      </c>
-      <c r="D117" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="118" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A118" s="19" t="s">
-        <v>223</v>
-      </c>
-      <c r="D118" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="119" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A119" s="19" t="s">
-        <v>218</v>
-      </c>
-      <c r="D119" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="120" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A120" s="19" t="s">
-        <v>236</v>
-      </c>
-      <c r="D120" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="121" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A121" s="19" t="s">
-        <v>225</v>
-      </c>
-      <c r="D121" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="122" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A122" s="19" t="s">
-        <v>234</v>
-      </c>
-      <c r="D122" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="123" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A123" s="19" t="s">
-        <v>222</v>
-      </c>
-      <c r="D123" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="124" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A124" s="19" t="s">
-        <v>219</v>
-      </c>
-      <c r="D124" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="125" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A125" s="19" t="s">
-        <v>240</v>
-      </c>
-      <c r="D125" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="126" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A126" s="19" t="s">
-        <v>210</v>
-      </c>
-      <c r="D126" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="127" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A127" s="19" t="s">
-        <v>207</v>
-      </c>
-      <c r="D127" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="128" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A128" s="19" t="s">
-        <v>227</v>
-      </c>
-      <c r="D128" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="129" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A129" s="19" t="s">
-        <v>203</v>
-      </c>
-      <c r="D129" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="130" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A130" s="19" t="s">
-        <v>206</v>
-      </c>
-      <c r="D130" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="131" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A131" s="19" t="s">
-        <v>245</v>
-      </c>
       <c r="D131" t="s">
         <v>35</v>
       </c>
     </row>
+    <row r="132" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A132" s="20" t="s">
+        <v>309</v>
+      </c>
+      <c r="D132" s="20" t="s">
+        <v>35</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:A131"/>
-  <conditionalFormatting sqref="A3:A25 A27:A131">
+  <autoFilter ref="A1:A130" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
+  <conditionalFormatting sqref="A3:A130">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3418,11 +3431,11 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.26953125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3433,7 +3446,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>19</v>
       </c>
@@ -3441,7 +3454,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>21</v>
       </c>
@@ -3449,7 +3462,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>23</v>
       </c>

</xml_diff>

<commit_message>
update emi_co2_neg_imp as OUTPUT topology
</commit_message>
<xml_diff>
--- a/config_data/mapping_v4.xlsx
+++ b/config_data/mapping_v4.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Xchange\Studis\Apath\materials_DAdapter\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\00_ESA\641_SEDOS BMWi\04-Arbeitspakete\AP9-Modellierung\data_adapter_TIMES\data_adapter_times_power\data_adapter_times\config_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20378953-E476-477C-B1EA-F383DD9AB48D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{264CA57A-3BC9-4867-9C7D-DC7F43D699EA}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="8150" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="8150" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SEDOS_parameters" sheetId="5" r:id="rId1"/>
@@ -92,7 +92,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="417" uniqueCount="310">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="419" uniqueCount="311">
   <si>
     <t>TIMES</t>
   </si>
@@ -115,913 +115,916 @@
     <t>demand_annual</t>
   </si>
   <si>
+    <t>ACT_COST</t>
+  </si>
+  <si>
+    <t>NCAP_BND</t>
+  </si>
+  <si>
+    <t>PRC_RESID</t>
+  </si>
+  <si>
+    <t>NCAP_FOM</t>
+  </si>
+  <si>
+    <t>NCAP_TLIFE</t>
+  </si>
+  <si>
+    <t>Absolute upper bound on level of investment in new weight capacity for a period.</t>
+  </si>
+  <si>
+    <t>Investment costs for new capacity per unit weight.</t>
+  </si>
+  <si>
+    <t>Operation independent costs for capacity per unit weight.</t>
+  </si>
+  <si>
+    <t>Technical lifetime of a process.</t>
+  </si>
+  <si>
+    <t>Projected annual demand for a commodity.</t>
+  </si>
+  <si>
+    <t>Comment</t>
+  </si>
+  <si>
+    <t>UP</t>
+  </si>
+  <si>
+    <t>max</t>
+  </si>
+  <si>
+    <t>LO</t>
+  </si>
+  <si>
+    <t>min</t>
+  </si>
+  <si>
+    <t>FX</t>
+  </si>
+  <si>
+    <t>fix</t>
+  </si>
+  <si>
+    <t>FLO_SHAR</t>
+  </si>
+  <si>
+    <t>COM_PROJ</t>
+  </si>
+  <si>
+    <t>CommName</t>
+  </si>
+  <si>
+    <t>CommDesc</t>
+  </si>
+  <si>
+    <t>Unit</t>
+  </si>
+  <si>
+    <t>Csets</t>
+  </si>
+  <si>
+    <t>Commodity Name</t>
+  </si>
+  <si>
+    <t>Commodity Description</t>
+  </si>
+  <si>
+    <t>*Commodity Set Membership</t>
+  </si>
+  <si>
+    <t>iip_steel_sinter</t>
+  </si>
+  <si>
+    <t>MAT</t>
+  </si>
+  <si>
+    <t>iip_steel_crudesteel</t>
+  </si>
+  <si>
+    <t>iip_steel_sponge_iron</t>
+  </si>
+  <si>
+    <t>iip_steel_scrap</t>
+  </si>
+  <si>
+    <t>iip_steel_raw_iron</t>
+  </si>
+  <si>
+    <t>iip_steel_iron_pellets</t>
+  </si>
+  <si>
+    <t>type</t>
+  </si>
+  <si>
+    <t>SEDOS_unit</t>
+  </si>
+  <si>
+    <t>isAbout</t>
+  </si>
+  <si>
+    <t>valueReference</t>
+  </si>
+  <si>
+    <t>Constraints</t>
+  </si>
+  <si>
+    <t>demand_timeseries</t>
+  </si>
+  <si>
+    <t>timeindex_start</t>
+  </si>
+  <si>
+    <t>timeindex_resolution</t>
+  </si>
+  <si>
+    <t>NCAP_AF</t>
+  </si>
+  <si>
+    <t>Constant output ratio in relation to installed capacity. (= h/a)</t>
+  </si>
+  <si>
+    <t>FLO_EFF</t>
+  </si>
+  <si>
+    <t>Commodity-specific conversion factor (multiplication of input and output factors yields the efficiency of the process).</t>
+  </si>
+  <si>
+    <t>Minimum share of flow commodity c based upon the sum of individual flows defined by the commodity group cg belonging to process p.</t>
+  </si>
+  <si>
+    <t>Maximum share of flow commodity c based upon the sum of individual flows defined by the commodity group cg belonging to process p.</t>
+  </si>
+  <si>
+    <t>Fixed share of flow commodity c based upon the sum of individual flows defined by the commodity group cg belonging to process p.</t>
+  </si>
+  <si>
+    <t>capacity_w_inst_0</t>
+  </si>
+  <si>
+    <t>Existing weight capacity of a process.</t>
+  </si>
+  <si>
+    <t>NCAP_COST</t>
+  </si>
+  <si>
+    <t>cost_inv_w</t>
+  </si>
+  <si>
+    <t>cost_fix_w</t>
+  </si>
+  <si>
+    <t>cost_var_w</t>
+  </si>
+  <si>
+    <t>Variable costs per throughput weight unit output. (excluding fuel costs).</t>
+  </si>
+  <si>
+    <t>capacity_w_abs_new_max</t>
+  </si>
+  <si>
+    <t>capacity_e_inst_0</t>
+  </si>
+  <si>
+    <t>Existing storage energy capacity.</t>
+  </si>
+  <si>
+    <t>cost_inv_e</t>
+  </si>
+  <si>
+    <t>Investment costs for new storage energy capacity.</t>
+  </si>
+  <si>
+    <t>cost_fix_e</t>
+  </si>
+  <si>
+    <t>Operation independent costs for existing and new storage energy capacity.</t>
+  </si>
+  <si>
+    <t>cost_var_e</t>
+  </si>
+  <si>
+    <t>Variable costs per throughput energy unit output. (excluding fuel costs).</t>
+  </si>
+  <si>
+    <t>capacity_e_abs_new_max</t>
+  </si>
+  <si>
+    <t>Absolute upper bound on level of investment in new storage energy capacity for a period.</t>
+  </si>
+  <si>
+    <t>capacity_p_inst_0</t>
+  </si>
+  <si>
+    <t>capacity_p_abs_new_max</t>
+  </si>
+  <si>
+    <t>cost_inv_p</t>
+  </si>
+  <si>
+    <t>Investment costs for new throughput power output capacity.</t>
+  </si>
+  <si>
+    <t>cost_fix_p</t>
+  </si>
+  <si>
+    <t>Operation independent costs for existing and new throughput power output capacity.</t>
+  </si>
+  <si>
+    <t>IRE_PRICE</t>
+  </si>
+  <si>
+    <t>commodity_price</t>
+  </si>
+  <si>
+    <t>Cost/Revenue for purchasing/selling one unit (MWh) of a stock or buy commodity.</t>
+  </si>
+  <si>
+    <t>iip_coke_oven_gas</t>
+  </si>
+  <si>
+    <t>iip_aluminum_alumina</t>
+  </si>
+  <si>
+    <t>iip_aluminum_crude</t>
+  </si>
+  <si>
+    <t>iip_aluminum_scrap</t>
+  </si>
+  <si>
+    <t>iip_black_liquor</t>
+  </si>
+  <si>
+    <t>iip_cement_clinker</t>
+  </si>
+  <si>
+    <t>iip_cement_rawmeal</t>
+  </si>
+  <si>
+    <t>iip_coke</t>
+  </si>
+  <si>
+    <t>iip_copper_scrap</t>
+  </si>
+  <si>
+    <t>iip_glass_cont_batch</t>
+  </si>
+  <si>
+    <t>iip_glass_cont_melt</t>
+  </si>
+  <si>
+    <t>iip_glass_flat_batch</t>
+  </si>
+  <si>
+    <t>iip_glass_flat_form</t>
+  </si>
+  <si>
+    <t>iip_glass_flat_melt</t>
+  </si>
+  <si>
+    <t>iip_heat_proc</t>
+  </si>
+  <si>
+    <t>iip_paper_pulp</t>
+  </si>
+  <si>
+    <t>iip_paper_recycle</t>
+  </si>
+  <si>
+    <t>co2_limit</t>
+  </si>
+  <si>
+    <t>potential_annual_max</t>
+  </si>
+  <si>
+    <t>shared_potential_id</t>
+  </si>
+  <si>
+    <t>capacity_p_min</t>
+  </si>
+  <si>
+    <t>capacity_p_max</t>
+  </si>
+  <si>
+    <t>capacity_e_min</t>
+  </si>
+  <si>
+    <t>capacity_e_max</t>
+  </si>
+  <si>
+    <t>capacity_w_min</t>
+  </si>
+  <si>
+    <t>capacity_w_max</t>
+  </si>
+  <si>
+    <t>capacity_tra_inst_0</t>
+  </si>
+  <si>
+    <t>availability_timeseries_fixed</t>
+  </si>
+  <si>
+    <t>availability_timeseries_max</t>
+  </si>
+  <si>
+    <t>wacc</t>
+  </si>
+  <si>
+    <t>cost_inv_tra</t>
+  </si>
+  <si>
+    <t>cost_fix_tra</t>
+  </si>
+  <si>
+    <t>cost_var_tra</t>
+  </si>
+  <si>
+    <t>conversion_factor_&lt;commodity&gt;</t>
+  </si>
+  <si>
+    <t>flow_share_min_&lt;commodity&gt;</t>
+  </si>
+  <si>
+    <t>flow_share_max_&lt;commodity&gt;</t>
+  </si>
+  <si>
+    <t>flow_share_fix_&lt;commodity&gt;</t>
+  </si>
+  <si>
+    <t>conversion_factor_timeseries_&lt;commodity&gt;</t>
+  </si>
+  <si>
+    <t>ef_&lt;input-commodity&gt;_&lt;emission&gt;</t>
+  </si>
+  <si>
+    <t>cb_coefficient</t>
+  </si>
+  <si>
+    <t>cv_coefficient</t>
+  </si>
+  <si>
+    <t>efficiency_sto_in</t>
+  </si>
+  <si>
+    <t>efficiency_sto_out</t>
+  </si>
+  <si>
+    <t>sto_init</t>
+  </si>
+  <si>
+    <t>sto_self_discharge</t>
+  </si>
+  <si>
+    <t>sto_ep_ratio_binding</t>
+  </si>
+  <si>
+    <t>sto_ep_ratio_optional</t>
+  </si>
+  <si>
+    <t>sto_cycles_max</t>
+  </si>
+  <si>
+    <t>capacity_tra_connection_max</t>
+  </si>
+  <si>
+    <t>capacity_tra_connection_timeseries</t>
+  </si>
+  <si>
+    <t>mileage</t>
+  </si>
+  <si>
+    <t>market_share_range</t>
+  </si>
+  <si>
+    <t>occupancy_rate</t>
+  </si>
+  <si>
+    <t>tonnage</t>
+  </si>
+  <si>
+    <t>share_tra_charge_mode</t>
+  </si>
+  <si>
+    <t>sto_min_timeseries</t>
+  </si>
+  <si>
+    <t>sto_max_timeseries</t>
+  </si>
+  <si>
+    <t>optional_limitations</t>
+  </si>
+  <si>
+    <t>id</t>
+  </si>
+  <si>
+    <t>region</t>
+  </si>
+  <si>
+    <t>year</t>
+  </si>
+  <si>
+    <t>bandwidth_type</t>
+  </si>
+  <si>
+    <t>version</t>
+  </si>
+  <si>
+    <t>method</t>
+  </si>
+  <si>
+    <t>source</t>
+  </si>
+  <si>
+    <t>comment</t>
+  </si>
+  <si>
+    <t>timeindex_stop</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>1/NCAP_CHPR?</t>
+  </si>
+  <si>
+    <t>NCAP_CEH</t>
+  </si>
+  <si>
+    <t>S_EFF</t>
+  </si>
+  <si>
+    <t>UC</t>
+  </si>
+  <si>
+    <t>COMBND_NET</t>
+  </si>
+  <si>
+    <t>ACT_COSTS</t>
+  </si>
+  <si>
+    <t>(?)</t>
+  </si>
+  <si>
+    <t>CO2 net emission budget for a period.</t>
+  </si>
+  <si>
+    <t>Maximum annual energy use of a commodity. </t>
+  </si>
+  <si>
+    <t>normalized demand timeseries which gets multiplied with demand_annual</t>
+  </si>
+  <si>
+    <t>specifies a name for a potential group in which all components share the same potential (e.g. wind turibine)</t>
+  </si>
+  <si>
+    <t>Existing throughput power output capacity per process in a certain year.</t>
+  </si>
+  <si>
+    <t>Minimum installable required throughput power output capacity per process.</t>
+  </si>
+  <si>
+    <t>Maximum installable required throughput power output capacity per process.</t>
+  </si>
+  <si>
+    <t>Minimum required storage energy capacity.</t>
+  </si>
+  <si>
+    <t>Maximum allowed storage energy capacity.</t>
+  </si>
+  <si>
+    <t>Maximum weight capacity of a process.</t>
+  </si>
+  <si>
+    <t>Minimum weight capacity of a process.</t>
+  </si>
+  <si>
+    <t>Number of vehicles.</t>
+  </si>
+  <si>
+    <t>Absolute upper bound on level of investment in new power output capacity for a period.</t>
+  </si>
+  <si>
+    <t>Time series of fixed capacity factor in relation to installed capacity.</t>
+  </si>
+  <si>
+    <t>Time series of maximum capacity factor in relation to installed capacity.</t>
+  </si>
+  <si>
+    <t>Percentage of costs for capital after taxes. Used to calculate annuity factor for investment costs.</t>
+  </si>
+  <si>
+    <t>Investment costs for new vehicle unit.</t>
+  </si>
+  <si>
+    <t>Operation independent costs for existing and new vehicle units.</t>
+  </si>
+  <si>
+    <t>Time-variable commodity-specific conversion factor.</t>
+  </si>
+  <si>
+    <t>Input-specific emission factor.</t>
+  </si>
+  <si>
+    <t>The Cb-coefficient (backpressure coefficient) is defined as the maximum power generation capacity in backpressure mode divided by the maximum heat production capacity (including flue gas condensation if applicable).</t>
+  </si>
+  <si>
+    <t>The Cv-value for an extraction steam turbine is defined as the loss of electricity production, when the heat production is increased one unit at constant fuel input.</t>
+  </si>
+  <si>
+    <t>Energy efficiency of power input.</t>
+  </si>
+  <si>
+    <t>Energy efficiency of power output.</t>
+  </si>
+  <si>
+    <t>The initial state of charge of a storage.</t>
+  </si>
+  <si>
+    <t>Storage losses over time.</t>
+  </si>
+  <si>
+    <t>Fixed ratio of the storage energy capacity to its power output capacity.</t>
+  </si>
+  <si>
+    <t>Optional fixed ratio of the storage energy capacity to its power output capacity.</t>
+  </si>
+  <si>
+    <t>Defines the maximum number of full storage cycle equivalents over the lifetime.</t>
+  </si>
+  <si>
+    <t>Maximum connection capacity of an average electric vehicle, taken the connection availability into acocunt.</t>
+  </si>
+  <si>
+    <t>Connection capacity of an average electric vehicle.</t>
+  </si>
+  <si>
+    <t>Yearly mileage of a vehicle.</t>
+  </si>
+  <si>
+    <t>Range of market share.</t>
+  </si>
+  <si>
+    <t>Occupancy rate of a vehicle.</t>
+  </si>
+  <si>
+    <t>Tonnes transported per vehicle.</t>
+  </si>
+  <si>
+    <t>Proportion of fleet that load with a soecific charge mode..</t>
+  </si>
+  <si>
+    <t>Time series of min battery state of charge.</t>
+  </si>
+  <si>
+    <t>Time series of max battery state of charge.</t>
+  </si>
+  <si>
+    <t>User constraint to describe market limitations.</t>
+  </si>
+  <si>
+    <t>Scenario/Milestone steps in the defined time horizon of the intertemporal model</t>
+  </si>
+  <si>
+    <t>Have to figure it out, how to implement</t>
+  </si>
+  <si>
+    <t>data columns info</t>
+  </si>
+  <si>
+    <t>NCAP_CHPR</t>
+  </si>
+  <si>
+    <t>iip_auto_parts_pc_phev</t>
+  </si>
+  <si>
+    <t>iip_chemi_steam</t>
+  </si>
+  <si>
+    <t>iip_auto_painted_pc_fcev</t>
+  </si>
+  <si>
+    <t>iip_elec</t>
+  </si>
+  <si>
+    <t>iip_auto_parts_lcv_icev</t>
+  </si>
+  <si>
+    <t>iip_auto_painted_pc_icev</t>
+  </si>
+  <si>
+    <t>iip_auto_painted_lcv_icev</t>
+  </si>
+  <si>
+    <t>iip_chemi_naphtha</t>
+  </si>
+  <si>
+    <t>iip_auto_btry_hcv_icev</t>
+  </si>
+  <si>
+    <t>iip_auto_painted_lcv_fcev</t>
+  </si>
+  <si>
+    <t>iip_chemi_meoh_h2</t>
+  </si>
+  <si>
+    <t>iip_steam</t>
+  </si>
+  <si>
+    <t>iip_auto_parts_lcv_fcev</t>
+  </si>
+  <si>
+    <t>iip_chemi_process_heat</t>
+  </si>
+  <si>
+    <t>iip_auto_btry_lcv_bev</t>
+  </si>
+  <si>
+    <t>iip_auto_parts_pc_icev</t>
+  </si>
+  <si>
+    <t>iip_chemi_heavy_fuel_oil</t>
+  </si>
+  <si>
+    <t>iip_auto_btry_pc_fcev</t>
+  </si>
+  <si>
+    <t>iip_auto_painted_hcv_icev</t>
+  </si>
+  <si>
+    <t>iip_auto_parts_hcv_icev</t>
+  </si>
+  <si>
+    <t>iip_chemi_machine_drive</t>
+  </si>
+  <si>
+    <t>iip_auto_painted_hcv_fcev</t>
+  </si>
+  <si>
+    <t>iip_auto_btry_pc_bev</t>
+  </si>
+  <si>
+    <t>iip_auto_parts_pc_bev</t>
+  </si>
+  <si>
+    <t>iip_auto_btry_pc_phev</t>
+  </si>
+  <si>
+    <t>iip_chemi_nh3_h2</t>
+  </si>
+  <si>
+    <t>iip_auto_painted_pc_bev</t>
+  </si>
+  <si>
+    <t>iip_blafu_gas</t>
+  </si>
+  <si>
+    <t>iip_chemi_methanol</t>
+  </si>
+  <si>
+    <t>iip_chemi_biomethanol</t>
+  </si>
+  <si>
+    <t>iip_auto_btry_hcv_fcev</t>
+  </si>
+  <si>
+    <t>iip_auto_btry_lcv_fcev</t>
+  </si>
+  <si>
+    <t>iip_auto_parts_lcv_bev</t>
+  </si>
+  <si>
+    <t>iip_auto_painted_hcv_bev</t>
+  </si>
+  <si>
+    <t>iip_auto_parts_hcv_fcev</t>
+  </si>
+  <si>
+    <t>iip_auto_btry_pc_icev</t>
+  </si>
+  <si>
+    <t>iip_chemi_electro_chem</t>
+  </si>
+  <si>
+    <t>iip_auto_btry_hcv_bev</t>
+  </si>
+  <si>
+    <t>iip_auto_parts_pc_fcev</t>
+  </si>
+  <si>
+    <t>iip_auto_painted_lcv_bev</t>
+  </si>
+  <si>
+    <t>iip_chemi_meoh_f_h2</t>
+  </si>
+  <si>
+    <t>iip_chemi_mtg_mtk_h2</t>
+  </si>
+  <si>
+    <t>iip_chemi_nh3</t>
+  </si>
+  <si>
+    <t>iip_auto_btry_lcv_icev</t>
+  </si>
+  <si>
+    <t>iip_auto_painted_pc_phev</t>
+  </si>
+  <si>
+    <t>iip_chemi_biomass</t>
+  </si>
+  <si>
+    <t>iip_auto_parts_hcv_bev</t>
+  </si>
+  <si>
+    <t>iip_chemi_methane</t>
+  </si>
+  <si>
+    <t>iip_chemi_processes_others</t>
+  </si>
+  <si>
+    <t>exo_aluminum</t>
+  </si>
+  <si>
+    <t>sec_waste_heat_high_aluminum</t>
+  </si>
+  <si>
+    <t>exo_cement</t>
+  </si>
+  <si>
+    <t>sec_waste_heat_high_cement</t>
+  </si>
+  <si>
+    <t>exo_copper</t>
+  </si>
+  <si>
+    <t>sec_waste_heat_high_copper</t>
+  </si>
+  <si>
+    <t>exo_glass_flat</t>
+  </si>
+  <si>
+    <t>exo_glass_cont</t>
+  </si>
+  <si>
+    <t>exo_glass_fibe</t>
+  </si>
+  <si>
+    <t>sec_waste_heat_high_glass</t>
+  </si>
+  <si>
+    <t>exo_glass_spec</t>
+  </si>
+  <si>
+    <t>exo_steel</t>
+  </si>
+  <si>
+    <t>sec_waste_heat_high_steel</t>
+  </si>
+  <si>
+    <t>iip_blafu_gas_in</t>
+  </si>
+  <si>
+    <t>pri_biomass_stemwood</t>
+  </si>
+  <si>
+    <t>emi_ch4_f_ind</t>
+  </si>
+  <si>
+    <t>emi_ch4_p_ind</t>
+  </si>
+  <si>
+    <t>emi_co2_f_ind</t>
+  </si>
+  <si>
+    <t>emi_co2_p_ind</t>
+  </si>
+  <si>
+    <t>emi_co2_reusable</t>
+  </si>
+  <si>
+    <t>emi_co2_stored</t>
+  </si>
+  <si>
+    <t>pri_coal</t>
+  </si>
+  <si>
+    <t>iip_coke_oven_gas_in</t>
+  </si>
+  <si>
+    <t>sec_elec_ind</t>
+  </si>
+  <si>
+    <t>sec_methane</t>
+  </si>
+  <si>
+    <t>sec_hydrogen</t>
+  </si>
+  <si>
+    <t>sec_heavy_fuel_oil</t>
+  </si>
+  <si>
+    <t>emi_n2o_f_ind</t>
+  </si>
+  <si>
+    <t>emi_co2_neg_fuel_cc_ind</t>
+  </si>
+  <si>
+    <t>emi_co2_neg_proc_cc_ind</t>
+  </si>
+  <si>
+    <t>pri_sewage_sludge</t>
+  </si>
+  <si>
+    <t>pri_waste_non_bio</t>
+  </si>
+  <si>
+    <t>exo_paper_hq</t>
+  </si>
+  <si>
+    <t>exo_paper_lq</t>
+  </si>
+  <si>
+    <t>sec_waste_heat_high_paper</t>
+  </si>
+  <si>
+    <t>sec_elec</t>
+  </si>
+  <si>
+    <t>exo_chemi_btx</t>
+  </si>
+  <si>
+    <t>exo_chemi_others</t>
+  </si>
+  <si>
+    <t>sec_heat_district_high_ind</t>
+  </si>
+  <si>
+    <t>sec_lpg</t>
+  </si>
+  <si>
+    <t>pri_waste_municipal_bio</t>
+  </si>
+  <si>
+    <t>sec_naphtha</t>
+  </si>
+  <si>
+    <t>sec_refinery_gas</t>
+  </si>
+  <si>
+    <t>sec_waste_heat_high_chemi</t>
+  </si>
+  <si>
+    <t>exo_chemi_cl2</t>
+  </si>
+  <si>
+    <t>exo_chemi_methanol</t>
+  </si>
+  <si>
+    <t>exo_chemi_nh3</t>
+  </si>
+  <si>
+    <t>exo_chemi_olefins</t>
+  </si>
+  <si>
+    <t>sec_gasoline_orig</t>
+  </si>
+  <si>
+    <t>sec_kerosene_orig</t>
+  </si>
+  <si>
+    <t>iip_chemi_lpg</t>
+  </si>
+  <si>
+    <t>sec_ammonia_orig</t>
+  </si>
+  <si>
+    <t>sec_methanol_orig</t>
+  </si>
+  <si>
+    <t>sec_biomethanol_orig</t>
+  </si>
+  <si>
+    <t>emi_n2o_p_ind</t>
+  </si>
+  <si>
+    <t>exo_agri_livestock</t>
+  </si>
+  <si>
+    <t>Availability</t>
+  </si>
+  <si>
+    <t>ACTFLO~DEMO</t>
+  </si>
+  <si>
+    <t>emi_co2_neg_imp</t>
+  </si>
+  <si>
+    <t>emi_co2_neg_air_bio</t>
+  </si>
+  <si>
+    <t>emi_co2_neg_air_dacc</t>
+  </si>
+  <si>
     <t>ACT_BND</t>
-  </si>
-  <si>
-    <t>ACT_COST</t>
-  </si>
-  <si>
-    <t>NCAP_BND</t>
-  </si>
-  <si>
-    <t>PRC_RESID</t>
-  </si>
-  <si>
-    <t>NCAP_FOM</t>
-  </si>
-  <si>
-    <t>NCAP_TLIFE</t>
-  </si>
-  <si>
-    <t>Absolute upper bound on level of investment in new weight capacity for a period.</t>
-  </si>
-  <si>
-    <t>Investment costs for new capacity per unit weight.</t>
-  </si>
-  <si>
-    <t>Operation independent costs for capacity per unit weight.</t>
-  </si>
-  <si>
-    <t>Technical lifetime of a process.</t>
-  </si>
-  <si>
-    <t>Projected annual demand for a commodity.</t>
-  </si>
-  <si>
-    <t>Comment</t>
-  </si>
-  <si>
-    <t>UP</t>
-  </si>
-  <si>
-    <t>max</t>
-  </si>
-  <si>
-    <t>LO</t>
-  </si>
-  <si>
-    <t>min</t>
-  </si>
-  <si>
-    <t>FX</t>
-  </si>
-  <si>
-    <t>fix</t>
-  </si>
-  <si>
-    <t>FLO_SHAR</t>
-  </si>
-  <si>
-    <t>COM_PROJ</t>
-  </si>
-  <si>
-    <t>CommName</t>
-  </si>
-  <si>
-    <t>CommDesc</t>
-  </si>
-  <si>
-    <t>Unit</t>
-  </si>
-  <si>
-    <t>Csets</t>
-  </si>
-  <si>
-    <t>Commodity Name</t>
-  </si>
-  <si>
-    <t>Commodity Description</t>
-  </si>
-  <si>
-    <t>*Commodity Set Membership</t>
-  </si>
-  <si>
-    <t>iip_steel_sinter</t>
-  </si>
-  <si>
-    <t>MAT</t>
-  </si>
-  <si>
-    <t>iip_steel_crudesteel</t>
-  </si>
-  <si>
-    <t>iip_steel_sponge_iron</t>
-  </si>
-  <si>
-    <t>iip_steel_scrap</t>
-  </si>
-  <si>
-    <t>iip_steel_raw_iron</t>
-  </si>
-  <si>
-    <t>iip_steel_iron_pellets</t>
-  </si>
-  <si>
-    <t>type</t>
-  </si>
-  <si>
-    <t>SEDOS_unit</t>
-  </si>
-  <si>
-    <t>isAbout</t>
-  </si>
-  <si>
-    <t>valueReference</t>
-  </si>
-  <si>
-    <t>Constraints</t>
-  </si>
-  <si>
-    <t>demand_timeseries</t>
-  </si>
-  <si>
-    <t>timeindex_start</t>
-  </si>
-  <si>
-    <t>timeindex_resolution</t>
-  </si>
-  <si>
-    <t>NCAP_AF</t>
-  </si>
-  <si>
-    <t>Constant output ratio in relation to installed capacity. (= h/a)</t>
-  </si>
-  <si>
-    <t>FLO_EFF</t>
-  </si>
-  <si>
-    <t>Commodity-specific conversion factor (multiplication of input and output factors yields the efficiency of the process).</t>
-  </si>
-  <si>
-    <t>Minimum share of flow commodity c based upon the sum of individual flows defined by the commodity group cg belonging to process p.</t>
-  </si>
-  <si>
-    <t>Maximum share of flow commodity c based upon the sum of individual flows defined by the commodity group cg belonging to process p.</t>
-  </si>
-  <si>
-    <t>Fixed share of flow commodity c based upon the sum of individual flows defined by the commodity group cg belonging to process p.</t>
-  </si>
-  <si>
-    <t>capacity_w_inst_0</t>
-  </si>
-  <si>
-    <t>Existing weight capacity of a process.</t>
-  </si>
-  <si>
-    <t>NCAP_COST</t>
-  </si>
-  <si>
-    <t>cost_inv_w</t>
-  </si>
-  <si>
-    <t>cost_fix_w</t>
-  </si>
-  <si>
-    <t>cost_var_w</t>
-  </si>
-  <si>
-    <t>Variable costs per throughput weight unit output. (excluding fuel costs).</t>
-  </si>
-  <si>
-    <t>capacity_w_abs_new_max</t>
-  </si>
-  <si>
-    <t>capacity_e_inst_0</t>
-  </si>
-  <si>
-    <t>Existing storage energy capacity.</t>
-  </si>
-  <si>
-    <t>cost_inv_e</t>
-  </si>
-  <si>
-    <t>Investment costs for new storage energy capacity.</t>
-  </si>
-  <si>
-    <t>cost_fix_e</t>
-  </si>
-  <si>
-    <t>Operation independent costs for existing and new storage energy capacity.</t>
-  </si>
-  <si>
-    <t>cost_var_e</t>
-  </si>
-  <si>
-    <t>Variable costs per throughput energy unit output. (excluding fuel costs).</t>
-  </si>
-  <si>
-    <t>capacity_e_abs_new_max</t>
-  </si>
-  <si>
-    <t>Absolute upper bound on level of investment in new storage energy capacity for a period.</t>
-  </si>
-  <si>
-    <t>capacity_p_inst_0</t>
-  </si>
-  <si>
-    <t>capacity_p_abs_new_max</t>
-  </si>
-  <si>
-    <t>cost_inv_p</t>
-  </si>
-  <si>
-    <t>Investment costs for new throughput power output capacity.</t>
-  </si>
-  <si>
-    <t>cost_fix_p</t>
-  </si>
-  <si>
-    <t>Operation independent costs for existing and new throughput power output capacity.</t>
-  </si>
-  <si>
-    <t>IRE_PRICE</t>
-  </si>
-  <si>
-    <t>commodity_price</t>
-  </si>
-  <si>
-    <t>Cost/Revenue for purchasing/selling one unit (MWh) of a stock or buy commodity.</t>
-  </si>
-  <si>
-    <t>iip_coke_oven_gas</t>
-  </si>
-  <si>
-    <t>iip_aluminum_alumina</t>
-  </si>
-  <si>
-    <t>iip_aluminum_crude</t>
-  </si>
-  <si>
-    <t>iip_aluminum_scrap</t>
-  </si>
-  <si>
-    <t>iip_black_liquor</t>
-  </si>
-  <si>
-    <t>iip_cement_clinker</t>
-  </si>
-  <si>
-    <t>iip_cement_rawmeal</t>
-  </si>
-  <si>
-    <t>iip_coke</t>
-  </si>
-  <si>
-    <t>iip_copper_scrap</t>
-  </si>
-  <si>
-    <t>iip_glass_cont_batch</t>
-  </si>
-  <si>
-    <t>iip_glass_cont_melt</t>
-  </si>
-  <si>
-    <t>iip_glass_flat_batch</t>
-  </si>
-  <si>
-    <t>iip_glass_flat_form</t>
-  </si>
-  <si>
-    <t>iip_glass_flat_melt</t>
-  </si>
-  <si>
-    <t>iip_heat_proc</t>
-  </si>
-  <si>
-    <t>iip_paper_pulp</t>
-  </si>
-  <si>
-    <t>iip_paper_recycle</t>
-  </si>
-  <si>
-    <t>co2_limit</t>
-  </si>
-  <si>
-    <t>potential_annual_max</t>
-  </si>
-  <si>
-    <t>shared_potential_id</t>
-  </si>
-  <si>
-    <t>capacity_p_min</t>
-  </si>
-  <si>
-    <t>capacity_p_max</t>
-  </si>
-  <si>
-    <t>capacity_e_min</t>
-  </si>
-  <si>
-    <t>capacity_e_max</t>
-  </si>
-  <si>
-    <t>capacity_w_min</t>
-  </si>
-  <si>
-    <t>capacity_w_max</t>
-  </si>
-  <si>
-    <t>capacity_tra_inst_0</t>
-  </si>
-  <si>
-    <t>availability_timeseries_fixed</t>
-  </si>
-  <si>
-    <t>availability_timeseries_max</t>
-  </si>
-  <si>
-    <t>wacc</t>
-  </si>
-  <si>
-    <t>cost_inv_tra</t>
-  </si>
-  <si>
-    <t>cost_fix_tra</t>
-  </si>
-  <si>
-    <t>cost_var_tra</t>
-  </si>
-  <si>
-    <t>conversion_factor_&lt;commodity&gt;</t>
-  </si>
-  <si>
-    <t>flow_share_min_&lt;commodity&gt;</t>
-  </si>
-  <si>
-    <t>flow_share_max_&lt;commodity&gt;</t>
-  </si>
-  <si>
-    <t>flow_share_fix_&lt;commodity&gt;</t>
-  </si>
-  <si>
-    <t>conversion_factor_timeseries_&lt;commodity&gt;</t>
-  </si>
-  <si>
-    <t>ef_&lt;input-commodity&gt;_&lt;emission&gt;</t>
-  </si>
-  <si>
-    <t>cb_coefficient</t>
-  </si>
-  <si>
-    <t>cv_coefficient</t>
-  </si>
-  <si>
-    <t>efficiency_sto_in</t>
-  </si>
-  <si>
-    <t>efficiency_sto_out</t>
-  </si>
-  <si>
-    <t>sto_init</t>
-  </si>
-  <si>
-    <t>sto_self_discharge</t>
-  </si>
-  <si>
-    <t>sto_ep_ratio_binding</t>
-  </si>
-  <si>
-    <t>sto_ep_ratio_optional</t>
-  </si>
-  <si>
-    <t>sto_cycles_max</t>
-  </si>
-  <si>
-    <t>capacity_tra_connection_max</t>
-  </si>
-  <si>
-    <t>capacity_tra_connection_timeseries</t>
-  </si>
-  <si>
-    <t>mileage</t>
-  </si>
-  <si>
-    <t>market_share_range</t>
-  </si>
-  <si>
-    <t>occupancy_rate</t>
-  </si>
-  <si>
-    <t>tonnage</t>
-  </si>
-  <si>
-    <t>share_tra_charge_mode</t>
-  </si>
-  <si>
-    <t>sto_min_timeseries</t>
-  </si>
-  <si>
-    <t>sto_max_timeseries</t>
-  </si>
-  <si>
-    <t>optional_limitations</t>
-  </si>
-  <si>
-    <t>id</t>
-  </si>
-  <si>
-    <t>region</t>
-  </si>
-  <si>
-    <t>year</t>
-  </si>
-  <si>
-    <t>bandwidth_type</t>
-  </si>
-  <si>
-    <t>version</t>
-  </si>
-  <si>
-    <t>method</t>
-  </si>
-  <si>
-    <t>source</t>
-  </si>
-  <si>
-    <t>comment</t>
-  </si>
-  <si>
-    <t>timeindex_stop</t>
-  </si>
-  <si>
-    <t>-</t>
-  </si>
-  <si>
-    <t>1/NCAP_CHPR?</t>
-  </si>
-  <si>
-    <t>NCAP_CEH</t>
-  </si>
-  <si>
-    <t>S_EFF</t>
-  </si>
-  <si>
-    <t>UC</t>
-  </si>
-  <si>
-    <t>COMBND_NET</t>
-  </si>
-  <si>
-    <t>ACT_COSTS</t>
-  </si>
-  <si>
-    <t>(?)</t>
-  </si>
-  <si>
-    <t>CO2 net emission budget for a period.</t>
-  </si>
-  <si>
-    <t>Maximum annual energy use of a commodity. </t>
-  </si>
-  <si>
-    <t>normalized demand timeseries which gets multiplied with demand_annual</t>
-  </si>
-  <si>
-    <t>specifies a name for a potential group in which all components share the same potential (e.g. wind turibine)</t>
-  </si>
-  <si>
-    <t>Existing throughput power output capacity per process in a certain year.</t>
-  </si>
-  <si>
-    <t>Minimum installable required throughput power output capacity per process.</t>
-  </si>
-  <si>
-    <t>Maximum installable required throughput power output capacity per process.</t>
-  </si>
-  <si>
-    <t>Minimum required storage energy capacity.</t>
-  </si>
-  <si>
-    <t>Maximum allowed storage energy capacity.</t>
-  </si>
-  <si>
-    <t>Maximum weight capacity of a process.</t>
-  </si>
-  <si>
-    <t>Minimum weight capacity of a process.</t>
-  </si>
-  <si>
-    <t>Number of vehicles.</t>
-  </si>
-  <si>
-    <t>Absolute upper bound on level of investment in new power output capacity for a period.</t>
-  </si>
-  <si>
-    <t>Time series of fixed capacity factor in relation to installed capacity.</t>
-  </si>
-  <si>
-    <t>Time series of maximum capacity factor in relation to installed capacity.</t>
-  </si>
-  <si>
-    <t>Percentage of costs for capital after taxes. Used to calculate annuity factor for investment costs.</t>
-  </si>
-  <si>
-    <t>Investment costs for new vehicle unit.</t>
-  </si>
-  <si>
-    <t>Operation independent costs for existing and new vehicle units.</t>
-  </si>
-  <si>
-    <t>Time-variable commodity-specific conversion factor.</t>
-  </si>
-  <si>
-    <t>Input-specific emission factor.</t>
-  </si>
-  <si>
-    <t>The Cb-coefficient (backpressure coefficient) is defined as the maximum power generation capacity in backpressure mode divided by the maximum heat production capacity (including flue gas condensation if applicable).</t>
-  </si>
-  <si>
-    <t>The Cv-value for an extraction steam turbine is defined as the loss of electricity production, when the heat production is increased one unit at constant fuel input.</t>
-  </si>
-  <si>
-    <t>Energy efficiency of power input.</t>
-  </si>
-  <si>
-    <t>Energy efficiency of power output.</t>
-  </si>
-  <si>
-    <t>The initial state of charge of a storage.</t>
-  </si>
-  <si>
-    <t>Storage losses over time.</t>
-  </si>
-  <si>
-    <t>Fixed ratio of the storage energy capacity to its power output capacity.</t>
-  </si>
-  <si>
-    <t>Optional fixed ratio of the storage energy capacity to its power output capacity.</t>
-  </si>
-  <si>
-    <t>Defines the maximum number of full storage cycle equivalents over the lifetime.</t>
-  </si>
-  <si>
-    <t>Maximum connection capacity of an average electric vehicle, taken the connection availability into acocunt.</t>
-  </si>
-  <si>
-    <t>Connection capacity of an average electric vehicle.</t>
-  </si>
-  <si>
-    <t>Yearly mileage of a vehicle.</t>
-  </si>
-  <si>
-    <t>Range of market share.</t>
-  </si>
-  <si>
-    <t>Occupancy rate of a vehicle.</t>
-  </si>
-  <si>
-    <t>Tonnes transported per vehicle.</t>
-  </si>
-  <si>
-    <t>Proportion of fleet that load with a soecific charge mode..</t>
-  </si>
-  <si>
-    <t>Time series of min battery state of charge.</t>
-  </si>
-  <si>
-    <t>Time series of max battery state of charge.</t>
-  </si>
-  <si>
-    <t>User constraint to describe market limitations.</t>
-  </si>
-  <si>
-    <t>Scenario/Milestone steps in the defined time horizon of the intertemporal model</t>
-  </si>
-  <si>
-    <t>Have to figure it out, how to implement</t>
-  </si>
-  <si>
-    <t>data columns info</t>
-  </si>
-  <si>
-    <t>NCAP_CHPR</t>
-  </si>
-  <si>
-    <t>iip_auto_parts_pc_phev</t>
-  </si>
-  <si>
-    <t>iip_chemi_steam</t>
-  </si>
-  <si>
-    <t>iip_auto_painted_pc_fcev</t>
-  </si>
-  <si>
-    <t>iip_elec</t>
-  </si>
-  <si>
-    <t>iip_auto_parts_lcv_icev</t>
-  </si>
-  <si>
-    <t>iip_auto_painted_pc_icev</t>
-  </si>
-  <si>
-    <t>iip_auto_painted_lcv_icev</t>
-  </si>
-  <si>
-    <t>iip_chemi_naphtha</t>
-  </si>
-  <si>
-    <t>iip_auto_btry_hcv_icev</t>
-  </si>
-  <si>
-    <t>iip_auto_painted_lcv_fcev</t>
-  </si>
-  <si>
-    <t>iip_chemi_meoh_h2</t>
-  </si>
-  <si>
-    <t>iip_steam</t>
-  </si>
-  <si>
-    <t>iip_auto_parts_lcv_fcev</t>
-  </si>
-  <si>
-    <t>iip_chemi_process_heat</t>
-  </si>
-  <si>
-    <t>iip_auto_btry_lcv_bev</t>
-  </si>
-  <si>
-    <t>iip_auto_parts_pc_icev</t>
-  </si>
-  <si>
-    <t>iip_chemi_heavy_fuel_oil</t>
-  </si>
-  <si>
-    <t>iip_auto_btry_pc_fcev</t>
-  </si>
-  <si>
-    <t>iip_auto_painted_hcv_icev</t>
-  </si>
-  <si>
-    <t>iip_auto_parts_hcv_icev</t>
-  </si>
-  <si>
-    <t>iip_chemi_machine_drive</t>
-  </si>
-  <si>
-    <t>iip_auto_painted_hcv_fcev</t>
-  </si>
-  <si>
-    <t>iip_auto_btry_pc_bev</t>
-  </si>
-  <si>
-    <t>iip_auto_parts_pc_bev</t>
-  </si>
-  <si>
-    <t>iip_auto_btry_pc_phev</t>
-  </si>
-  <si>
-    <t>iip_chemi_nh3_h2</t>
-  </si>
-  <si>
-    <t>iip_auto_painted_pc_bev</t>
-  </si>
-  <si>
-    <t>iip_blafu_gas</t>
-  </si>
-  <si>
-    <t>iip_chemi_methanol</t>
-  </si>
-  <si>
-    <t>iip_chemi_biomethanol</t>
-  </si>
-  <si>
-    <t>iip_auto_btry_hcv_fcev</t>
-  </si>
-  <si>
-    <t>iip_auto_btry_lcv_fcev</t>
-  </si>
-  <si>
-    <t>iip_auto_parts_lcv_bev</t>
-  </si>
-  <si>
-    <t>iip_auto_painted_hcv_bev</t>
-  </si>
-  <si>
-    <t>iip_auto_parts_hcv_fcev</t>
-  </si>
-  <si>
-    <t>iip_auto_btry_pc_icev</t>
-  </si>
-  <si>
-    <t>iip_chemi_electro_chem</t>
-  </si>
-  <si>
-    <t>iip_auto_btry_hcv_bev</t>
-  </si>
-  <si>
-    <t>iip_auto_parts_pc_fcev</t>
-  </si>
-  <si>
-    <t>iip_auto_painted_lcv_bev</t>
-  </si>
-  <si>
-    <t>iip_chemi_meoh_f_h2</t>
-  </si>
-  <si>
-    <t>iip_chemi_mtg_mtk_h2</t>
-  </si>
-  <si>
-    <t>iip_chemi_nh3</t>
-  </si>
-  <si>
-    <t>iip_auto_btry_lcv_icev</t>
-  </si>
-  <si>
-    <t>iip_auto_painted_pc_phev</t>
-  </si>
-  <si>
-    <t>iip_chemi_biomass</t>
-  </si>
-  <si>
-    <t>iip_auto_parts_hcv_bev</t>
-  </si>
-  <si>
-    <t>iip_chemi_methane</t>
-  </si>
-  <si>
-    <t>iip_chemi_processes_others</t>
-  </si>
-  <si>
-    <t>exo_aluminum</t>
-  </si>
-  <si>
-    <t>sec_waste_heat_high_aluminum</t>
-  </si>
-  <si>
-    <t>exo_cement</t>
-  </si>
-  <si>
-    <t>sec_waste_heat_high_cement</t>
-  </si>
-  <si>
-    <t>exo_copper</t>
-  </si>
-  <si>
-    <t>sec_waste_heat_high_copper</t>
-  </si>
-  <si>
-    <t>exo_glass_flat</t>
-  </si>
-  <si>
-    <t>exo_glass_cont</t>
-  </si>
-  <si>
-    <t>exo_glass_fibe</t>
-  </si>
-  <si>
-    <t>sec_waste_heat_high_glass</t>
-  </si>
-  <si>
-    <t>exo_glass_spec</t>
-  </si>
-  <si>
-    <t>exo_steel</t>
-  </si>
-  <si>
-    <t>sec_waste_heat_high_steel</t>
-  </si>
-  <si>
-    <t>iip_blafu_gas_in</t>
-  </si>
-  <si>
-    <t>pri_biomass_stemwood</t>
-  </si>
-  <si>
-    <t>emi_ch4_f_ind</t>
-  </si>
-  <si>
-    <t>emi_ch4_p_ind</t>
-  </si>
-  <si>
-    <t>emi_co2_f_ind</t>
-  </si>
-  <si>
-    <t>emi_co2_p_ind</t>
-  </si>
-  <si>
-    <t>emi_co2_reusable</t>
-  </si>
-  <si>
-    <t>emi_co2_stored</t>
-  </si>
-  <si>
-    <t>pri_coal</t>
-  </si>
-  <si>
-    <t>iip_coke_oven_gas_in</t>
-  </si>
-  <si>
-    <t>sec_elec_ind</t>
-  </si>
-  <si>
-    <t>sec_methane</t>
-  </si>
-  <si>
-    <t>sec_hydrogen</t>
-  </si>
-  <si>
-    <t>sec_heavy_fuel_oil</t>
-  </si>
-  <si>
-    <t>emi_n2o_f_ind</t>
-  </si>
-  <si>
-    <t>emi_co2_neg_fuel_cc_ind</t>
-  </si>
-  <si>
-    <t>emi_co2_neg_proc_cc_ind</t>
-  </si>
-  <si>
-    <t>pri_sewage_sludge</t>
-  </si>
-  <si>
-    <t>pri_waste_non_bio</t>
-  </si>
-  <si>
-    <t>exo_paper_hq</t>
-  </si>
-  <si>
-    <t>exo_paper_lq</t>
-  </si>
-  <si>
-    <t>sec_waste_heat_high_paper</t>
-  </si>
-  <si>
-    <t>sec_elec</t>
-  </si>
-  <si>
-    <t>exo_chemi_btx</t>
-  </si>
-  <si>
-    <t>exo_chemi_others</t>
-  </si>
-  <si>
-    <t>sec_heat_district_high_ind</t>
-  </si>
-  <si>
-    <t>sec_lpg</t>
-  </si>
-  <si>
-    <t>pri_waste_municipal_bio</t>
-  </si>
-  <si>
-    <t>sec_naphtha</t>
-  </si>
-  <si>
-    <t>sec_refinery_gas</t>
-  </si>
-  <si>
-    <t>sec_waste_heat_high_chemi</t>
-  </si>
-  <si>
-    <t>exo_chemi_cl2</t>
-  </si>
-  <si>
-    <t>exo_chemi_methanol</t>
-  </si>
-  <si>
-    <t>exo_chemi_nh3</t>
-  </si>
-  <si>
-    <t>exo_chemi_olefins</t>
-  </si>
-  <si>
-    <t>sec_gasoline_orig</t>
-  </si>
-  <si>
-    <t>sec_kerosene_orig</t>
-  </si>
-  <si>
-    <t>iip_chemi_lpg</t>
-  </si>
-  <si>
-    <t>sec_ammonia_orig</t>
-  </si>
-  <si>
-    <t>sec_methanol_orig</t>
-  </si>
-  <si>
-    <t>sec_biomethanol_orig</t>
-  </si>
-  <si>
-    <t>emi_n2o_p_ind</t>
-  </si>
-  <si>
-    <t>exo_agri_livestock</t>
-  </si>
-  <si>
-    <t>Availability</t>
-  </si>
-  <si>
-    <t>ACTFLO~DEMO</t>
-  </si>
-  <si>
-    <t>emi_co2_neg_imp</t>
-  </si>
-  <si>
-    <t>emi_co2_neg_air_bio</t>
   </si>
 </sst>
 </file>
@@ -1086,7 +1089,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1114,6 +1117,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="8" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="-0.249977111117893"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1151,7 +1160,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1197,6 +1206,10 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1548,36 +1561,36 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="F1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="I1" s="1" t="s">
-        <v>45</v>
-      </c>
       <c r="J1" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C2" s="12" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.35">
@@ -1585,58 +1598,58 @@
         <v>5</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C4" t="s">
         <v>81</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="C4" t="s">
-        <v>82</v>
-      </c>
       <c r="J4" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A5" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>7</v>
+      <c r="A5" s="21" t="s">
+        <v>100</v>
+      </c>
+      <c r="B5" s="22" t="s">
+        <v>310</v>
       </c>
       <c r="C5" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="I5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="N5" s="9"/>
       <c r="O5" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A6" s="9" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B6" s="9"/>
       <c r="C6" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="N6" s="7"/>
       <c r="O6" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.35">
@@ -1644,189 +1657,189 @@
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C7" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A8" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B8" s="9"/>
       <c r="C8" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C9" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C10" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="I10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C11" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="I11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C12" t="s">
         <v>64</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C12" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C13" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="I13" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C14" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I14" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C15" t="s">
         <v>56</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C15" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C16" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I16" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C17" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="I17" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C18" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C19" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="I19" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C20" t="s">
         <v>72</v>
       </c>
-      <c r="B20" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C20" t="s">
-        <v>73</v>
-      </c>
       <c r="I20" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A21" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C21" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="I21" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.35">
@@ -1834,497 +1847,497 @@
         <v>4</v>
       </c>
       <c r="B22" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C22" t="s">
         <v>49</v>
-      </c>
-      <c r="C22" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A23" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C23" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A24" s="9" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C24" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B25" s="2"/>
       <c r="C25" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="J25" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C26" t="s">
         <v>76</v>
-      </c>
-      <c r="B26" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="C26" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A27" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C27" t="s">
         <v>66</v>
-      </c>
-      <c r="B27" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="C27" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C28" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A29" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C29" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C30" t="s">
         <v>78</v>
-      </c>
-      <c r="B30" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C30" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A31" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C31" t="s">
         <v>68</v>
-      </c>
-      <c r="B31" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C31" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A32" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C32" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A33" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C33" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A34" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C34" t="s">
         <v>70</v>
-      </c>
-      <c r="B34" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C34" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A35" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A36" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C36" t="s">
         <v>61</v>
-      </c>
-      <c r="B36" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C36" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A37" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B37" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C37" t="s">
         <v>51</v>
-      </c>
-      <c r="C37" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A38" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C38" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I38" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A39" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C39" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="I39" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A40" s="2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C40" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="I40" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A41" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C41" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A42" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B42" s="2"/>
       <c r="C42" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A43" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C43" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="J43" s="2" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A44" s="2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C44" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A45" s="2" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C45" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A46" s="9" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B46" s="9"/>
       <c r="C46" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A47" s="9" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B47" s="9"/>
       <c r="C47" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A48" s="9" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B48" s="9"/>
       <c r="C48" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A49" s="9" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B49" s="9"/>
       <c r="C49" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A50" s="9" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B50" s="9"/>
       <c r="C50" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A51" s="9" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B51" s="9"/>
       <c r="C51" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A52" s="9" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B52" s="9"/>
       <c r="C52" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A53" s="9" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B53" s="9"/>
       <c r="C53" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A54" s="2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="C54" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A55" s="9" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B55" s="9"/>
       <c r="C55" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A56" s="2" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="C56" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A57" s="10" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="C57" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A58" s="10" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B58" s="11"/>
       <c r="C58" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A59" s="9" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B59" s="11"/>
       <c r="C59" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A60" s="9" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B60" s="11"/>
       <c r="C60" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A61" s="10" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B61" s="10" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C61" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A62" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B62" s="6"/>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A63" s="7" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B63" s="6"/>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A64" s="7" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A65" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B65" s="6"/>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A66" s="7" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B66" s="6"/>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A67" s="7" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B67" s="6"/>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A68" s="7" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B68" s="6"/>
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A69" s="7" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B69" s="6"/>
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A70" s="7" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B70" s="6"/>
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A71" s="7" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B71" s="6"/>
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A72" s="7" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B72" s="6"/>
     </row>
     <row r="73" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A73" s="7" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B73" s="6"/>
     </row>
@@ -2478,7 +2491,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:D132"/>
+  <dimension ref="A1:D133"/>
   <sheetFormatPr defaultColWidth="9.26953125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="32.453125" bestFit="1" customWidth="1"/>
@@ -2489,935 +2502,943 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="C1" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="D1" s="3" t="s">
         <v>29</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B2" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="C2" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D2" s="5" t="s">
         <v>32</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="D2" s="5" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" s="14" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="15" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" s="14" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" s="14" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D6" s="13"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="15" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" s="14" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="D8" s="13"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" s="14" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" s="14" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="D10" s="13"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" s="14" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="D11" s="13"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" s="16" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="D12" s="13"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" s="16" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="D13" s="13"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" s="17" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D14" s="13"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" s="18" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="D15" s="13"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" s="16" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="D16" s="13"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" s="16" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="D17" s="13"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" s="16" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="D18" s="13"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" s="15" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="D19" s="13"/>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" s="15" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D20" s="13"/>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21" s="17" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D21" s="13"/>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" s="17" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="D22" s="13"/>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" s="17" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D23" s="13"/>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A24" s="17" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D24" s="13"/>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A25" s="17" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="D25" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A26" s="17" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="D26" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A27" s="16" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="D27" s="13"/>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A28" s="16" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D28" s="13"/>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A29" s="16" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="D29" s="13"/>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A30" s="16" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D30" s="13"/>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A31" s="16" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="D31" s="13"/>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A32" s="16" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="D32" s="13"/>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A33" s="16" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="D33" s="13"/>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A34" s="16" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="D34" s="13"/>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A35" s="14" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D35" s="13"/>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A36" s="16" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="D36" s="13"/>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A37" s="16" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="D37" s="13"/>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A38" s="16" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="D38" s="13"/>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A39" s="16" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="D39" s="13"/>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A40" s="16" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="D40" s="13"/>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A41" s="16" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="D41" s="13"/>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A42" s="16" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="D42" s="13"/>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A43" s="16" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="D43" s="13"/>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A44" s="16" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="D44" s="13"/>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A45" s="16" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D45" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A46" s="16" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D46" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A47" s="16" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D47" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A48" s="16" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D48" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A49" s="16" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D49" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A50" s="16" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D50" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A51" s="16" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D51" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A52" s="16" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D52" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A53" s="16" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D53" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A54" s="15" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D54" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A55" s="15" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D55" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A56" s="15" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D56" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A57" s="18" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D57" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A58" s="18" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D58" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A59" s="18" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D59" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A60" s="18" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D60" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A61" s="18" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D61" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A62" s="15" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D62" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A63" s="15" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D63" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A64" s="17" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="D64" s="13"/>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A65" s="13" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="D65" s="13"/>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A66" s="13" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="D66" s="13"/>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A67" s="13" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="D67" s="13"/>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A68" s="13" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="D68" s="13"/>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="D69" s="13"/>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D70" s="13"/>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="D71" s="13"/>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="D72" s="13"/>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="D73" s="13"/>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D74" s="13"/>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="D75" s="13"/>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="D76" s="13"/>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="D77" s="13"/>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="D78" s="13"/>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="D79" s="13"/>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="D80" s="13"/>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="D81" s="13"/>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="D82" s="13"/>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="D83" s="13"/>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="D84" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="D85" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="D86" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D87" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="D88" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="D89" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="D90" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="D91" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="D92" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="D93" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="D94" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="D95" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="D96" s="13"/>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="D97" s="13"/>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="D98" s="13"/>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="D99" s="13"/>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="D100" s="13"/>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A101" s="19" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="D101" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A102" s="19" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="D102" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A103" s="19" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="D103" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A104" s="19" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="D104" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A105" s="19" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="D105" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A106" s="19" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="D106" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A107" s="19" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="D107" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A108" s="19" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="D108" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A109" s="19" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D109" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A110" s="19" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="D110" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A111" s="19" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="D111" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A112" s="19" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="D112" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A113" s="19" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="D113" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A114" s="19" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D114" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A115" s="19" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="D115" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A116" s="19" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="D116" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A117" s="19" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="D117" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A118" s="19" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D118" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A119" s="19" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="D119" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A120" s="19" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="D120" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A121" s="19" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="D121" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A122" s="19" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="D122" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A123" s="19" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="D123" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A124" s="19" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="D124" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A125" s="19" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D125" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A126" s="19" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="D126" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="127" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A127" s="19" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D127" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="128" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A128" s="19" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D128" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="129" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A129" s="19" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="D129" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="130" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A130" s="19" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="D130" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="131" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A131" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="D131" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A132" s="20" t="s">
+        <v>308</v>
+      </c>
+      <c r="D132" s="20" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="133" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A133" t="s">
         <v>309</v>
       </c>
-      <c r="D132" s="20" t="s">
-        <v>35</v>
+      <c r="D133" t="s">
+        <v>34</v>
       </c>
     </row>
   </sheetData>
@@ -3443,31 +3464,31 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B2" t="s">
         <v>19</v>
-      </c>
-      <c r="B2" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" t="s">
         <v>21</v>
-      </c>
-      <c r="B3" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4" t="s">
         <v>23</v>
-      </c>
-      <c r="B4" t="s">
-        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update "emi_co2_neg_air_bio" as OUTPUT
</commit_message>
<xml_diff>
--- a/config_data/mapping_v4.xlsx
+++ b/config_data/mapping_v4.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Xchange\Studis\Apath\materials_DAdapter\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\00_ESA\641_SEDOS BMWi\04-Arbeitspakete\AP9-Modellierung\data_adapter_TIMES\data_adapter_times_power\data_adapter_times\config_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20378953-E476-477C-B1EA-F383DD9AB48D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{264CA57A-3BC9-4867-9C7D-DC7F43D699EA}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="8150" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="8150" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SEDOS_parameters" sheetId="5" r:id="rId1"/>
@@ -92,7 +92,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="417" uniqueCount="310">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="419" uniqueCount="311">
   <si>
     <t>TIMES</t>
   </si>
@@ -115,913 +115,916 @@
     <t>demand_annual</t>
   </si>
   <si>
+    <t>ACT_COST</t>
+  </si>
+  <si>
+    <t>NCAP_BND</t>
+  </si>
+  <si>
+    <t>PRC_RESID</t>
+  </si>
+  <si>
+    <t>NCAP_FOM</t>
+  </si>
+  <si>
+    <t>NCAP_TLIFE</t>
+  </si>
+  <si>
+    <t>Absolute upper bound on level of investment in new weight capacity for a period.</t>
+  </si>
+  <si>
+    <t>Investment costs for new capacity per unit weight.</t>
+  </si>
+  <si>
+    <t>Operation independent costs for capacity per unit weight.</t>
+  </si>
+  <si>
+    <t>Technical lifetime of a process.</t>
+  </si>
+  <si>
+    <t>Projected annual demand for a commodity.</t>
+  </si>
+  <si>
+    <t>Comment</t>
+  </si>
+  <si>
+    <t>UP</t>
+  </si>
+  <si>
+    <t>max</t>
+  </si>
+  <si>
+    <t>LO</t>
+  </si>
+  <si>
+    <t>min</t>
+  </si>
+  <si>
+    <t>FX</t>
+  </si>
+  <si>
+    <t>fix</t>
+  </si>
+  <si>
+    <t>FLO_SHAR</t>
+  </si>
+  <si>
+    <t>COM_PROJ</t>
+  </si>
+  <si>
+    <t>CommName</t>
+  </si>
+  <si>
+    <t>CommDesc</t>
+  </si>
+  <si>
+    <t>Unit</t>
+  </si>
+  <si>
+    <t>Csets</t>
+  </si>
+  <si>
+    <t>Commodity Name</t>
+  </si>
+  <si>
+    <t>Commodity Description</t>
+  </si>
+  <si>
+    <t>*Commodity Set Membership</t>
+  </si>
+  <si>
+    <t>iip_steel_sinter</t>
+  </si>
+  <si>
+    <t>MAT</t>
+  </si>
+  <si>
+    <t>iip_steel_crudesteel</t>
+  </si>
+  <si>
+    <t>iip_steel_sponge_iron</t>
+  </si>
+  <si>
+    <t>iip_steel_scrap</t>
+  </si>
+  <si>
+    <t>iip_steel_raw_iron</t>
+  </si>
+  <si>
+    <t>iip_steel_iron_pellets</t>
+  </si>
+  <si>
+    <t>type</t>
+  </si>
+  <si>
+    <t>SEDOS_unit</t>
+  </si>
+  <si>
+    <t>isAbout</t>
+  </si>
+  <si>
+    <t>valueReference</t>
+  </si>
+  <si>
+    <t>Constraints</t>
+  </si>
+  <si>
+    <t>demand_timeseries</t>
+  </si>
+  <si>
+    <t>timeindex_start</t>
+  </si>
+  <si>
+    <t>timeindex_resolution</t>
+  </si>
+  <si>
+    <t>NCAP_AF</t>
+  </si>
+  <si>
+    <t>Constant output ratio in relation to installed capacity. (= h/a)</t>
+  </si>
+  <si>
+    <t>FLO_EFF</t>
+  </si>
+  <si>
+    <t>Commodity-specific conversion factor (multiplication of input and output factors yields the efficiency of the process).</t>
+  </si>
+  <si>
+    <t>Minimum share of flow commodity c based upon the sum of individual flows defined by the commodity group cg belonging to process p.</t>
+  </si>
+  <si>
+    <t>Maximum share of flow commodity c based upon the sum of individual flows defined by the commodity group cg belonging to process p.</t>
+  </si>
+  <si>
+    <t>Fixed share of flow commodity c based upon the sum of individual flows defined by the commodity group cg belonging to process p.</t>
+  </si>
+  <si>
+    <t>capacity_w_inst_0</t>
+  </si>
+  <si>
+    <t>Existing weight capacity of a process.</t>
+  </si>
+  <si>
+    <t>NCAP_COST</t>
+  </si>
+  <si>
+    <t>cost_inv_w</t>
+  </si>
+  <si>
+    <t>cost_fix_w</t>
+  </si>
+  <si>
+    <t>cost_var_w</t>
+  </si>
+  <si>
+    <t>Variable costs per throughput weight unit output. (excluding fuel costs).</t>
+  </si>
+  <si>
+    <t>capacity_w_abs_new_max</t>
+  </si>
+  <si>
+    <t>capacity_e_inst_0</t>
+  </si>
+  <si>
+    <t>Existing storage energy capacity.</t>
+  </si>
+  <si>
+    <t>cost_inv_e</t>
+  </si>
+  <si>
+    <t>Investment costs for new storage energy capacity.</t>
+  </si>
+  <si>
+    <t>cost_fix_e</t>
+  </si>
+  <si>
+    <t>Operation independent costs for existing and new storage energy capacity.</t>
+  </si>
+  <si>
+    <t>cost_var_e</t>
+  </si>
+  <si>
+    <t>Variable costs per throughput energy unit output. (excluding fuel costs).</t>
+  </si>
+  <si>
+    <t>capacity_e_abs_new_max</t>
+  </si>
+  <si>
+    <t>Absolute upper bound on level of investment in new storage energy capacity for a period.</t>
+  </si>
+  <si>
+    <t>capacity_p_inst_0</t>
+  </si>
+  <si>
+    <t>capacity_p_abs_new_max</t>
+  </si>
+  <si>
+    <t>cost_inv_p</t>
+  </si>
+  <si>
+    <t>Investment costs for new throughput power output capacity.</t>
+  </si>
+  <si>
+    <t>cost_fix_p</t>
+  </si>
+  <si>
+    <t>Operation independent costs for existing and new throughput power output capacity.</t>
+  </si>
+  <si>
+    <t>IRE_PRICE</t>
+  </si>
+  <si>
+    <t>commodity_price</t>
+  </si>
+  <si>
+    <t>Cost/Revenue for purchasing/selling one unit (MWh) of a stock or buy commodity.</t>
+  </si>
+  <si>
+    <t>iip_coke_oven_gas</t>
+  </si>
+  <si>
+    <t>iip_aluminum_alumina</t>
+  </si>
+  <si>
+    <t>iip_aluminum_crude</t>
+  </si>
+  <si>
+    <t>iip_aluminum_scrap</t>
+  </si>
+  <si>
+    <t>iip_black_liquor</t>
+  </si>
+  <si>
+    <t>iip_cement_clinker</t>
+  </si>
+  <si>
+    <t>iip_cement_rawmeal</t>
+  </si>
+  <si>
+    <t>iip_coke</t>
+  </si>
+  <si>
+    <t>iip_copper_scrap</t>
+  </si>
+  <si>
+    <t>iip_glass_cont_batch</t>
+  </si>
+  <si>
+    <t>iip_glass_cont_melt</t>
+  </si>
+  <si>
+    <t>iip_glass_flat_batch</t>
+  </si>
+  <si>
+    <t>iip_glass_flat_form</t>
+  </si>
+  <si>
+    <t>iip_glass_flat_melt</t>
+  </si>
+  <si>
+    <t>iip_heat_proc</t>
+  </si>
+  <si>
+    <t>iip_paper_pulp</t>
+  </si>
+  <si>
+    <t>iip_paper_recycle</t>
+  </si>
+  <si>
+    <t>co2_limit</t>
+  </si>
+  <si>
+    <t>potential_annual_max</t>
+  </si>
+  <si>
+    <t>shared_potential_id</t>
+  </si>
+  <si>
+    <t>capacity_p_min</t>
+  </si>
+  <si>
+    <t>capacity_p_max</t>
+  </si>
+  <si>
+    <t>capacity_e_min</t>
+  </si>
+  <si>
+    <t>capacity_e_max</t>
+  </si>
+  <si>
+    <t>capacity_w_min</t>
+  </si>
+  <si>
+    <t>capacity_w_max</t>
+  </si>
+  <si>
+    <t>capacity_tra_inst_0</t>
+  </si>
+  <si>
+    <t>availability_timeseries_fixed</t>
+  </si>
+  <si>
+    <t>availability_timeseries_max</t>
+  </si>
+  <si>
+    <t>wacc</t>
+  </si>
+  <si>
+    <t>cost_inv_tra</t>
+  </si>
+  <si>
+    <t>cost_fix_tra</t>
+  </si>
+  <si>
+    <t>cost_var_tra</t>
+  </si>
+  <si>
+    <t>conversion_factor_&lt;commodity&gt;</t>
+  </si>
+  <si>
+    <t>flow_share_min_&lt;commodity&gt;</t>
+  </si>
+  <si>
+    <t>flow_share_max_&lt;commodity&gt;</t>
+  </si>
+  <si>
+    <t>flow_share_fix_&lt;commodity&gt;</t>
+  </si>
+  <si>
+    <t>conversion_factor_timeseries_&lt;commodity&gt;</t>
+  </si>
+  <si>
+    <t>ef_&lt;input-commodity&gt;_&lt;emission&gt;</t>
+  </si>
+  <si>
+    <t>cb_coefficient</t>
+  </si>
+  <si>
+    <t>cv_coefficient</t>
+  </si>
+  <si>
+    <t>efficiency_sto_in</t>
+  </si>
+  <si>
+    <t>efficiency_sto_out</t>
+  </si>
+  <si>
+    <t>sto_init</t>
+  </si>
+  <si>
+    <t>sto_self_discharge</t>
+  </si>
+  <si>
+    <t>sto_ep_ratio_binding</t>
+  </si>
+  <si>
+    <t>sto_ep_ratio_optional</t>
+  </si>
+  <si>
+    <t>sto_cycles_max</t>
+  </si>
+  <si>
+    <t>capacity_tra_connection_max</t>
+  </si>
+  <si>
+    <t>capacity_tra_connection_timeseries</t>
+  </si>
+  <si>
+    <t>mileage</t>
+  </si>
+  <si>
+    <t>market_share_range</t>
+  </si>
+  <si>
+    <t>occupancy_rate</t>
+  </si>
+  <si>
+    <t>tonnage</t>
+  </si>
+  <si>
+    <t>share_tra_charge_mode</t>
+  </si>
+  <si>
+    <t>sto_min_timeseries</t>
+  </si>
+  <si>
+    <t>sto_max_timeseries</t>
+  </si>
+  <si>
+    <t>optional_limitations</t>
+  </si>
+  <si>
+    <t>id</t>
+  </si>
+  <si>
+    <t>region</t>
+  </si>
+  <si>
+    <t>year</t>
+  </si>
+  <si>
+    <t>bandwidth_type</t>
+  </si>
+  <si>
+    <t>version</t>
+  </si>
+  <si>
+    <t>method</t>
+  </si>
+  <si>
+    <t>source</t>
+  </si>
+  <si>
+    <t>comment</t>
+  </si>
+  <si>
+    <t>timeindex_stop</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>1/NCAP_CHPR?</t>
+  </si>
+  <si>
+    <t>NCAP_CEH</t>
+  </si>
+  <si>
+    <t>S_EFF</t>
+  </si>
+  <si>
+    <t>UC</t>
+  </si>
+  <si>
+    <t>COMBND_NET</t>
+  </si>
+  <si>
+    <t>ACT_COSTS</t>
+  </si>
+  <si>
+    <t>(?)</t>
+  </si>
+  <si>
+    <t>CO2 net emission budget for a period.</t>
+  </si>
+  <si>
+    <t>Maximum annual energy use of a commodity. </t>
+  </si>
+  <si>
+    <t>normalized demand timeseries which gets multiplied with demand_annual</t>
+  </si>
+  <si>
+    <t>specifies a name for a potential group in which all components share the same potential (e.g. wind turibine)</t>
+  </si>
+  <si>
+    <t>Existing throughput power output capacity per process in a certain year.</t>
+  </si>
+  <si>
+    <t>Minimum installable required throughput power output capacity per process.</t>
+  </si>
+  <si>
+    <t>Maximum installable required throughput power output capacity per process.</t>
+  </si>
+  <si>
+    <t>Minimum required storage energy capacity.</t>
+  </si>
+  <si>
+    <t>Maximum allowed storage energy capacity.</t>
+  </si>
+  <si>
+    <t>Maximum weight capacity of a process.</t>
+  </si>
+  <si>
+    <t>Minimum weight capacity of a process.</t>
+  </si>
+  <si>
+    <t>Number of vehicles.</t>
+  </si>
+  <si>
+    <t>Absolute upper bound on level of investment in new power output capacity for a period.</t>
+  </si>
+  <si>
+    <t>Time series of fixed capacity factor in relation to installed capacity.</t>
+  </si>
+  <si>
+    <t>Time series of maximum capacity factor in relation to installed capacity.</t>
+  </si>
+  <si>
+    <t>Percentage of costs for capital after taxes. Used to calculate annuity factor for investment costs.</t>
+  </si>
+  <si>
+    <t>Investment costs for new vehicle unit.</t>
+  </si>
+  <si>
+    <t>Operation independent costs for existing and new vehicle units.</t>
+  </si>
+  <si>
+    <t>Time-variable commodity-specific conversion factor.</t>
+  </si>
+  <si>
+    <t>Input-specific emission factor.</t>
+  </si>
+  <si>
+    <t>The Cb-coefficient (backpressure coefficient) is defined as the maximum power generation capacity in backpressure mode divided by the maximum heat production capacity (including flue gas condensation if applicable).</t>
+  </si>
+  <si>
+    <t>The Cv-value for an extraction steam turbine is defined as the loss of electricity production, when the heat production is increased one unit at constant fuel input.</t>
+  </si>
+  <si>
+    <t>Energy efficiency of power input.</t>
+  </si>
+  <si>
+    <t>Energy efficiency of power output.</t>
+  </si>
+  <si>
+    <t>The initial state of charge of a storage.</t>
+  </si>
+  <si>
+    <t>Storage losses over time.</t>
+  </si>
+  <si>
+    <t>Fixed ratio of the storage energy capacity to its power output capacity.</t>
+  </si>
+  <si>
+    <t>Optional fixed ratio of the storage energy capacity to its power output capacity.</t>
+  </si>
+  <si>
+    <t>Defines the maximum number of full storage cycle equivalents over the lifetime.</t>
+  </si>
+  <si>
+    <t>Maximum connection capacity of an average electric vehicle, taken the connection availability into acocunt.</t>
+  </si>
+  <si>
+    <t>Connection capacity of an average electric vehicle.</t>
+  </si>
+  <si>
+    <t>Yearly mileage of a vehicle.</t>
+  </si>
+  <si>
+    <t>Range of market share.</t>
+  </si>
+  <si>
+    <t>Occupancy rate of a vehicle.</t>
+  </si>
+  <si>
+    <t>Tonnes transported per vehicle.</t>
+  </si>
+  <si>
+    <t>Proportion of fleet that load with a soecific charge mode..</t>
+  </si>
+  <si>
+    <t>Time series of min battery state of charge.</t>
+  </si>
+  <si>
+    <t>Time series of max battery state of charge.</t>
+  </si>
+  <si>
+    <t>User constraint to describe market limitations.</t>
+  </si>
+  <si>
+    <t>Scenario/Milestone steps in the defined time horizon of the intertemporal model</t>
+  </si>
+  <si>
+    <t>Have to figure it out, how to implement</t>
+  </si>
+  <si>
+    <t>data columns info</t>
+  </si>
+  <si>
+    <t>NCAP_CHPR</t>
+  </si>
+  <si>
+    <t>iip_auto_parts_pc_phev</t>
+  </si>
+  <si>
+    <t>iip_chemi_steam</t>
+  </si>
+  <si>
+    <t>iip_auto_painted_pc_fcev</t>
+  </si>
+  <si>
+    <t>iip_elec</t>
+  </si>
+  <si>
+    <t>iip_auto_parts_lcv_icev</t>
+  </si>
+  <si>
+    <t>iip_auto_painted_pc_icev</t>
+  </si>
+  <si>
+    <t>iip_auto_painted_lcv_icev</t>
+  </si>
+  <si>
+    <t>iip_chemi_naphtha</t>
+  </si>
+  <si>
+    <t>iip_auto_btry_hcv_icev</t>
+  </si>
+  <si>
+    <t>iip_auto_painted_lcv_fcev</t>
+  </si>
+  <si>
+    <t>iip_chemi_meoh_h2</t>
+  </si>
+  <si>
+    <t>iip_steam</t>
+  </si>
+  <si>
+    <t>iip_auto_parts_lcv_fcev</t>
+  </si>
+  <si>
+    <t>iip_chemi_process_heat</t>
+  </si>
+  <si>
+    <t>iip_auto_btry_lcv_bev</t>
+  </si>
+  <si>
+    <t>iip_auto_parts_pc_icev</t>
+  </si>
+  <si>
+    <t>iip_chemi_heavy_fuel_oil</t>
+  </si>
+  <si>
+    <t>iip_auto_btry_pc_fcev</t>
+  </si>
+  <si>
+    <t>iip_auto_painted_hcv_icev</t>
+  </si>
+  <si>
+    <t>iip_auto_parts_hcv_icev</t>
+  </si>
+  <si>
+    <t>iip_chemi_machine_drive</t>
+  </si>
+  <si>
+    <t>iip_auto_painted_hcv_fcev</t>
+  </si>
+  <si>
+    <t>iip_auto_btry_pc_bev</t>
+  </si>
+  <si>
+    <t>iip_auto_parts_pc_bev</t>
+  </si>
+  <si>
+    <t>iip_auto_btry_pc_phev</t>
+  </si>
+  <si>
+    <t>iip_chemi_nh3_h2</t>
+  </si>
+  <si>
+    <t>iip_auto_painted_pc_bev</t>
+  </si>
+  <si>
+    <t>iip_blafu_gas</t>
+  </si>
+  <si>
+    <t>iip_chemi_methanol</t>
+  </si>
+  <si>
+    <t>iip_chemi_biomethanol</t>
+  </si>
+  <si>
+    <t>iip_auto_btry_hcv_fcev</t>
+  </si>
+  <si>
+    <t>iip_auto_btry_lcv_fcev</t>
+  </si>
+  <si>
+    <t>iip_auto_parts_lcv_bev</t>
+  </si>
+  <si>
+    <t>iip_auto_painted_hcv_bev</t>
+  </si>
+  <si>
+    <t>iip_auto_parts_hcv_fcev</t>
+  </si>
+  <si>
+    <t>iip_auto_btry_pc_icev</t>
+  </si>
+  <si>
+    <t>iip_chemi_electro_chem</t>
+  </si>
+  <si>
+    <t>iip_auto_btry_hcv_bev</t>
+  </si>
+  <si>
+    <t>iip_auto_parts_pc_fcev</t>
+  </si>
+  <si>
+    <t>iip_auto_painted_lcv_bev</t>
+  </si>
+  <si>
+    <t>iip_chemi_meoh_f_h2</t>
+  </si>
+  <si>
+    <t>iip_chemi_mtg_mtk_h2</t>
+  </si>
+  <si>
+    <t>iip_chemi_nh3</t>
+  </si>
+  <si>
+    <t>iip_auto_btry_lcv_icev</t>
+  </si>
+  <si>
+    <t>iip_auto_painted_pc_phev</t>
+  </si>
+  <si>
+    <t>iip_chemi_biomass</t>
+  </si>
+  <si>
+    <t>iip_auto_parts_hcv_bev</t>
+  </si>
+  <si>
+    <t>iip_chemi_methane</t>
+  </si>
+  <si>
+    <t>iip_chemi_processes_others</t>
+  </si>
+  <si>
+    <t>exo_aluminum</t>
+  </si>
+  <si>
+    <t>sec_waste_heat_high_aluminum</t>
+  </si>
+  <si>
+    <t>exo_cement</t>
+  </si>
+  <si>
+    <t>sec_waste_heat_high_cement</t>
+  </si>
+  <si>
+    <t>exo_copper</t>
+  </si>
+  <si>
+    <t>sec_waste_heat_high_copper</t>
+  </si>
+  <si>
+    <t>exo_glass_flat</t>
+  </si>
+  <si>
+    <t>exo_glass_cont</t>
+  </si>
+  <si>
+    <t>exo_glass_fibe</t>
+  </si>
+  <si>
+    <t>sec_waste_heat_high_glass</t>
+  </si>
+  <si>
+    <t>exo_glass_spec</t>
+  </si>
+  <si>
+    <t>exo_steel</t>
+  </si>
+  <si>
+    <t>sec_waste_heat_high_steel</t>
+  </si>
+  <si>
+    <t>iip_blafu_gas_in</t>
+  </si>
+  <si>
+    <t>pri_biomass_stemwood</t>
+  </si>
+  <si>
+    <t>emi_ch4_f_ind</t>
+  </si>
+  <si>
+    <t>emi_ch4_p_ind</t>
+  </si>
+  <si>
+    <t>emi_co2_f_ind</t>
+  </si>
+  <si>
+    <t>emi_co2_p_ind</t>
+  </si>
+  <si>
+    <t>emi_co2_reusable</t>
+  </si>
+  <si>
+    <t>emi_co2_stored</t>
+  </si>
+  <si>
+    <t>pri_coal</t>
+  </si>
+  <si>
+    <t>iip_coke_oven_gas_in</t>
+  </si>
+  <si>
+    <t>sec_elec_ind</t>
+  </si>
+  <si>
+    <t>sec_methane</t>
+  </si>
+  <si>
+    <t>sec_hydrogen</t>
+  </si>
+  <si>
+    <t>sec_heavy_fuel_oil</t>
+  </si>
+  <si>
+    <t>emi_n2o_f_ind</t>
+  </si>
+  <si>
+    <t>emi_co2_neg_fuel_cc_ind</t>
+  </si>
+  <si>
+    <t>emi_co2_neg_proc_cc_ind</t>
+  </si>
+  <si>
+    <t>pri_sewage_sludge</t>
+  </si>
+  <si>
+    <t>pri_waste_non_bio</t>
+  </si>
+  <si>
+    <t>exo_paper_hq</t>
+  </si>
+  <si>
+    <t>exo_paper_lq</t>
+  </si>
+  <si>
+    <t>sec_waste_heat_high_paper</t>
+  </si>
+  <si>
+    <t>sec_elec</t>
+  </si>
+  <si>
+    <t>exo_chemi_btx</t>
+  </si>
+  <si>
+    <t>exo_chemi_others</t>
+  </si>
+  <si>
+    <t>sec_heat_district_high_ind</t>
+  </si>
+  <si>
+    <t>sec_lpg</t>
+  </si>
+  <si>
+    <t>pri_waste_municipal_bio</t>
+  </si>
+  <si>
+    <t>sec_naphtha</t>
+  </si>
+  <si>
+    <t>sec_refinery_gas</t>
+  </si>
+  <si>
+    <t>sec_waste_heat_high_chemi</t>
+  </si>
+  <si>
+    <t>exo_chemi_cl2</t>
+  </si>
+  <si>
+    <t>exo_chemi_methanol</t>
+  </si>
+  <si>
+    <t>exo_chemi_nh3</t>
+  </si>
+  <si>
+    <t>exo_chemi_olefins</t>
+  </si>
+  <si>
+    <t>sec_gasoline_orig</t>
+  </si>
+  <si>
+    <t>sec_kerosene_orig</t>
+  </si>
+  <si>
+    <t>iip_chemi_lpg</t>
+  </si>
+  <si>
+    <t>sec_ammonia_orig</t>
+  </si>
+  <si>
+    <t>sec_methanol_orig</t>
+  </si>
+  <si>
+    <t>sec_biomethanol_orig</t>
+  </si>
+  <si>
+    <t>emi_n2o_p_ind</t>
+  </si>
+  <si>
+    <t>exo_agri_livestock</t>
+  </si>
+  <si>
+    <t>Availability</t>
+  </si>
+  <si>
+    <t>ACTFLO~DEMO</t>
+  </si>
+  <si>
+    <t>emi_co2_neg_imp</t>
+  </si>
+  <si>
+    <t>emi_co2_neg_air_bio</t>
+  </si>
+  <si>
+    <t>emi_co2_neg_air_dacc</t>
+  </si>
+  <si>
     <t>ACT_BND</t>
-  </si>
-  <si>
-    <t>ACT_COST</t>
-  </si>
-  <si>
-    <t>NCAP_BND</t>
-  </si>
-  <si>
-    <t>PRC_RESID</t>
-  </si>
-  <si>
-    <t>NCAP_FOM</t>
-  </si>
-  <si>
-    <t>NCAP_TLIFE</t>
-  </si>
-  <si>
-    <t>Absolute upper bound on level of investment in new weight capacity for a period.</t>
-  </si>
-  <si>
-    <t>Investment costs for new capacity per unit weight.</t>
-  </si>
-  <si>
-    <t>Operation independent costs for capacity per unit weight.</t>
-  </si>
-  <si>
-    <t>Technical lifetime of a process.</t>
-  </si>
-  <si>
-    <t>Projected annual demand for a commodity.</t>
-  </si>
-  <si>
-    <t>Comment</t>
-  </si>
-  <si>
-    <t>UP</t>
-  </si>
-  <si>
-    <t>max</t>
-  </si>
-  <si>
-    <t>LO</t>
-  </si>
-  <si>
-    <t>min</t>
-  </si>
-  <si>
-    <t>FX</t>
-  </si>
-  <si>
-    <t>fix</t>
-  </si>
-  <si>
-    <t>FLO_SHAR</t>
-  </si>
-  <si>
-    <t>COM_PROJ</t>
-  </si>
-  <si>
-    <t>CommName</t>
-  </si>
-  <si>
-    <t>CommDesc</t>
-  </si>
-  <si>
-    <t>Unit</t>
-  </si>
-  <si>
-    <t>Csets</t>
-  </si>
-  <si>
-    <t>Commodity Name</t>
-  </si>
-  <si>
-    <t>Commodity Description</t>
-  </si>
-  <si>
-    <t>*Commodity Set Membership</t>
-  </si>
-  <si>
-    <t>iip_steel_sinter</t>
-  </si>
-  <si>
-    <t>MAT</t>
-  </si>
-  <si>
-    <t>iip_steel_crudesteel</t>
-  </si>
-  <si>
-    <t>iip_steel_sponge_iron</t>
-  </si>
-  <si>
-    <t>iip_steel_scrap</t>
-  </si>
-  <si>
-    <t>iip_steel_raw_iron</t>
-  </si>
-  <si>
-    <t>iip_steel_iron_pellets</t>
-  </si>
-  <si>
-    <t>type</t>
-  </si>
-  <si>
-    <t>SEDOS_unit</t>
-  </si>
-  <si>
-    <t>isAbout</t>
-  </si>
-  <si>
-    <t>valueReference</t>
-  </si>
-  <si>
-    <t>Constraints</t>
-  </si>
-  <si>
-    <t>demand_timeseries</t>
-  </si>
-  <si>
-    <t>timeindex_start</t>
-  </si>
-  <si>
-    <t>timeindex_resolution</t>
-  </si>
-  <si>
-    <t>NCAP_AF</t>
-  </si>
-  <si>
-    <t>Constant output ratio in relation to installed capacity. (= h/a)</t>
-  </si>
-  <si>
-    <t>FLO_EFF</t>
-  </si>
-  <si>
-    <t>Commodity-specific conversion factor (multiplication of input and output factors yields the efficiency of the process).</t>
-  </si>
-  <si>
-    <t>Minimum share of flow commodity c based upon the sum of individual flows defined by the commodity group cg belonging to process p.</t>
-  </si>
-  <si>
-    <t>Maximum share of flow commodity c based upon the sum of individual flows defined by the commodity group cg belonging to process p.</t>
-  </si>
-  <si>
-    <t>Fixed share of flow commodity c based upon the sum of individual flows defined by the commodity group cg belonging to process p.</t>
-  </si>
-  <si>
-    <t>capacity_w_inst_0</t>
-  </si>
-  <si>
-    <t>Existing weight capacity of a process.</t>
-  </si>
-  <si>
-    <t>NCAP_COST</t>
-  </si>
-  <si>
-    <t>cost_inv_w</t>
-  </si>
-  <si>
-    <t>cost_fix_w</t>
-  </si>
-  <si>
-    <t>cost_var_w</t>
-  </si>
-  <si>
-    <t>Variable costs per throughput weight unit output. (excluding fuel costs).</t>
-  </si>
-  <si>
-    <t>capacity_w_abs_new_max</t>
-  </si>
-  <si>
-    <t>capacity_e_inst_0</t>
-  </si>
-  <si>
-    <t>Existing storage energy capacity.</t>
-  </si>
-  <si>
-    <t>cost_inv_e</t>
-  </si>
-  <si>
-    <t>Investment costs for new storage energy capacity.</t>
-  </si>
-  <si>
-    <t>cost_fix_e</t>
-  </si>
-  <si>
-    <t>Operation independent costs for existing and new storage energy capacity.</t>
-  </si>
-  <si>
-    <t>cost_var_e</t>
-  </si>
-  <si>
-    <t>Variable costs per throughput energy unit output. (excluding fuel costs).</t>
-  </si>
-  <si>
-    <t>capacity_e_abs_new_max</t>
-  </si>
-  <si>
-    <t>Absolute upper bound on level of investment in new storage energy capacity for a period.</t>
-  </si>
-  <si>
-    <t>capacity_p_inst_0</t>
-  </si>
-  <si>
-    <t>capacity_p_abs_new_max</t>
-  </si>
-  <si>
-    <t>cost_inv_p</t>
-  </si>
-  <si>
-    <t>Investment costs for new throughput power output capacity.</t>
-  </si>
-  <si>
-    <t>cost_fix_p</t>
-  </si>
-  <si>
-    <t>Operation independent costs for existing and new throughput power output capacity.</t>
-  </si>
-  <si>
-    <t>IRE_PRICE</t>
-  </si>
-  <si>
-    <t>commodity_price</t>
-  </si>
-  <si>
-    <t>Cost/Revenue for purchasing/selling one unit (MWh) of a stock or buy commodity.</t>
-  </si>
-  <si>
-    <t>iip_coke_oven_gas</t>
-  </si>
-  <si>
-    <t>iip_aluminum_alumina</t>
-  </si>
-  <si>
-    <t>iip_aluminum_crude</t>
-  </si>
-  <si>
-    <t>iip_aluminum_scrap</t>
-  </si>
-  <si>
-    <t>iip_black_liquor</t>
-  </si>
-  <si>
-    <t>iip_cement_clinker</t>
-  </si>
-  <si>
-    <t>iip_cement_rawmeal</t>
-  </si>
-  <si>
-    <t>iip_coke</t>
-  </si>
-  <si>
-    <t>iip_copper_scrap</t>
-  </si>
-  <si>
-    <t>iip_glass_cont_batch</t>
-  </si>
-  <si>
-    <t>iip_glass_cont_melt</t>
-  </si>
-  <si>
-    <t>iip_glass_flat_batch</t>
-  </si>
-  <si>
-    <t>iip_glass_flat_form</t>
-  </si>
-  <si>
-    <t>iip_glass_flat_melt</t>
-  </si>
-  <si>
-    <t>iip_heat_proc</t>
-  </si>
-  <si>
-    <t>iip_paper_pulp</t>
-  </si>
-  <si>
-    <t>iip_paper_recycle</t>
-  </si>
-  <si>
-    <t>co2_limit</t>
-  </si>
-  <si>
-    <t>potential_annual_max</t>
-  </si>
-  <si>
-    <t>shared_potential_id</t>
-  </si>
-  <si>
-    <t>capacity_p_min</t>
-  </si>
-  <si>
-    <t>capacity_p_max</t>
-  </si>
-  <si>
-    <t>capacity_e_min</t>
-  </si>
-  <si>
-    <t>capacity_e_max</t>
-  </si>
-  <si>
-    <t>capacity_w_min</t>
-  </si>
-  <si>
-    <t>capacity_w_max</t>
-  </si>
-  <si>
-    <t>capacity_tra_inst_0</t>
-  </si>
-  <si>
-    <t>availability_timeseries_fixed</t>
-  </si>
-  <si>
-    <t>availability_timeseries_max</t>
-  </si>
-  <si>
-    <t>wacc</t>
-  </si>
-  <si>
-    <t>cost_inv_tra</t>
-  </si>
-  <si>
-    <t>cost_fix_tra</t>
-  </si>
-  <si>
-    <t>cost_var_tra</t>
-  </si>
-  <si>
-    <t>conversion_factor_&lt;commodity&gt;</t>
-  </si>
-  <si>
-    <t>flow_share_min_&lt;commodity&gt;</t>
-  </si>
-  <si>
-    <t>flow_share_max_&lt;commodity&gt;</t>
-  </si>
-  <si>
-    <t>flow_share_fix_&lt;commodity&gt;</t>
-  </si>
-  <si>
-    <t>conversion_factor_timeseries_&lt;commodity&gt;</t>
-  </si>
-  <si>
-    <t>ef_&lt;input-commodity&gt;_&lt;emission&gt;</t>
-  </si>
-  <si>
-    <t>cb_coefficient</t>
-  </si>
-  <si>
-    <t>cv_coefficient</t>
-  </si>
-  <si>
-    <t>efficiency_sto_in</t>
-  </si>
-  <si>
-    <t>efficiency_sto_out</t>
-  </si>
-  <si>
-    <t>sto_init</t>
-  </si>
-  <si>
-    <t>sto_self_discharge</t>
-  </si>
-  <si>
-    <t>sto_ep_ratio_binding</t>
-  </si>
-  <si>
-    <t>sto_ep_ratio_optional</t>
-  </si>
-  <si>
-    <t>sto_cycles_max</t>
-  </si>
-  <si>
-    <t>capacity_tra_connection_max</t>
-  </si>
-  <si>
-    <t>capacity_tra_connection_timeseries</t>
-  </si>
-  <si>
-    <t>mileage</t>
-  </si>
-  <si>
-    <t>market_share_range</t>
-  </si>
-  <si>
-    <t>occupancy_rate</t>
-  </si>
-  <si>
-    <t>tonnage</t>
-  </si>
-  <si>
-    <t>share_tra_charge_mode</t>
-  </si>
-  <si>
-    <t>sto_min_timeseries</t>
-  </si>
-  <si>
-    <t>sto_max_timeseries</t>
-  </si>
-  <si>
-    <t>optional_limitations</t>
-  </si>
-  <si>
-    <t>id</t>
-  </si>
-  <si>
-    <t>region</t>
-  </si>
-  <si>
-    <t>year</t>
-  </si>
-  <si>
-    <t>bandwidth_type</t>
-  </si>
-  <si>
-    <t>version</t>
-  </si>
-  <si>
-    <t>method</t>
-  </si>
-  <si>
-    <t>source</t>
-  </si>
-  <si>
-    <t>comment</t>
-  </si>
-  <si>
-    <t>timeindex_stop</t>
-  </si>
-  <si>
-    <t>-</t>
-  </si>
-  <si>
-    <t>1/NCAP_CHPR?</t>
-  </si>
-  <si>
-    <t>NCAP_CEH</t>
-  </si>
-  <si>
-    <t>S_EFF</t>
-  </si>
-  <si>
-    <t>UC</t>
-  </si>
-  <si>
-    <t>COMBND_NET</t>
-  </si>
-  <si>
-    <t>ACT_COSTS</t>
-  </si>
-  <si>
-    <t>(?)</t>
-  </si>
-  <si>
-    <t>CO2 net emission budget for a period.</t>
-  </si>
-  <si>
-    <t>Maximum annual energy use of a commodity. </t>
-  </si>
-  <si>
-    <t>normalized demand timeseries which gets multiplied with demand_annual</t>
-  </si>
-  <si>
-    <t>specifies a name for a potential group in which all components share the same potential (e.g. wind turibine)</t>
-  </si>
-  <si>
-    <t>Existing throughput power output capacity per process in a certain year.</t>
-  </si>
-  <si>
-    <t>Minimum installable required throughput power output capacity per process.</t>
-  </si>
-  <si>
-    <t>Maximum installable required throughput power output capacity per process.</t>
-  </si>
-  <si>
-    <t>Minimum required storage energy capacity.</t>
-  </si>
-  <si>
-    <t>Maximum allowed storage energy capacity.</t>
-  </si>
-  <si>
-    <t>Maximum weight capacity of a process.</t>
-  </si>
-  <si>
-    <t>Minimum weight capacity of a process.</t>
-  </si>
-  <si>
-    <t>Number of vehicles.</t>
-  </si>
-  <si>
-    <t>Absolute upper bound on level of investment in new power output capacity for a period.</t>
-  </si>
-  <si>
-    <t>Time series of fixed capacity factor in relation to installed capacity.</t>
-  </si>
-  <si>
-    <t>Time series of maximum capacity factor in relation to installed capacity.</t>
-  </si>
-  <si>
-    <t>Percentage of costs for capital after taxes. Used to calculate annuity factor for investment costs.</t>
-  </si>
-  <si>
-    <t>Investment costs for new vehicle unit.</t>
-  </si>
-  <si>
-    <t>Operation independent costs for existing and new vehicle units.</t>
-  </si>
-  <si>
-    <t>Time-variable commodity-specific conversion factor.</t>
-  </si>
-  <si>
-    <t>Input-specific emission factor.</t>
-  </si>
-  <si>
-    <t>The Cb-coefficient (backpressure coefficient) is defined as the maximum power generation capacity in backpressure mode divided by the maximum heat production capacity (including flue gas condensation if applicable).</t>
-  </si>
-  <si>
-    <t>The Cv-value for an extraction steam turbine is defined as the loss of electricity production, when the heat production is increased one unit at constant fuel input.</t>
-  </si>
-  <si>
-    <t>Energy efficiency of power input.</t>
-  </si>
-  <si>
-    <t>Energy efficiency of power output.</t>
-  </si>
-  <si>
-    <t>The initial state of charge of a storage.</t>
-  </si>
-  <si>
-    <t>Storage losses over time.</t>
-  </si>
-  <si>
-    <t>Fixed ratio of the storage energy capacity to its power output capacity.</t>
-  </si>
-  <si>
-    <t>Optional fixed ratio of the storage energy capacity to its power output capacity.</t>
-  </si>
-  <si>
-    <t>Defines the maximum number of full storage cycle equivalents over the lifetime.</t>
-  </si>
-  <si>
-    <t>Maximum connection capacity of an average electric vehicle, taken the connection availability into acocunt.</t>
-  </si>
-  <si>
-    <t>Connection capacity of an average electric vehicle.</t>
-  </si>
-  <si>
-    <t>Yearly mileage of a vehicle.</t>
-  </si>
-  <si>
-    <t>Range of market share.</t>
-  </si>
-  <si>
-    <t>Occupancy rate of a vehicle.</t>
-  </si>
-  <si>
-    <t>Tonnes transported per vehicle.</t>
-  </si>
-  <si>
-    <t>Proportion of fleet that load with a soecific charge mode..</t>
-  </si>
-  <si>
-    <t>Time series of min battery state of charge.</t>
-  </si>
-  <si>
-    <t>Time series of max battery state of charge.</t>
-  </si>
-  <si>
-    <t>User constraint to describe market limitations.</t>
-  </si>
-  <si>
-    <t>Scenario/Milestone steps in the defined time horizon of the intertemporal model</t>
-  </si>
-  <si>
-    <t>Have to figure it out, how to implement</t>
-  </si>
-  <si>
-    <t>data columns info</t>
-  </si>
-  <si>
-    <t>NCAP_CHPR</t>
-  </si>
-  <si>
-    <t>iip_auto_parts_pc_phev</t>
-  </si>
-  <si>
-    <t>iip_chemi_steam</t>
-  </si>
-  <si>
-    <t>iip_auto_painted_pc_fcev</t>
-  </si>
-  <si>
-    <t>iip_elec</t>
-  </si>
-  <si>
-    <t>iip_auto_parts_lcv_icev</t>
-  </si>
-  <si>
-    <t>iip_auto_painted_pc_icev</t>
-  </si>
-  <si>
-    <t>iip_auto_painted_lcv_icev</t>
-  </si>
-  <si>
-    <t>iip_chemi_naphtha</t>
-  </si>
-  <si>
-    <t>iip_auto_btry_hcv_icev</t>
-  </si>
-  <si>
-    <t>iip_auto_painted_lcv_fcev</t>
-  </si>
-  <si>
-    <t>iip_chemi_meoh_h2</t>
-  </si>
-  <si>
-    <t>iip_steam</t>
-  </si>
-  <si>
-    <t>iip_auto_parts_lcv_fcev</t>
-  </si>
-  <si>
-    <t>iip_chemi_process_heat</t>
-  </si>
-  <si>
-    <t>iip_auto_btry_lcv_bev</t>
-  </si>
-  <si>
-    <t>iip_auto_parts_pc_icev</t>
-  </si>
-  <si>
-    <t>iip_chemi_heavy_fuel_oil</t>
-  </si>
-  <si>
-    <t>iip_auto_btry_pc_fcev</t>
-  </si>
-  <si>
-    <t>iip_auto_painted_hcv_icev</t>
-  </si>
-  <si>
-    <t>iip_auto_parts_hcv_icev</t>
-  </si>
-  <si>
-    <t>iip_chemi_machine_drive</t>
-  </si>
-  <si>
-    <t>iip_auto_painted_hcv_fcev</t>
-  </si>
-  <si>
-    <t>iip_auto_btry_pc_bev</t>
-  </si>
-  <si>
-    <t>iip_auto_parts_pc_bev</t>
-  </si>
-  <si>
-    <t>iip_auto_btry_pc_phev</t>
-  </si>
-  <si>
-    <t>iip_chemi_nh3_h2</t>
-  </si>
-  <si>
-    <t>iip_auto_painted_pc_bev</t>
-  </si>
-  <si>
-    <t>iip_blafu_gas</t>
-  </si>
-  <si>
-    <t>iip_chemi_methanol</t>
-  </si>
-  <si>
-    <t>iip_chemi_biomethanol</t>
-  </si>
-  <si>
-    <t>iip_auto_btry_hcv_fcev</t>
-  </si>
-  <si>
-    <t>iip_auto_btry_lcv_fcev</t>
-  </si>
-  <si>
-    <t>iip_auto_parts_lcv_bev</t>
-  </si>
-  <si>
-    <t>iip_auto_painted_hcv_bev</t>
-  </si>
-  <si>
-    <t>iip_auto_parts_hcv_fcev</t>
-  </si>
-  <si>
-    <t>iip_auto_btry_pc_icev</t>
-  </si>
-  <si>
-    <t>iip_chemi_electro_chem</t>
-  </si>
-  <si>
-    <t>iip_auto_btry_hcv_bev</t>
-  </si>
-  <si>
-    <t>iip_auto_parts_pc_fcev</t>
-  </si>
-  <si>
-    <t>iip_auto_painted_lcv_bev</t>
-  </si>
-  <si>
-    <t>iip_chemi_meoh_f_h2</t>
-  </si>
-  <si>
-    <t>iip_chemi_mtg_mtk_h2</t>
-  </si>
-  <si>
-    <t>iip_chemi_nh3</t>
-  </si>
-  <si>
-    <t>iip_auto_btry_lcv_icev</t>
-  </si>
-  <si>
-    <t>iip_auto_painted_pc_phev</t>
-  </si>
-  <si>
-    <t>iip_chemi_biomass</t>
-  </si>
-  <si>
-    <t>iip_auto_parts_hcv_bev</t>
-  </si>
-  <si>
-    <t>iip_chemi_methane</t>
-  </si>
-  <si>
-    <t>iip_chemi_processes_others</t>
-  </si>
-  <si>
-    <t>exo_aluminum</t>
-  </si>
-  <si>
-    <t>sec_waste_heat_high_aluminum</t>
-  </si>
-  <si>
-    <t>exo_cement</t>
-  </si>
-  <si>
-    <t>sec_waste_heat_high_cement</t>
-  </si>
-  <si>
-    <t>exo_copper</t>
-  </si>
-  <si>
-    <t>sec_waste_heat_high_copper</t>
-  </si>
-  <si>
-    <t>exo_glass_flat</t>
-  </si>
-  <si>
-    <t>exo_glass_cont</t>
-  </si>
-  <si>
-    <t>exo_glass_fibe</t>
-  </si>
-  <si>
-    <t>sec_waste_heat_high_glass</t>
-  </si>
-  <si>
-    <t>exo_glass_spec</t>
-  </si>
-  <si>
-    <t>exo_steel</t>
-  </si>
-  <si>
-    <t>sec_waste_heat_high_steel</t>
-  </si>
-  <si>
-    <t>iip_blafu_gas_in</t>
-  </si>
-  <si>
-    <t>pri_biomass_stemwood</t>
-  </si>
-  <si>
-    <t>emi_ch4_f_ind</t>
-  </si>
-  <si>
-    <t>emi_ch4_p_ind</t>
-  </si>
-  <si>
-    <t>emi_co2_f_ind</t>
-  </si>
-  <si>
-    <t>emi_co2_p_ind</t>
-  </si>
-  <si>
-    <t>emi_co2_reusable</t>
-  </si>
-  <si>
-    <t>emi_co2_stored</t>
-  </si>
-  <si>
-    <t>pri_coal</t>
-  </si>
-  <si>
-    <t>iip_coke_oven_gas_in</t>
-  </si>
-  <si>
-    <t>sec_elec_ind</t>
-  </si>
-  <si>
-    <t>sec_methane</t>
-  </si>
-  <si>
-    <t>sec_hydrogen</t>
-  </si>
-  <si>
-    <t>sec_heavy_fuel_oil</t>
-  </si>
-  <si>
-    <t>emi_n2o_f_ind</t>
-  </si>
-  <si>
-    <t>emi_co2_neg_fuel_cc_ind</t>
-  </si>
-  <si>
-    <t>emi_co2_neg_proc_cc_ind</t>
-  </si>
-  <si>
-    <t>pri_sewage_sludge</t>
-  </si>
-  <si>
-    <t>pri_waste_non_bio</t>
-  </si>
-  <si>
-    <t>exo_paper_hq</t>
-  </si>
-  <si>
-    <t>exo_paper_lq</t>
-  </si>
-  <si>
-    <t>sec_waste_heat_high_paper</t>
-  </si>
-  <si>
-    <t>sec_elec</t>
-  </si>
-  <si>
-    <t>exo_chemi_btx</t>
-  </si>
-  <si>
-    <t>exo_chemi_others</t>
-  </si>
-  <si>
-    <t>sec_heat_district_high_ind</t>
-  </si>
-  <si>
-    <t>sec_lpg</t>
-  </si>
-  <si>
-    <t>pri_waste_municipal_bio</t>
-  </si>
-  <si>
-    <t>sec_naphtha</t>
-  </si>
-  <si>
-    <t>sec_refinery_gas</t>
-  </si>
-  <si>
-    <t>sec_waste_heat_high_chemi</t>
-  </si>
-  <si>
-    <t>exo_chemi_cl2</t>
-  </si>
-  <si>
-    <t>exo_chemi_methanol</t>
-  </si>
-  <si>
-    <t>exo_chemi_nh3</t>
-  </si>
-  <si>
-    <t>exo_chemi_olefins</t>
-  </si>
-  <si>
-    <t>sec_gasoline_orig</t>
-  </si>
-  <si>
-    <t>sec_kerosene_orig</t>
-  </si>
-  <si>
-    <t>iip_chemi_lpg</t>
-  </si>
-  <si>
-    <t>sec_ammonia_orig</t>
-  </si>
-  <si>
-    <t>sec_methanol_orig</t>
-  </si>
-  <si>
-    <t>sec_biomethanol_orig</t>
-  </si>
-  <si>
-    <t>emi_n2o_p_ind</t>
-  </si>
-  <si>
-    <t>exo_agri_livestock</t>
-  </si>
-  <si>
-    <t>Availability</t>
-  </si>
-  <si>
-    <t>ACTFLO~DEMO</t>
-  </si>
-  <si>
-    <t>emi_co2_neg_imp</t>
-  </si>
-  <si>
-    <t>emi_co2_neg_air_bio</t>
   </si>
 </sst>
 </file>
@@ -1086,7 +1089,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1114,6 +1117,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="8" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="-0.249977111117893"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1151,7 +1160,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1197,6 +1206,10 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1548,36 +1561,36 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="F1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="I1" s="1" t="s">
-        <v>45</v>
-      </c>
       <c r="J1" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C2" s="12" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.35">
@@ -1585,58 +1598,58 @@
         <v>5</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C4" t="s">
         <v>81</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="C4" t="s">
-        <v>82</v>
-      </c>
       <c r="J4" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A5" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>7</v>
+      <c r="A5" s="21" t="s">
+        <v>100</v>
+      </c>
+      <c r="B5" s="22" t="s">
+        <v>310</v>
       </c>
       <c r="C5" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="I5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="N5" s="9"/>
       <c r="O5" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A6" s="9" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B6" s="9"/>
       <c r="C6" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="N6" s="7"/>
       <c r="O6" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.35">
@@ -1644,189 +1657,189 @@
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C7" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A8" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B8" s="9"/>
       <c r="C8" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C9" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C10" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="I10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C11" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="I11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C12" t="s">
         <v>64</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C12" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C13" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="I13" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C14" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I14" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C15" t="s">
         <v>56</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C15" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C16" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I16" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C17" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="I17" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C18" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C19" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="I19" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C20" t="s">
         <v>72</v>
       </c>
-      <c r="B20" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C20" t="s">
-        <v>73</v>
-      </c>
       <c r="I20" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A21" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C21" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="I21" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.35">
@@ -1834,497 +1847,497 @@
         <v>4</v>
       </c>
       <c r="B22" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C22" t="s">
         <v>49</v>
-      </c>
-      <c r="C22" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A23" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C23" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A24" s="9" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C24" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B25" s="2"/>
       <c r="C25" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="J25" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C26" t="s">
         <v>76</v>
-      </c>
-      <c r="B26" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="C26" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A27" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C27" t="s">
         <v>66</v>
-      </c>
-      <c r="B27" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="C27" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C28" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A29" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C29" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C30" t="s">
         <v>78</v>
-      </c>
-      <c r="B30" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C30" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A31" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C31" t="s">
         <v>68</v>
-      </c>
-      <c r="B31" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C31" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A32" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C32" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A33" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C33" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A34" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C34" t="s">
         <v>70</v>
-      </c>
-      <c r="B34" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C34" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A35" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A36" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C36" t="s">
         <v>61</v>
-      </c>
-      <c r="B36" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C36" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A37" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B37" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C37" t="s">
         <v>51</v>
-      </c>
-      <c r="C37" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A38" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C38" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I38" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A39" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C39" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="I39" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A40" s="2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C40" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="I40" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A41" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C41" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A42" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B42" s="2"/>
       <c r="C42" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A43" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C43" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="J43" s="2" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A44" s="2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C44" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A45" s="2" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C45" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A46" s="9" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B46" s="9"/>
       <c r="C46" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A47" s="9" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B47" s="9"/>
       <c r="C47" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A48" s="9" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B48" s="9"/>
       <c r="C48" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A49" s="9" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B49" s="9"/>
       <c r="C49" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A50" s="9" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B50" s="9"/>
       <c r="C50" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A51" s="9" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B51" s="9"/>
       <c r="C51" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A52" s="9" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B52" s="9"/>
       <c r="C52" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A53" s="9" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B53" s="9"/>
       <c r="C53" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A54" s="2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="C54" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A55" s="9" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B55" s="9"/>
       <c r="C55" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A56" s="2" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="C56" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A57" s="10" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="C57" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A58" s="10" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B58" s="11"/>
       <c r="C58" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A59" s="9" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B59" s="11"/>
       <c r="C59" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A60" s="9" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B60" s="11"/>
       <c r="C60" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A61" s="10" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B61" s="10" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C61" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A62" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B62" s="6"/>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A63" s="7" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B63" s="6"/>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A64" s="7" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A65" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B65" s="6"/>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A66" s="7" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B66" s="6"/>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A67" s="7" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B67" s="6"/>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A68" s="7" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B68" s="6"/>
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A69" s="7" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B69" s="6"/>
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A70" s="7" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B70" s="6"/>
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A71" s="7" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B71" s="6"/>
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A72" s="7" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B72" s="6"/>
     </row>
     <row r="73" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A73" s="7" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B73" s="6"/>
     </row>
@@ -2478,7 +2491,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:D132"/>
+  <dimension ref="A1:D133"/>
   <sheetFormatPr defaultColWidth="9.26953125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="32.453125" bestFit="1" customWidth="1"/>
@@ -2489,935 +2502,943 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="C1" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="D1" s="3" t="s">
         <v>29</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B2" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="C2" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D2" s="5" t="s">
         <v>32</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="D2" s="5" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" s="14" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="15" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" s="14" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" s="14" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D6" s="13"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="15" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" s="14" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="D8" s="13"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" s="14" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" s="14" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="D10" s="13"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" s="14" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="D11" s="13"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" s="16" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="D12" s="13"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" s="16" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="D13" s="13"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" s="17" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D14" s="13"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" s="18" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="D15" s="13"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" s="16" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="D16" s="13"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" s="16" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="D17" s="13"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" s="16" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="D18" s="13"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" s="15" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="D19" s="13"/>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" s="15" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D20" s="13"/>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21" s="17" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D21" s="13"/>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" s="17" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="D22" s="13"/>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" s="17" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D23" s="13"/>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A24" s="17" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D24" s="13"/>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A25" s="17" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="D25" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A26" s="17" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="D26" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A27" s="16" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="D27" s="13"/>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A28" s="16" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D28" s="13"/>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A29" s="16" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="D29" s="13"/>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A30" s="16" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D30" s="13"/>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A31" s="16" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="D31" s="13"/>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A32" s="16" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="D32" s="13"/>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A33" s="16" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="D33" s="13"/>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A34" s="16" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="D34" s="13"/>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A35" s="14" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D35" s="13"/>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A36" s="16" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="D36" s="13"/>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A37" s="16" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="D37" s="13"/>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A38" s="16" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="D38" s="13"/>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A39" s="16" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="D39" s="13"/>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A40" s="16" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="D40" s="13"/>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A41" s="16" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="D41" s="13"/>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A42" s="16" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="D42" s="13"/>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A43" s="16" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="D43" s="13"/>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A44" s="16" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="D44" s="13"/>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A45" s="16" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D45" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A46" s="16" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D46" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A47" s="16" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D47" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A48" s="16" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D48" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A49" s="16" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D49" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A50" s="16" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D50" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A51" s="16" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D51" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A52" s="16" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D52" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A53" s="16" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D53" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A54" s="15" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D54" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A55" s="15" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D55" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A56" s="15" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D56" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A57" s="18" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D57" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A58" s="18" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D58" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A59" s="18" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D59" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A60" s="18" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D60" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A61" s="18" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D61" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A62" s="15" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D62" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A63" s="15" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D63" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A64" s="17" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="D64" s="13"/>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A65" s="13" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="D65" s="13"/>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A66" s="13" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="D66" s="13"/>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A67" s="13" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="D67" s="13"/>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A68" s="13" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="D68" s="13"/>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="D69" s="13"/>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D70" s="13"/>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="D71" s="13"/>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="D72" s="13"/>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="D73" s="13"/>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D74" s="13"/>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="D75" s="13"/>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="D76" s="13"/>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="D77" s="13"/>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="D78" s="13"/>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="D79" s="13"/>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="D80" s="13"/>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="D81" s="13"/>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="D82" s="13"/>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="D83" s="13"/>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="D84" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="D85" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="D86" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D87" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="D88" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="D89" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="D90" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="D91" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="D92" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="D93" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="D94" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="D95" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="D96" s="13"/>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="D97" s="13"/>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="D98" s="13"/>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="D99" s="13"/>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="D100" s="13"/>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A101" s="19" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="D101" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A102" s="19" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="D102" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A103" s="19" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="D103" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A104" s="19" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="D104" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A105" s="19" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="D105" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A106" s="19" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="D106" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A107" s="19" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="D107" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A108" s="19" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="D108" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A109" s="19" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D109" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A110" s="19" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="D110" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A111" s="19" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="D111" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A112" s="19" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="D112" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A113" s="19" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="D113" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A114" s="19" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D114" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A115" s="19" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="D115" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A116" s="19" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="D116" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A117" s="19" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="D117" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A118" s="19" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D118" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A119" s="19" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="D119" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A120" s="19" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="D120" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A121" s="19" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="D121" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A122" s="19" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="D122" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A123" s="19" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="D123" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A124" s="19" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="D124" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A125" s="19" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D125" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A126" s="19" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="D126" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="127" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A127" s="19" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D127" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="128" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A128" s="19" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D128" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="129" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A129" s="19" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="D129" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="130" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A130" s="19" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="D130" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="131" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A131" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="D131" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A132" s="20" t="s">
+        <v>308</v>
+      </c>
+      <c r="D132" s="20" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="133" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A133" t="s">
         <v>309</v>
       </c>
-      <c r="D132" s="20" t="s">
-        <v>35</v>
+      <c r="D133" t="s">
+        <v>34</v>
       </c>
     </row>
   </sheetData>
@@ -3443,31 +3464,31 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B2" t="s">
         <v>19</v>
-      </c>
-      <c r="B2" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" t="s">
         <v>21</v>
-      </c>
-      <c r="B3" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4" t="s">
         <v>23</v>
-      </c>
-      <c r="B4" t="s">
-        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update OUTPUT for all regionsemi_co2_neg_air_bio_
</commit_message>
<xml_diff>
--- a/config_data/mapping_v4.xlsx
+++ b/config_data/mapping_v4.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\00_ESA\641_SEDOS BMWi\04-Arbeitspakete\AP9-Modellierung\data_adapter_TIMES\data_adapter_times_power\data_adapter_times\config_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{264CA57A-3BC9-4867-9C7D-DC7F43D699EA}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0393C43B-C710-4D6C-93C5-3984053CA1C3}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="8150" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -92,7 +92,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="419" uniqueCount="311">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="419" uniqueCount="310">
   <si>
     <t>TIMES</t>
   </si>
@@ -1022,9 +1022,6 @@
   </si>
   <si>
     <t>emi_co2_neg_air_dacc</t>
-  </si>
-  <si>
-    <t>ACT_BND</t>
   </si>
 </sst>
 </file>
@@ -1160,7 +1157,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1209,7 +1206,6 @@
     <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1622,8 +1618,8 @@
       <c r="A5" s="21" t="s">
         <v>100</v>
       </c>
-      <c r="B5" s="22" t="s">
-        <v>310</v>
+      <c r="B5" s="20" t="s">
+        <v>9</v>
       </c>
       <c r="C5" t="s">
         <v>158</v>

</xml_diff>

<commit_message>
upsate spelling mistakes > helper_ind_tra_
</commit_message>
<xml_diff>
--- a/config_data/mapping_v4.xlsx
+++ b/config_data/mapping_v4.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20416"/>
+  <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Xchange\Studis\Apath\HiWi Project\config_data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\00_ESA\641_SEDOS BMWi\04-Arbeitspakete\AP9-Modellierung\data_adapter_TIMES\data_adapter_times_power\data_adapter_times\config_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0393C43B-C710-4D6C-93C5-3984053CA1C3}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="8145" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="8150" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SEDOS_parameters" sheetId="5" r:id="rId1"/>
@@ -17,7 +18,7 @@
     <sheet name="limits" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">commodity_set!$A$1:$A$131</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">commodity_set!$A$1:$A$130</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
@@ -29,12 +30,12 @@
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>Islam, Md Anik</author>
   </authors>
   <commentList>
-    <comment ref="B43" authorId="0" shapeId="0">
+    <comment ref="B43" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
       <text>
         <r>
           <rPr>
@@ -64,12 +65,12 @@
 </file>
 
 <file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>Gary Goldstein</author>
   </authors>
   <commentList>
-    <comment ref="D1" authorId="0" shapeId="0">
+    <comment ref="D1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000001000000}">
       <text>
         <r>
           <rPr>
@@ -91,7 +92,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="415" uniqueCount="309">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="419" uniqueCount="310">
   <si>
     <t>TIMES</t>
   </si>
@@ -114,9 +115,6 @@
     <t>demand_annual</t>
   </si>
   <si>
-    <t>ACT_BND</t>
-  </si>
-  <si>
     <t>ACT_COST</t>
   </si>
   <si>
@@ -1015,6 +1013,12 @@
   </si>
   <si>
     <t>ACTFLO~DEMO</t>
+  </si>
+  <si>
+    <t>emi_co2_neg_imp</t>
+  </si>
+  <si>
+    <t>emi_co2_neg_air_bio</t>
   </si>
   <si>
     <t>emi_co2_neg_air_dacc</t>
@@ -1023,7 +1027,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1082,7 +1086,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1110,6 +1114,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="8" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="-0.249977111117893"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1147,7 +1157,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1192,10 +1202,14 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Normal 10" xfId="1"/>
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 10" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
   </cellStyles>
   <dxfs count="1">
     <dxf>
@@ -1517,22 +1531,22 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:O120"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="37.7109375" customWidth="1"/>
-    <col min="2" max="2" width="25.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="31.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="37.7265625" customWidth="1"/>
+    <col min="2" max="2" width="25.7265625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="31.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.26953125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="18" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="22.28515625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.7265625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.7265625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="22.26953125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -1543,925 +1557,925 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="F1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="I1" s="1" t="s">
-        <v>45</v>
-      </c>
       <c r="J1" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C2" s="12" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>5</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C4" t="s">
         <v>81</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="C4" t="s">
-        <v>82</v>
-      </c>
       <c r="J4" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>7</v>
+        <v>155</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A5" s="21" t="s">
+        <v>100</v>
+      </c>
+      <c r="B5" s="20" t="s">
+        <v>9</v>
       </c>
       <c r="C5" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="I5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="N5" s="9"/>
       <c r="O5" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A6" s="9" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B6" s="9"/>
       <c r="C6" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="N6" s="7"/>
       <c r="O6" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C7" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A8" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B8" s="9"/>
       <c r="C8" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A9" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A10" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10" t="s">
+        <v>162</v>
+      </c>
+      <c r="I10" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A11" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C11" t="s">
+        <v>163</v>
+      </c>
+      <c r="I11" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A12" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C12" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A13" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C13" t="s">
+        <v>164</v>
+      </c>
+      <c r="I13" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A14" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C14" t="s">
+        <v>165</v>
+      </c>
+      <c r="I14" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A15" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C15" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A16" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C16" t="s">
+        <v>166</v>
+      </c>
+      <c r="I16" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A17" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C17" t="s">
+        <v>167</v>
+      </c>
+      <c r="I17" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A18" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C18" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A19" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="B9" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C9" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C10" t="s">
-        <v>163</v>
-      </c>
-      <c r="I10" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C11" t="s">
-        <v>164</v>
-      </c>
-      <c r="I11" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C12" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C13" t="s">
-        <v>165</v>
-      </c>
-      <c r="I13" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A14" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C14" t="s">
-        <v>166</v>
-      </c>
-      <c r="I14" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A15" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C15" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A16" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C16" t="s">
-        <v>167</v>
-      </c>
-      <c r="I16" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A17" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C17" t="s">
-        <v>168</v>
-      </c>
-      <c r="I17" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A18" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C18" t="s">
+      <c r="B19" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C19" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A19" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C19" t="s">
-        <v>170</v>
-      </c>
       <c r="I19" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C20" t="s">
         <v>72</v>
       </c>
-      <c r="B20" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C20" t="s">
-        <v>73</v>
-      </c>
       <c r="I20" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A21" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C21" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="I21" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B22" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C22" t="s">
         <v>49</v>
       </c>
-      <c r="C22" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A23" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C23" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A24" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="B23" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="C23" t="s">
+      <c r="B24" s="9" t="s">
+        <v>149</v>
+      </c>
+      <c r="C24" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A24" s="9" t="s">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A25" s="2" t="s">
         <v>111</v>
-      </c>
-      <c r="B24" s="9" t="s">
-        <v>150</v>
-      </c>
-      <c r="C24" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A25" s="2" t="s">
-        <v>112</v>
       </c>
       <c r="B25" s="2"/>
       <c r="C25" t="s">
+        <v>172</v>
+      </c>
+      <c r="J25" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A26" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C26" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A27" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C27" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A28" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C28" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A29" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C29" t="s">
         <v>173</v>
       </c>
-      <c r="J25" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A26" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="B26" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="C26" t="s">
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A30" s="2" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A27" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="B27" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="C27" t="s">
+      <c r="B30" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C30" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A31" s="2" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A28" s="2" t="s">
+      <c r="B31" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C31" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A32" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="B28" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="C28" t="s">
+      <c r="B32" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C32" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A29" s="2" t="s">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A33" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="B29" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="C29" t="s">
+      <c r="B33" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C33" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A30" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="B30" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C30" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A31" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="B31" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C31" t="s">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A34" s="2" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A32" s="2" t="s">
+      <c r="B34" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C34" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A35" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A36" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="B32" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C32" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A33" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="B33" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C33" t="s">
+      <c r="B36" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C36" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A37" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C37" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A38" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C38" t="s">
+        <v>52</v>
+      </c>
+      <c r="I38" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A39" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C39" t="s">
+        <v>53</v>
+      </c>
+      <c r="I39" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A40" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C40" t="s">
+        <v>54</v>
+      </c>
+      <c r="I40" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A41" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C41" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A34" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="B34" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C34" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A35" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="B35" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A36" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="B36" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C36" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A37" s="2" t="s">
-        <v>116</v>
-      </c>
-      <c r="B37" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="C37" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A38" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="B38" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="C38" t="s">
-        <v>53</v>
-      </c>
-      <c r="I38" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A39" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="B39" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="C39" t="s">
-        <v>54</v>
-      </c>
-      <c r="I39" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A40" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="B40" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="C40" t="s">
-        <v>55</v>
-      </c>
-      <c r="I40" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A41" s="2" t="s">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A42" s="2" t="s">
         <v>120</v>
-      </c>
-      <c r="B41" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="C41" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A42" s="2" t="s">
-        <v>121</v>
       </c>
       <c r="B42" s="2"/>
       <c r="C42" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A43" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="C43" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A43" s="2" t="s">
+      <c r="J43" s="2" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A44" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="B43" s="2" t="s">
-        <v>200</v>
-      </c>
-      <c r="C43" t="s">
+      <c r="B44" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="C44" t="s">
         <v>178</v>
       </c>
-      <c r="J43" s="2" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A44" s="2" t="s">
+    </row>
+    <row r="45" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A45" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="B44" s="2" t="s">
+      <c r="B45" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="C44" t="s">
+      <c r="C45" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A45" s="2" t="s">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A46" s="9" t="s">
         <v>124</v>
-      </c>
-      <c r="B45" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="C45" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A46" s="9" t="s">
-        <v>125</v>
       </c>
       <c r="B46" s="9"/>
       <c r="C46" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A47" s="9" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B47" s="9"/>
       <c r="C47" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A48" s="9" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B48" s="9"/>
       <c r="C48" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A49" s="9" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B49" s="9"/>
       <c r="C49" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A50" s="9" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B50" s="9"/>
       <c r="C50" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A51" s="9" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B51" s="9"/>
       <c r="C51" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A52" s="9" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B52" s="9"/>
       <c r="C52" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A53" s="9" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B53" s="9"/>
       <c r="C53" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A54" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>305</v>
+      </c>
+      <c r="C54" t="s">
         <v>188</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A54" s="2" t="s">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A55" s="9" t="s">
         <v>133</v>
-      </c>
-      <c r="B54" s="2" t="s">
-        <v>306</v>
-      </c>
-      <c r="C54" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A55" s="9" t="s">
-        <v>134</v>
       </c>
       <c r="B55" s="9"/>
       <c r="C55" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A56" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="B56" s="2" t="s">
+        <v>306</v>
+      </c>
+      <c r="C56" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A56" s="2" t="s">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A57" s="10" t="s">
         <v>135</v>
       </c>
-      <c r="B56" s="2" t="s">
-        <v>307</v>
-      </c>
-      <c r="C56" t="s">
+      <c r="B57" s="2" t="s">
+        <v>306</v>
+      </c>
+      <c r="C57" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A57" s="10" t="s">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A58" s="10" t="s">
         <v>136</v>
-      </c>
-      <c r="B57" s="2" t="s">
-        <v>307</v>
-      </c>
-      <c r="C57" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A58" s="10" t="s">
-        <v>137</v>
       </c>
       <c r="B58" s="11"/>
       <c r="C58" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A59" s="9" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B59" s="11"/>
       <c r="C59" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A60" s="9" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B60" s="11"/>
       <c r="C60" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A61" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="B61" s="10" t="s">
+        <v>153</v>
+      </c>
+      <c r="C61" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A61" s="10" t="s">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A62" s="7" t="s">
         <v>140</v>
       </c>
-      <c r="B61" s="10" t="s">
-        <v>154</v>
-      </c>
-      <c r="C61" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A62" s="7" t="s">
+      <c r="B62" s="6"/>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A63" s="7" t="s">
         <v>141</v>
       </c>
-      <c r="B62" s="6"/>
-    </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A63" s="7" t="s">
+      <c r="B63" s="6"/>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A64" s="7" t="s">
         <v>142</v>
-      </c>
-      <c r="B63" s="6"/>
-    </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A64" s="7" t="s">
-        <v>143</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A65" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B65" s="6"/>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A66" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="B66" s="6"/>
+    </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A67" s="7" t="s">
         <v>144</v>
       </c>
-      <c r="B66" s="6"/>
-    </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A67" s="7" t="s">
+      <c r="B67" s="6"/>
+    </row>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A68" s="7" t="s">
         <v>145</v>
       </c>
-      <c r="B67" s="6"/>
-    </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A68" s="7" t="s">
+      <c r="B68" s="6"/>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A69" s="7" t="s">
         <v>146</v>
       </c>
-      <c r="B68" s="6"/>
-    </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A69" s="7" t="s">
+      <c r="B69" s="6"/>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A70" s="7" t="s">
         <v>147</v>
       </c>
-      <c r="B69" s="6"/>
-    </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A70" s="7" t="s">
+      <c r="B70" s="6"/>
+    </row>
+    <row r="71" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A71" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="B71" s="6"/>
+    </row>
+    <row r="72" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A72" s="7" t="s">
         <v>148</v>
       </c>
-      <c r="B70" s="6"/>
-    </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A71" s="7" t="s">
+      <c r="B72" s="6"/>
+    </row>
+    <row r="73" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A73" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="B71" s="6"/>
-    </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A72" s="7" t="s">
-        <v>149</v>
-      </c>
-      <c r="B72" s="6"/>
-    </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A73" s="7" t="s">
-        <v>48</v>
-      </c>
       <c r="B73" s="6"/>
     </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B74" s="6"/>
     </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B75" s="6"/>
     </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B76" s="6"/>
     </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B77" s="6"/>
     </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B78" s="6"/>
     </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B79" s="6"/>
     </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B80" s="6"/>
     </row>
-    <row r="81" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="81" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B81" s="6"/>
     </row>
-    <row r="82" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="82" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B82" s="6"/>
     </row>
-    <row r="83" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="83" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B83" s="6"/>
     </row>
-    <row r="84" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="84" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B84" s="6"/>
     </row>
-    <row r="85" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="85" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B85" s="6"/>
     </row>
-    <row r="86" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="86" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B86" s="6"/>
     </row>
-    <row r="87" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="87" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B87" s="6"/>
     </row>
-    <row r="88" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="88" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B88" s="6"/>
     </row>
-    <row r="89" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="89" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B89" s="6"/>
     </row>
-    <row r="90" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="90" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B90" s="6"/>
     </row>
-    <row r="91" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="91" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B91" s="6"/>
     </row>
-    <row r="92" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="92" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B92" s="6"/>
     </row>
-    <row r="93" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="93" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B93" s="6"/>
     </row>
-    <row r="94" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="94" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B94" s="6"/>
     </row>
-    <row r="95" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="95" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B95" s="6"/>
     </row>
-    <row r="96" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="96" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B96" s="6"/>
     </row>
-    <row r="97" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="97" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B97" s="6"/>
     </row>
-    <row r="98" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="98" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B98" s="6"/>
     </row>
-    <row r="99" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="99" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B99" s="6"/>
     </row>
-    <row r="100" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="100" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B100" s="6"/>
     </row>
-    <row r="101" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="101" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B101" s="6"/>
     </row>
-    <row r="102" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="102" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B102" s="6"/>
     </row>
-    <row r="103" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="103" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B103" s="6"/>
     </row>
-    <row r="104" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="104" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B104" s="6"/>
     </row>
-    <row r="105" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="105" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B105" s="6"/>
     </row>
-    <row r="106" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="106" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B106" s="6"/>
     </row>
-    <row r="107" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="107" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B107" s="6"/>
     </row>
-    <row r="108" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="108" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B108" s="6"/>
     </row>
-    <row r="109" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="109" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B109" s="6"/>
     </row>
-    <row r="110" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="110" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B110" s="6"/>
     </row>
-    <row r="111" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="111" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B111" s="6"/>
     </row>
-    <row r="112" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="112" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B112" s="6"/>
     </row>
-    <row r="113" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="113" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B113" s="6"/>
     </row>
-    <row r="114" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="114" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B114" s="6"/>
     </row>
-    <row r="115" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="115" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B115" s="6"/>
     </row>
-    <row r="116" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="116" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B116" s="6"/>
     </row>
-    <row r="117" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="117" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B117" s="6"/>
     </row>
-    <row r="118" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="118" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B118" s="6"/>
     </row>
-    <row r="119" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="119" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B119" s="6"/>
     </row>
-    <row r="120" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="120" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B120" s="6"/>
     </row>
   </sheetData>
@@ -2472,944 +2486,960 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D131"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:D133"/>
+  <sheetFormatPr defaultColWidth="9.26953125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="32.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.5703125" customWidth="1"/>
-    <col min="3" max="3" width="15.42578125" customWidth="1"/>
-    <col min="4" max="4" width="23.7109375" customWidth="1"/>
+    <col min="1" max="1" width="32.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.54296875" customWidth="1"/>
+    <col min="3" max="3" width="15.453125" customWidth="1"/>
+    <col min="4" max="4" width="23.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="C1" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="D1" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="D1" s="3" t="s">
+    </row>
+    <row r="2" spans="1:4" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="5" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="5" t="s">
+      <c r="B2" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="C2" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D2" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="C2" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="D2" s="5" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" s="14" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" s="15" t="s">
         <v>250</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="15" t="s">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" s="14" t="s">
         <v>251</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="14" t="s">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" s="14" t="s">
         <v>252</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="14" t="s">
+      <c r="D6" s="13"/>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" s="15" t="s">
         <v>253</v>
       </c>
-      <c r="D6" s="13"/>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="15" t="s">
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" s="14" t="s">
         <v>254</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="14" t="s">
+      <c r="D8" s="13"/>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" s="14" t="s">
         <v>255</v>
       </c>
-      <c r="D8" s="13"/>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="14" t="s">
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" s="14" t="s">
         <v>256</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="14" t="s">
+      <c r="D10" s="13"/>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" s="14" t="s">
         <v>257</v>
       </c>
-      <c r="D10" s="13"/>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="14" t="s">
+      <c r="D11" s="13"/>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" s="16" t="s">
         <v>258</v>
       </c>
-      <c r="D11" s="13"/>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="16" t="s">
+      <c r="D12" s="13"/>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" s="16" t="s">
         <v>259</v>
       </c>
-      <c r="D12" s="13"/>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="16" t="s">
+      <c r="D13" s="13"/>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A14" s="17" t="s">
+        <v>203</v>
+      </c>
+      <c r="D14" s="13"/>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A15" s="18" t="s">
         <v>260</v>
       </c>
-      <c r="D13" s="13"/>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="17" t="s">
-        <v>204</v>
-      </c>
-      <c r="D14" s="13"/>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="18" t="s">
+      <c r="D15" s="13"/>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A16" s="16" t="s">
         <v>261</v>
       </c>
-      <c r="D15" s="13"/>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="16" t="s">
+      <c r="D16" s="13"/>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A17" s="16" t="s">
+        <v>227</v>
+      </c>
+      <c r="D17" s="13"/>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A18" s="16" t="s">
         <v>262</v>
       </c>
-      <c r="D16" s="13"/>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="16" t="s">
-        <v>228</v>
-      </c>
-      <c r="D17" s="13"/>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="16" t="s">
+      <c r="D18" s="13"/>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A19" s="15" t="s">
         <v>263</v>
       </c>
-      <c r="D18" s="13"/>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="15" t="s">
+      <c r="D19" s="13"/>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A20" s="15" t="s">
+        <v>86</v>
+      </c>
+      <c r="D20" s="13"/>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A21" s="17" t="s">
         <v>264</v>
       </c>
-      <c r="D19" s="13"/>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="D20" s="13"/>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="17" t="s">
+      <c r="D21" s="13"/>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A22" s="17" t="s">
         <v>265</v>
       </c>
-      <c r="D21" s="13"/>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="17" t="s">
+      <c r="D22" s="13"/>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A23" s="17" t="s">
         <v>266</v>
       </c>
-      <c r="D22" s="13"/>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="17" t="s">
+      <c r="D23" s="13"/>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A24" s="17" t="s">
         <v>267</v>
       </c>
-      <c r="D23" s="13"/>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="17" t="s">
+      <c r="D24" s="13"/>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A25" s="17" t="s">
         <v>268</v>
       </c>
-      <c r="D24" s="13"/>
-    </row>
-    <row r="25" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>308</v>
-      </c>
       <c r="D25" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A26" s="17" t="s">
         <v>269</v>
       </c>
       <c r="D26" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" s="17" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A27" s="16" t="s">
         <v>270</v>
       </c>
-      <c r="D27" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D27" s="13"/>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A28" s="16" t="s">
+        <v>82</v>
+      </c>
+      <c r="D28" s="13"/>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A29" s="16" t="s">
         <v>271</v>
       </c>
-      <c r="D28" s="13"/>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29" s="16" t="s">
-        <v>83</v>
-      </c>
       <c r="D29" s="13"/>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A30" s="16" t="s">
+        <v>89</v>
+      </c>
+      <c r="D30" s="13"/>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A31" s="16" t="s">
         <v>272</v>
       </c>
-      <c r="D30" s="13"/>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A31" s="16" t="s">
-        <v>90</v>
-      </c>
       <c r="D31" s="13"/>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A32" s="16" t="s">
         <v>273</v>
       </c>
       <c r="D32" s="13"/>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A33" s="16" t="s">
         <v>274</v>
       </c>
       <c r="D33" s="13"/>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A34" s="16" t="s">
         <v>275</v>
       </c>
       <c r="D34" s="13"/>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35" s="16" t="s">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A35" s="14" t="s">
+        <v>96</v>
+      </c>
+      <c r="D35" s="13"/>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A36" s="16" t="s">
         <v>276</v>
       </c>
-      <c r="D35" s="13"/>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" s="14" t="s">
-        <v>97</v>
-      </c>
       <c r="D36" s="13"/>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A37" s="16" t="s">
         <v>277</v>
       </c>
       <c r="D37" s="13"/>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A38" s="16" t="s">
         <v>278</v>
       </c>
       <c r="D38" s="13"/>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A39" s="16" t="s">
         <v>279</v>
       </c>
       <c r="D39" s="13"/>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A40" s="16" t="s">
+        <v>211</v>
+      </c>
+      <c r="D40" s="13"/>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A41" s="16" t="s">
         <v>280</v>
       </c>
-      <c r="D40" s="13"/>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41" s="16" t="s">
-        <v>212</v>
-      </c>
       <c r="D41" s="13"/>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A42" s="16" t="s">
         <v>281</v>
       </c>
       <c r="D42" s="13"/>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A43" s="16" t="s">
         <v>282</v>
       </c>
       <c r="D43" s="13"/>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A44" s="16" t="s">
         <v>283</v>
       </c>
       <c r="D44" s="13"/>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A45" s="16" t="s">
-        <v>284</v>
-      </c>
-      <c r="D45" s="13"/>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+        <v>83</v>
+      </c>
+      <c r="D45" s="13" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A46" s="16" t="s">
         <v>84</v>
       </c>
       <c r="D46" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A47" s="16" t="s">
         <v>85</v>
       </c>
       <c r="D47" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A48" s="16" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D48" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A49" s="16" t="s">
         <v>88</v>
       </c>
       <c r="D49" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A50" s="16" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D50" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A51" s="16" t="s">
+        <v>93</v>
+      </c>
+      <c r="D51" s="13" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A52" s="16" t="s">
+        <v>95</v>
+      </c>
+      <c r="D52" s="13" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A53" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="D53" s="13" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A54" s="15" t="s">
         <v>91</v>
       </c>
-      <c r="D51" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A52" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="D52" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A53" s="16" t="s">
-        <v>96</v>
-      </c>
-      <c r="D53" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A54" s="16" t="s">
-        <v>95</v>
-      </c>
       <c r="D54" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A55" s="15" t="s">
         <v>92</v>
       </c>
       <c r="D55" s="13" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A56" s="15" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A56" s="15" t="s">
-        <v>93</v>
-      </c>
       <c r="D56" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A57" s="15" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A57" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="D57" s="13" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A58" s="18" t="s">
+        <v>38</v>
+      </c>
+      <c r="D58" s="13" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A59" s="18" t="s">
+        <v>37</v>
+      </c>
+      <c r="D59" s="13" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A60" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="D60" s="13" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A61" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="D57" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A58" s="18" t="s">
-        <v>40</v>
-      </c>
-      <c r="D58" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A59" s="18" t="s">
-        <v>39</v>
-      </c>
-      <c r="D59" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A60" s="18" t="s">
-        <v>38</v>
-      </c>
-      <c r="D60" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A61" s="18" t="s">
-        <v>34</v>
-      </c>
       <c r="D61" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A62" s="18" t="s">
-        <v>37</v>
+        <v>34</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A62" s="15" t="s">
+        <v>97</v>
       </c>
       <c r="D62" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A63" s="15" t="s">
         <v>98</v>
       </c>
       <c r="D63" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A64" s="15" t="s">
-        <v>99</v>
-      </c>
-      <c r="D64" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A65" s="17" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A64" s="17" t="s">
+        <v>284</v>
+      </c>
+      <c r="D64" s="13"/>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A65" s="13" t="s">
         <v>285</v>
       </c>
       <c r="D65" s="13"/>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A66" s="13" t="s">
         <v>286</v>
       </c>
       <c r="D66" s="13"/>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A67" s="13" t="s">
+        <v>236</v>
+      </c>
+      <c r="D67" s="13"/>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A68" s="13" t="s">
         <v>287</v>
       </c>
-      <c r="D67" s="13"/>
-    </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A68" s="13" t="s">
-        <v>237</v>
-      </c>
       <c r="D68" s="13"/>
     </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A69" s="13" t="s">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A69" t="s">
         <v>288</v>
       </c>
       <c r="D69" s="13"/>
     </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
+        <v>220</v>
+      </c>
+      <c r="D70" s="13"/>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A71" t="s">
         <v>289</v>
       </c>
-      <c r="D70" s="13"/>
-    </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A71" t="s">
-        <v>221</v>
-      </c>
       <c r="D71" s="13"/>
     </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>290</v>
       </c>
       <c r="D72" s="13"/>
     </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
+        <v>248</v>
+      </c>
+      <c r="D73" s="13"/>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A74" t="s">
+        <v>213</v>
+      </c>
+      <c r="D74" s="13"/>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A75" t="s">
         <v>291</v>
       </c>
-      <c r="D73" s="13"/>
-    </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A74" t="s">
-        <v>249</v>
-      </c>
-      <c r="D74" s="13"/>
-    </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A75" t="s">
-        <v>214</v>
-      </c>
       <c r="D75" s="13"/>
     </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>292</v>
       </c>
       <c r="D76" s="13"/>
     </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
+        <v>201</v>
+      </c>
+      <c r="D77" s="13"/>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A78" t="s">
         <v>293</v>
       </c>
-      <c r="D77" s="13"/>
-    </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A78" t="s">
-        <v>202</v>
-      </c>
       <c r="D78" s="13"/>
     </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>294</v>
       </c>
       <c r="D79" s="13"/>
     </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>295</v>
       </c>
       <c r="D80" s="13"/>
     </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>296</v>
       </c>
       <c r="D81" s="13"/>
     </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>297</v>
       </c>
       <c r="D82" s="13"/>
     </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>298</v>
       </c>
       <c r="D83" s="13"/>
     </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
+        <v>229</v>
+      </c>
+      <c r="D84" s="13" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A85" t="s">
+        <v>245</v>
+      </c>
+      <c r="D85" s="13" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A86" t="s">
+        <v>247</v>
+      </c>
+      <c r="D86" s="13" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A87" t="s">
+        <v>216</v>
+      </c>
+      <c r="D87" s="13" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A88" t="s">
         <v>299</v>
       </c>
-      <c r="D84" s="13"/>
-    </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A85" t="s">
-        <v>230</v>
-      </c>
-      <c r="D85" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A86" t="s">
-        <v>246</v>
-      </c>
-      <c r="D86" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A87" t="s">
-        <v>248</v>
-      </c>
-      <c r="D87" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A88" t="s">
-        <v>217</v>
-      </c>
       <c r="D88" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
-        <v>300</v>
+        <v>207</v>
       </c>
       <c r="D89" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
-        <v>208</v>
+        <v>228</v>
       </c>
       <c r="D90" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
-        <v>229</v>
+        <v>210</v>
       </c>
       <c r="D91" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
-        <v>211</v>
+        <v>240</v>
       </c>
       <c r="D92" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
+        <v>225</v>
+      </c>
+      <c r="D93" s="13" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A94" t="s">
         <v>241</v>
       </c>
-      <c r="D93" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A94" t="s">
-        <v>226</v>
-      </c>
       <c r="D94" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
         <v>242</v>
       </c>
       <c r="D95" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="96" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
-        <v>243</v>
-      </c>
-      <c r="D96" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
+        <v>300</v>
+      </c>
+      <c r="D96" s="13"/>
+    </row>
+    <row r="97" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
         <v>301</v>
       </c>
       <c r="D97" s="13"/>
     </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
         <v>302</v>
       </c>
       <c r="D98" s="13"/>
     </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
         <v>303</v>
       </c>
       <c r="D99" s="13"/>
     </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
         <v>304</v>
       </c>
       <c r="D100" s="13"/>
     </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A101" t="s">
-        <v>305</v>
-      </c>
-      <c r="D101" s="13"/>
-    </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A101" s="19" t="s">
+        <v>246</v>
+      </c>
+      <c r="D101" s="13" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="102" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A102" s="19" t="s">
-        <v>247</v>
+        <v>234</v>
       </c>
       <c r="D102" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="103" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A103" s="19" t="s">
+        <v>219</v>
+      </c>
+      <c r="D103" s="13" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="104" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A104" s="19" t="s">
+        <v>232</v>
+      </c>
+      <c r="D104" s="13" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="105" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A105" s="19" t="s">
+        <v>212</v>
+      </c>
+      <c r="D105" s="13" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="106" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A106" s="19" t="s">
+        <v>204</v>
+      </c>
+      <c r="D106" s="13" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="107" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A107" s="19" t="s">
+        <v>223</v>
+      </c>
+      <c r="D107" s="13" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="108" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A108" s="19" t="s">
+        <v>238</v>
+      </c>
+      <c r="D108" s="13" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="109" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A109" s="19" t="s">
+        <v>215</v>
+      </c>
+      <c r="D109" s="13" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="110" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A110" s="19" t="s">
+        <v>200</v>
+      </c>
+      <c r="D110" s="13" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="111" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A111" s="19" t="s">
+        <v>237</v>
+      </c>
+      <c r="D111" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="112" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A112" s="19" t="s">
+        <v>230</v>
+      </c>
+      <c r="D112" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="113" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A113" s="19" t="s">
+        <v>208</v>
+      </c>
+      <c r="D113" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="114" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A114" s="19" t="s">
+        <v>214</v>
+      </c>
+      <c r="D114" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="115" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A115" s="19" t="s">
+        <v>231</v>
+      </c>
+      <c r="D115" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="116" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A116" s="19" t="s">
+        <v>243</v>
+      </c>
+      <c r="D116" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="117" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A117" s="19" t="s">
+        <v>222</v>
+      </c>
+      <c r="D117" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="118" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A118" s="19" t="s">
+        <v>217</v>
+      </c>
+      <c r="D118" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="119" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A119" s="19" t="s">
         <v>235</v>
       </c>
-      <c r="D103" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A104" s="19" t="s">
-        <v>220</v>
-      </c>
-      <c r="D104" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A105" s="19" t="s">
+      <c r="D119" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="120" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A120" s="19" t="s">
+        <v>224</v>
+      </c>
+      <c r="D120" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="121" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A121" s="19" t="s">
         <v>233</v>
       </c>
-      <c r="D105" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A106" s="19" t="s">
-        <v>213</v>
-      </c>
-      <c r="D106" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A107" s="19" t="s">
+      <c r="D121" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="122" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A122" s="19" t="s">
+        <v>221</v>
+      </c>
+      <c r="D122" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="123" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A123" s="19" t="s">
+        <v>218</v>
+      </c>
+      <c r="D123" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="124" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A124" s="19" t="s">
+        <v>239</v>
+      </c>
+      <c r="D124" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="125" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A125" s="19" t="s">
+        <v>209</v>
+      </c>
+      <c r="D125" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="126" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A126" s="19" t="s">
+        <v>206</v>
+      </c>
+      <c r="D126" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="127" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A127" s="19" t="s">
+        <v>226</v>
+      </c>
+      <c r="D127" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="128" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A128" s="19" t="s">
+        <v>202</v>
+      </c>
+      <c r="D128" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="129" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A129" s="19" t="s">
         <v>205</v>
       </c>
-      <c r="D107" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A108" s="19" t="s">
-        <v>224</v>
-      </c>
-      <c r="D108" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A109" s="19" t="s">
-        <v>239</v>
-      </c>
-      <c r="D109" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A110" s="19" t="s">
-        <v>216</v>
-      </c>
-      <c r="D110" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A111" s="19" t="s">
-        <v>201</v>
-      </c>
-      <c r="D111" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A112" s="19" t="s">
-        <v>238</v>
-      </c>
-      <c r="D112" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="113" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A113" s="19" t="s">
-        <v>231</v>
-      </c>
-      <c r="D113" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="114" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A114" s="19" t="s">
-        <v>209</v>
-      </c>
-      <c r="D114" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="115" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A115" s="19" t="s">
-        <v>215</v>
-      </c>
-      <c r="D115" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="116" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A116" s="19" t="s">
-        <v>232</v>
-      </c>
-      <c r="D116" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="117" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A117" s="19" t="s">
+      <c r="D129" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="130" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A130" s="19" t="s">
         <v>244</v>
       </c>
-      <c r="D117" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="118" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A118" s="19" t="s">
-        <v>223</v>
-      </c>
-      <c r="D118" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="119" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A119" s="19" t="s">
-        <v>218</v>
-      </c>
-      <c r="D119" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="120" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A120" s="19" t="s">
-        <v>236</v>
-      </c>
-      <c r="D120" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="121" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A121" s="19" t="s">
-        <v>225</v>
-      </c>
-      <c r="D121" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="122" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A122" s="19" t="s">
-        <v>234</v>
-      </c>
-      <c r="D122" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="123" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A123" s="19" t="s">
-        <v>222</v>
-      </c>
-      <c r="D123" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="124" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A124" s="19" t="s">
-        <v>219</v>
-      </c>
-      <c r="D124" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="125" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A125" s="19" t="s">
-        <v>240</v>
-      </c>
-      <c r="D125" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="126" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A126" s="19" t="s">
-        <v>210</v>
-      </c>
-      <c r="D126" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="127" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A127" s="19" t="s">
-        <v>207</v>
-      </c>
-      <c r="D127" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="128" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A128" s="19" t="s">
-        <v>227</v>
-      </c>
-      <c r="D128" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="129" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A129" s="19" t="s">
-        <v>203</v>
-      </c>
-      <c r="D129" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="130" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A130" s="19" t="s">
-        <v>206</v>
-      </c>
       <c r="D130" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="131" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A131" s="19" t="s">
-        <v>245</v>
+        <v>34</v>
+      </c>
+    </row>
+    <row r="131" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A131" t="s">
+        <v>307</v>
       </c>
       <c r="D131" t="s">
-        <v>35</v>
+        <v>34</v>
+      </c>
+    </row>
+    <row r="132" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A132" s="20" t="s">
+        <v>308</v>
+      </c>
+      <c r="D132" s="20" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="133" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A133" t="s">
+        <v>309</v>
+      </c>
+      <c r="D133" t="s">
+        <v>34</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:A131"/>
-  <conditionalFormatting sqref="A3:A24 A26:A131">
+  <autoFilter ref="A1:A130" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
+  <conditionalFormatting sqref="A3:A130">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3418,11 +3448,11 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.26953125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3430,31 +3460,31 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="B2" t="s">
         <v>19</v>
       </c>
-      <c r="B2" t="s">
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="B3" t="s">
         <v>21</v>
       </c>
-      <c r="B3" t="s">
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="B4" t="s">
         <v>23</v>
-      </c>
-      <c r="B4" t="s">
-        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>